<commit_message>
#29 Digikey BOM Completed
</commit_message>
<xml_diff>
--- a/Design Files/Baseboard-v2.0/BOM/Client_BOM_Baseboard-v2.0.xlsx
+++ b/Design Files/Baseboard-v2.0/BOM/Client_BOM_Baseboard-v2.0.xlsx
@@ -12,14 +12,14 @@
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="5 Boards" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="744" uniqueCount="417">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="802" uniqueCount="416">
   <si>
     <t>Component list</t>
   </si>
@@ -1194,12 +1194,6 @@
     <t>RC0201FR-071KL</t>
   </si>
   <si>
-    <t>RC-01W471JT</t>
-  </si>
-  <si>
-    <t>0402WGJ0220TCE</t>
-  </si>
-  <si>
     <t>Value</t>
   </si>
   <si>
@@ -1270,6 +1264,9 @@
   </si>
   <si>
     <t>Custom Supplier</t>
+  </si>
+  <si>
+    <t>CRCW040222R0FKEDHP</t>
   </si>
 </sst>
 </file>
@@ -1281,7 +1278,7 @@
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0000"/>
     <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="23" x14ac:knownFonts="1">
+  <fonts count="24" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1444,6 +1441,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -1471,7 +1475,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="24">
+  <borders count="23">
     <border>
       <left/>
       <right/>
@@ -1729,21 +1733,6 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -1911,6 +1900,101 @@
     <xf numFmtId="166" fontId="14" fillId="3" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="17" fillId="2" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="17" fillId="2" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="17" fillId="2" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="17" fillId="2" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="16" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="16" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1924,108 +2008,13 @@
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="22" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="17" fillId="2" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="17" fillId="2" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="17" fillId="2" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="17" fillId="2" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="16" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="16" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2399,13 +2388,13 @@
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
-      <c r="J1" s="61"/>
-      <c r="K1" s="61"/>
-      <c r="L1" s="61"/>
-      <c r="M1" s="61"/>
-      <c r="N1" s="61"/>
-      <c r="O1" s="61"/>
-      <c r="P1" s="61"/>
+      <c r="J1" s="92"/>
+      <c r="K1" s="92"/>
+      <c r="L1" s="92"/>
+      <c r="M1" s="92"/>
+      <c r="N1" s="92"/>
+      <c r="O1" s="92"/>
+      <c r="P1" s="92"/>
     </row>
     <row r="2" spans="1:16" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -2449,7 +2438,7 @@
       <c r="M3" s="4"/>
       <c r="N3" s="4"/>
       <c r="O3" s="4"/>
-      <c r="P3" s="62"/>
+      <c r="P3" s="93"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -2471,7 +2460,7 @@
       <c r="M4" s="5"/>
       <c r="N4" s="5"/>
       <c r="O4" s="5"/>
-      <c r="P4" s="63"/>
+      <c r="P4" s="94"/>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -2493,7 +2482,7 @@
       <c r="M5" s="5"/>
       <c r="N5" s="5"/>
       <c r="O5" s="5"/>
-      <c r="P5" s="63"/>
+      <c r="P5" s="94"/>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -2511,7 +2500,7 @@
       <c r="M6" s="5"/>
       <c r="N6" s="5"/>
       <c r="O6" s="5"/>
-      <c r="P6" s="63"/>
+      <c r="P6" s="94"/>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -2529,7 +2518,7 @@
       <c r="M7" s="7"/>
       <c r="N7" s="7"/>
       <c r="O7" s="7"/>
-      <c r="P7" s="63"/>
+      <c r="P7" s="94"/>
     </row>
     <row r="8" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -2547,7 +2536,7 @@
       <c r="M8" s="7"/>
       <c r="N8" s="7"/>
       <c r="O8" s="7"/>
-      <c r="P8" s="63"/>
+      <c r="P8" s="94"/>
     </row>
     <row r="9" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -2576,30 +2565,30 @@
         <v>293</v>
       </c>
       <c r="J9" s="29" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="K9" s="29" t="s">
         <v>375</v>
       </c>
-      <c r="L9" s="91" t="s">
+      <c r="L9" s="85" t="s">
+        <v>392</v>
+      </c>
+      <c r="M9" s="29" t="s">
+        <v>393</v>
+      </c>
+      <c r="N9" s="86" t="s">
         <v>394</v>
       </c>
-      <c r="M9" s="29" t="s">
+      <c r="O9" s="29" t="s">
         <v>395</v>
       </c>
-      <c r="N9" s="92" t="s">
+      <c r="P9" s="29" t="s">
         <v>396</v>
-      </c>
-      <c r="O9" s="29" t="s">
-        <v>397</v>
-      </c>
-      <c r="P9" s="29" t="s">
-        <v>398</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
-      <c r="B10" s="66">
+      <c r="B10" s="61">
         <f>ROW(B10) - ROW($B$9)</f>
         <v>1</v>
       </c>
@@ -2630,14 +2619,14 @@
       <c r="K10" s="44">
         <v>1</v>
       </c>
-      <c r="L10" s="80">
+      <c r="L10" s="75">
         <f>K10*5</f>
         <v>5</v>
       </c>
       <c r="M10" s="44" t="s">
         <v>378</v>
       </c>
-      <c r="N10" s="93" t="s">
+      <c r="N10" s="87" t="s">
         <v>378</v>
       </c>
       <c r="O10" s="52" t="s">
@@ -2647,7 +2636,7 @@
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
-      <c r="B11" s="67">
+      <c r="B11" s="62">
         <f t="shared" ref="B11:B89" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
@@ -2678,14 +2667,14 @@
       <c r="K11" s="31">
         <v>1</v>
       </c>
-      <c r="L11" s="79">
+      <c r="L11" s="74">
         <f t="shared" ref="L11" si="1">K11*5</f>
         <v>5</v>
       </c>
       <c r="M11" s="54" t="s">
-        <v>415</v>
-      </c>
-      <c r="N11" s="85">
+        <v>413</v>
+      </c>
+      <c r="N11" s="80">
         <v>0.48</v>
       </c>
       <c r="O11" s="55">
@@ -2696,7 +2685,7 @@
     </row>
     <row r="12" spans="1:16" ht="36" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
-      <c r="B12" s="66">
+      <c r="B12" s="61">
         <f>ROW(B12) - ROW($B$9)</f>
         <v>3</v>
       </c>
@@ -2727,14 +2716,14 @@
       <c r="K12" s="30">
         <v>25</v>
       </c>
-      <c r="L12" s="78">
+      <c r="L12" s="73">
         <f>K12*5</f>
         <v>125</v>
       </c>
-      <c r="M12" s="96" t="s">
-        <v>415</v>
-      </c>
-      <c r="N12" s="84">
+      <c r="M12" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N12" s="79">
         <v>1.03E-2</v>
       </c>
       <c r="O12" s="56">
@@ -2745,7 +2734,7 @@
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" s="1"/>
-      <c r="B13" s="67">
+      <c r="B13" s="62">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
@@ -2776,14 +2765,14 @@
       <c r="K13" s="31">
         <v>3</v>
       </c>
-      <c r="L13" s="79">
+      <c r="L13" s="74">
         <f t="shared" ref="L13" si="3">K13*5</f>
         <v>15</v>
       </c>
-      <c r="M13" s="96" t="s">
-        <v>415</v>
-      </c>
-      <c r="N13" s="85">
+      <c r="M13" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N13" s="80">
         <v>1.6E-2</v>
       </c>
       <c r="O13" s="55">
@@ -2794,7 +2783,7 @@
     </row>
     <row r="14" spans="1:16" ht="36" x14ac:dyDescent="0.25">
       <c r="A14" s="1"/>
-      <c r="B14" s="66">
+      <c r="B14" s="61">
         <f>ROW(B14) - ROW($B$9)</f>
         <v>5</v>
       </c>
@@ -2825,14 +2814,14 @@
       <c r="K14" s="30">
         <v>3</v>
       </c>
-      <c r="L14" s="78">
+      <c r="L14" s="73">
         <f>K14*5</f>
         <v>15</v>
       </c>
-      <c r="M14" s="97" t="s">
-        <v>416</v>
-      </c>
-      <c r="N14" s="84" t="s">
+      <c r="M14" s="90" t="s">
+        <v>414</v>
+      </c>
+      <c r="N14" s="79" t="s">
         <v>378</v>
       </c>
       <c r="O14" s="56" t="s">
@@ -2842,7 +2831,7 @@
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" s="1"/>
-      <c r="B15" s="67">
+      <c r="B15" s="62">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
@@ -2873,14 +2862,14 @@
       <c r="K15" s="31">
         <v>2</v>
       </c>
-      <c r="L15" s="79">
+      <c r="L15" s="74">
         <f t="shared" ref="L15" si="5">K15*5</f>
         <v>10</v>
       </c>
-      <c r="M15" s="96" t="s">
-        <v>415</v>
-      </c>
-      <c r="N15" s="85">
+      <c r="M15" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N15" s="80">
         <v>0.79600000000000004</v>
       </c>
       <c r="O15" s="55">
@@ -2891,7 +2880,7 @@
     </row>
     <row r="16" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
-      <c r="B16" s="66">
+      <c r="B16" s="61">
         <f>ROW(B16) - ROW($B$9)</f>
         <v>7</v>
       </c>
@@ -2922,14 +2911,14 @@
       <c r="K16" s="30">
         <v>1</v>
       </c>
-      <c r="L16" s="78">
+      <c r="L16" s="73">
         <f>K16*5</f>
         <v>5</v>
       </c>
-      <c r="M16" s="97" t="s">
-        <v>416</v>
-      </c>
-      <c r="N16" s="84" t="s">
+      <c r="M16" s="90" t="s">
+        <v>414</v>
+      </c>
+      <c r="N16" s="79" t="s">
         <v>378</v>
       </c>
       <c r="O16" s="56" t="s">
@@ -2939,7 +2928,7 @@
     </row>
     <row r="17" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="1"/>
-      <c r="B17" s="67">
+      <c r="B17" s="62">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
@@ -2970,14 +2959,14 @@
       <c r="K17" s="31">
         <v>1</v>
       </c>
-      <c r="L17" s="79">
+      <c r="L17" s="74">
         <f t="shared" ref="L17" si="7">K17*5</f>
         <v>5</v>
       </c>
-      <c r="M17" s="97" t="s">
-        <v>416</v>
-      </c>
-      <c r="N17" s="85" t="s">
+      <c r="M17" s="90" t="s">
+        <v>414</v>
+      </c>
+      <c r="N17" s="80" t="s">
         <v>378</v>
       </c>
       <c r="O17" s="55" t="s">
@@ -2987,7 +2976,7 @@
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18" s="1"/>
-      <c r="B18" s="66">
+      <c r="B18" s="61">
         <f>ROW(B18) - ROW($B$9)</f>
         <v>9</v>
       </c>
@@ -3018,14 +3007,14 @@
       <c r="K18" s="30">
         <v>1</v>
       </c>
-      <c r="L18" s="78">
+      <c r="L18" s="73">
         <f>K18*5</f>
         <v>5</v>
       </c>
-      <c r="M18" s="96" t="s">
-        <v>415</v>
-      </c>
-      <c r="N18" s="84">
+      <c r="M18" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N18" s="79">
         <v>3.42</v>
       </c>
       <c r="O18" s="56">
@@ -3036,7 +3025,7 @@
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19" s="1"/>
-      <c r="B19" s="67">
+      <c r="B19" s="62">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
@@ -3067,14 +3056,14 @@
       <c r="K19" s="31">
         <v>1</v>
       </c>
-      <c r="L19" s="79">
+      <c r="L19" s="74">
         <f t="shared" ref="L19" si="8">K19*5</f>
         <v>5</v>
       </c>
-      <c r="M19" s="96" t="s">
-        <v>415</v>
-      </c>
-      <c r="N19" s="85">
+      <c r="M19" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N19" s="80">
         <v>0.68</v>
       </c>
       <c r="O19" s="55">
@@ -3085,7 +3074,7 @@
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20" s="1"/>
-      <c r="B20" s="66">
+      <c r="B20" s="61">
         <f>ROW(B20) - ROW($B$9)</f>
         <v>11</v>
       </c>
@@ -3116,23 +3105,25 @@
       <c r="K20" s="30">
         <v>4</v>
       </c>
-      <c r="L20" s="78">
+      <c r="L20" s="73">
         <f>K20*5</f>
         <v>20</v>
       </c>
-      <c r="M20" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N20" s="84"/>
+      <c r="M20" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N20" s="79">
+        <v>6.2E-2</v>
+      </c>
       <c r="O20" s="56">
         <f>N20*L20</f>
-        <v>0</v>
+        <v>1.24</v>
       </c>
       <c r="P20" s="30"/>
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" s="1"/>
-      <c r="B21" s="67">
+      <c r="B21" s="62">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
@@ -3163,23 +3154,25 @@
       <c r="K21" s="31">
         <v>2</v>
       </c>
-      <c r="L21" s="79">
+      <c r="L21" s="74">
         <f t="shared" ref="L21" si="10">K21*5</f>
         <v>10</v>
       </c>
-      <c r="M21" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N21" s="85"/>
+      <c r="M21" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N21" s="80">
+        <v>0.121</v>
+      </c>
       <c r="O21" s="55">
         <f t="shared" ref="O21" si="11">N21*L21</f>
-        <v>0</v>
+        <v>1.21</v>
       </c>
       <c r="P21" s="31"/>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>
-      <c r="B22" s="66">
+      <c r="B22" s="61">
         <f>ROW(B22) - ROW($B$9)</f>
         <v>13</v>
       </c>
@@ -3210,23 +3203,25 @@
       <c r="K22" s="30">
         <v>2</v>
       </c>
-      <c r="L22" s="78">
+      <c r="L22" s="73">
         <f>K22*5</f>
         <v>10</v>
       </c>
-      <c r="M22" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N22" s="84"/>
+      <c r="M22" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N22" s="79">
+        <v>1.9E-2</v>
+      </c>
       <c r="O22" s="56">
         <f>N22*L22</f>
-        <v>0</v>
+        <v>0.19</v>
       </c>
       <c r="P22" s="30"/>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
-      <c r="B23" s="67">
+      <c r="B23" s="62">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
@@ -3257,23 +3252,25 @@
       <c r="K23" s="31">
         <v>3</v>
       </c>
-      <c r="L23" s="79">
+      <c r="L23" s="74">
         <f t="shared" ref="L23" si="12">K23*5</f>
         <v>15</v>
       </c>
-      <c r="M23" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N23" s="85"/>
+      <c r="M23" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N23" s="80">
+        <v>7.3999999999999996E-2</v>
+      </c>
       <c r="O23" s="55">
         <f t="shared" ref="O23" si="13">N23*L23</f>
-        <v>0</v>
+        <v>1.1099999999999999</v>
       </c>
       <c r="P23" s="31"/>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A24" s="1"/>
-      <c r="B24" s="66">
+      <c r="B24" s="61">
         <f>ROW(B24) - ROW($B$9)</f>
         <v>15</v>
       </c>
@@ -3304,23 +3301,25 @@
       <c r="K24" s="30">
         <v>1</v>
       </c>
-      <c r="L24" s="78">
+      <c r="L24" s="73">
         <f>K24*5</f>
         <v>5</v>
       </c>
-      <c r="M24" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N24" s="84"/>
+      <c r="M24" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N24" s="79">
+        <v>0.44</v>
+      </c>
       <c r="O24" s="56">
         <f>N24*L24</f>
-        <v>0</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="P24" s="30"/>
     </row>
-    <row r="25" spans="1:16" ht="24" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="1"/>
-      <c r="B25" s="67">
+      <c r="B25" s="62">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
@@ -3351,23 +3350,22 @@
       <c r="K25" s="31">
         <v>1</v>
       </c>
-      <c r="L25" s="79">
+      <c r="L25" s="74">
         <f t="shared" ref="L25" si="14">K25*5</f>
         <v>5</v>
       </c>
-      <c r="M25" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N25" s="85"/>
-      <c r="O25" s="55">
-        <f t="shared" ref="O25" si="15">N25*L25</f>
-        <v>0</v>
+      <c r="M25" s="90" t="s">
+        <v>414</v>
+      </c>
+      <c r="N25" s="80"/>
+      <c r="O25" s="55" t="s">
+        <v>378</v>
       </c>
       <c r="P25" s="31"/>
     </row>
     <row r="26" spans="1:16" ht="36" x14ac:dyDescent="0.25">
       <c r="A26" s="1"/>
-      <c r="B26" s="66">
+      <c r="B26" s="61">
         <f>ROW(B26) - ROW($B$9)</f>
         <v>17</v>
       </c>
@@ -3398,23 +3396,22 @@
       <c r="K26" s="30">
         <v>1</v>
       </c>
-      <c r="L26" s="78">
+      <c r="L26" s="73">
         <f>K26*5</f>
         <v>5</v>
       </c>
-      <c r="M26" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N26" s="84"/>
-      <c r="O26" s="56">
-        <f>N26*L26</f>
-        <v>0</v>
+      <c r="M26" s="90" t="s">
+        <v>414</v>
+      </c>
+      <c r="N26" s="79"/>
+      <c r="O26" s="56" t="s">
+        <v>378</v>
       </c>
       <c r="P26" s="30"/>
     </row>
-    <row r="27" spans="1:16" ht="24" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" s="1"/>
-      <c r="B27" s="67">
+      <c r="B27" s="62">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
@@ -3445,23 +3442,22 @@
       <c r="K27" s="31">
         <v>1</v>
       </c>
-      <c r="L27" s="79">
-        <f t="shared" ref="L27" si="16">K27*5</f>
+      <c r="L27" s="74">
+        <f t="shared" ref="L27" si="15">K27*5</f>
         <v>5</v>
       </c>
-      <c r="M27" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N27" s="85"/>
-      <c r="O27" s="55">
-        <f t="shared" ref="O27" si="17">N27*L27</f>
-        <v>0</v>
+      <c r="M27" s="90" t="s">
+        <v>414</v>
+      </c>
+      <c r="N27" s="80"/>
+      <c r="O27" s="55" t="s">
+        <v>378</v>
       </c>
       <c r="P27" s="31"/>
     </row>
     <row r="28" spans="1:16" ht="24" x14ac:dyDescent="0.25">
       <c r="A28" s="1"/>
-      <c r="B28" s="66">
+      <c r="B28" s="61">
         <f>ROW(B28) - ROW($B$9)</f>
         <v>19</v>
       </c>
@@ -3492,23 +3488,25 @@
       <c r="K28" s="30">
         <v>3</v>
       </c>
-      <c r="L28" s="78">
+      <c r="L28" s="73">
         <f>K28*5</f>
         <v>15</v>
       </c>
-      <c r="M28" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N28" s="84"/>
+      <c r="M28" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N28" s="79">
+        <v>0.184</v>
+      </c>
       <c r="O28" s="56">
         <f>N28*L28</f>
-        <v>0</v>
+        <v>2.76</v>
       </c>
       <c r="P28" s="30"/>
     </row>
     <row r="29" spans="1:16" ht="36" x14ac:dyDescent="0.25">
       <c r="A29" s="1"/>
-      <c r="B29" s="67">
+      <c r="B29" s="62">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
@@ -3539,23 +3537,22 @@
       <c r="K29" s="31">
         <v>2</v>
       </c>
-      <c r="L29" s="79">
-        <f t="shared" ref="L29" si="18">K29*5</f>
+      <c r="L29" s="74">
+        <f t="shared" ref="L29" si="16">K29*5</f>
         <v>10</v>
       </c>
-      <c r="M29" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N29" s="85"/>
-      <c r="O29" s="55">
-        <f t="shared" ref="O29" si="19">N29*L29</f>
-        <v>0</v>
+      <c r="M29" s="90" t="s">
+        <v>414</v>
+      </c>
+      <c r="N29" s="80"/>
+      <c r="O29" s="55" t="s">
+        <v>378</v>
       </c>
       <c r="P29" s="31"/>
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30" s="1"/>
-      <c r="B30" s="66">
+      <c r="B30" s="61">
         <f>ROW(B30) - ROW($B$9)</f>
         <v>21</v>
       </c>
@@ -3586,23 +3583,25 @@
       <c r="K30" s="30">
         <v>4</v>
       </c>
-      <c r="L30" s="78">
+      <c r="L30" s="73">
         <f>K30*5</f>
         <v>20</v>
       </c>
-      <c r="M30" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N30" s="84"/>
+      <c r="M30" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N30" s="79">
+        <v>0.32300000000000001</v>
+      </c>
       <c r="O30" s="56">
         <f>N30*L30</f>
-        <v>0</v>
+        <v>6.46</v>
       </c>
       <c r="P30" s="30"/>
     </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A31" s="1"/>
-      <c r="B31" s="67">
+      <c r="B31" s="62">
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
@@ -3633,23 +3632,22 @@
       <c r="K31" s="31">
         <v>4</v>
       </c>
-      <c r="L31" s="79">
-        <f t="shared" ref="L31" si="20">K31*5</f>
+      <c r="L31" s="74">
+        <f t="shared" ref="L31" si="17">K31*5</f>
         <v>20</v>
       </c>
-      <c r="M31" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N31" s="85"/>
-      <c r="O31" s="55">
-        <f t="shared" ref="O31" si="21">N31*L31</f>
-        <v>0</v>
+      <c r="M31" s="90" t="s">
+        <v>414</v>
+      </c>
+      <c r="N31" s="80"/>
+      <c r="O31" s="55" t="s">
+        <v>378</v>
       </c>
       <c r="P31" s="31"/>
     </row>
     <row r="32" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A32" s="1"/>
-      <c r="B32" s="66">
+      <c r="B32" s="61">
         <f>ROW(B32) - ROW($B$9)</f>
         <v>23</v>
       </c>
@@ -3680,23 +3678,25 @@
       <c r="K32" s="30">
         <v>1</v>
       </c>
-      <c r="L32" s="78">
+      <c r="L32" s="73">
         <f>K32*5</f>
         <v>5</v>
       </c>
-      <c r="M32" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N32" s="84"/>
+      <c r="M32" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N32" s="79">
+        <v>1.766</v>
+      </c>
       <c r="O32" s="56">
         <f>N32*L32</f>
-        <v>0</v>
+        <v>8.83</v>
       </c>
       <c r="P32" s="30"/>
     </row>
-    <row r="33" spans="1:16" ht="24" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A33" s="1"/>
-      <c r="B33" s="67">
+      <c r="B33" s="62">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
@@ -3727,23 +3727,22 @@
       <c r="K33" s="31">
         <v>1</v>
       </c>
-      <c r="L33" s="79">
-        <f t="shared" ref="L33" si="22">K33*5</f>
+      <c r="L33" s="74">
+        <f t="shared" ref="L33" si="18">K33*5</f>
         <v>5</v>
       </c>
-      <c r="M33" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N33" s="85"/>
-      <c r="O33" s="55">
-        <f t="shared" ref="O33" si="23">N33*L33</f>
-        <v>0</v>
+      <c r="M33" s="90" t="s">
+        <v>414</v>
+      </c>
+      <c r="N33" s="80"/>
+      <c r="O33" s="55" t="s">
+        <v>378</v>
       </c>
       <c r="P33" s="31"/>
     </row>
-    <row r="34" spans="1:16" ht="24" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A34" s="1"/>
-      <c r="B34" s="66">
+      <c r="B34" s="61">
         <f>ROW(B34) - ROW($B$9)</f>
         <v>25</v>
       </c>
@@ -3774,23 +3773,22 @@
       <c r="K34" s="30">
         <v>4</v>
       </c>
-      <c r="L34" s="78">
+      <c r="L34" s="73">
         <f>K34*5</f>
         <v>20</v>
       </c>
-      <c r="M34" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N34" s="84"/>
-      <c r="O34" s="56">
-        <f>N34*L34</f>
-        <v>0</v>
+      <c r="M34" s="90" t="s">
+        <v>414</v>
+      </c>
+      <c r="N34" s="79"/>
+      <c r="O34" s="56" t="s">
+        <v>378</v>
       </c>
       <c r="P34" s="30"/>
     </row>
     <row r="35" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A35" s="1"/>
-      <c r="B35" s="67">
+      <c r="B35" s="62">
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
@@ -3821,23 +3819,25 @@
       <c r="K35" s="31">
         <v>1</v>
       </c>
-      <c r="L35" s="79">
-        <f t="shared" ref="L35" si="24">K35*5</f>
+      <c r="L35" s="74">
+        <f t="shared" ref="L35" si="19">K35*5</f>
         <v>5</v>
       </c>
-      <c r="M35" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N35" s="85"/>
+      <c r="M35" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N35" s="80">
+        <v>0.28000000000000003</v>
+      </c>
       <c r="O35" s="55">
-        <f t="shared" ref="O35" si="25">N35*L35</f>
-        <v>0</v>
+        <f t="shared" ref="O35" si="20">N35*L35</f>
+        <v>1.4000000000000001</v>
       </c>
       <c r="P35" s="31"/>
     </row>
     <row r="36" spans="1:16" ht="48" x14ac:dyDescent="0.25">
       <c r="A36" s="1"/>
-      <c r="B36" s="66">
+      <c r="B36" s="61">
         <f>ROW(B36) - ROW($B$9)</f>
         <v>27</v>
       </c>
@@ -3868,23 +3868,24 @@
       <c r="K36" s="30">
         <v>8</v>
       </c>
-      <c r="L36" s="78">
+      <c r="L36" s="73">
         <f>K36*5</f>
         <v>40</v>
       </c>
-      <c r="M36" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N36" s="84"/>
-      <c r="O36" s="56">
-        <f>N36*L36</f>
-        <v>0</v>
+      <c r="M36" s="90" t="s">
+        <v>414</v>
+      </c>
+      <c r="N36" s="79" t="s">
+        <v>378</v>
+      </c>
+      <c r="O36" s="56" t="s">
+        <v>378</v>
       </c>
       <c r="P36" s="30"/>
     </row>
-    <row r="37" spans="1:16" ht="24" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A37" s="1"/>
-      <c r="B37" s="67">
+      <c r="B37" s="62">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
@@ -3915,23 +3916,24 @@
       <c r="K37" s="31">
         <v>1</v>
       </c>
-      <c r="L37" s="79">
-        <f t="shared" ref="L37" si="26">K37*5</f>
+      <c r="L37" s="74">
+        <f t="shared" ref="L37" si="21">K37*5</f>
         <v>5</v>
       </c>
-      <c r="M37" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N37" s="85"/>
-      <c r="O37" s="55">
-        <f t="shared" ref="O37" si="27">N37*L37</f>
-        <v>0</v>
+      <c r="M37" s="90" t="s">
+        <v>414</v>
+      </c>
+      <c r="N37" s="80" t="s">
+        <v>378</v>
+      </c>
+      <c r="O37" s="55" t="s">
+        <v>378</v>
       </c>
       <c r="P37" s="31"/>
     </row>
     <row r="38" spans="1:16" ht="48" x14ac:dyDescent="0.25">
       <c r="A38" s="1"/>
-      <c r="B38" s="66">
+      <c r="B38" s="61">
         <f>ROW(B38) - ROW($B$9)</f>
         <v>29</v>
       </c>
@@ -3962,23 +3964,24 @@
       <c r="K38" s="30">
         <v>4</v>
       </c>
-      <c r="L38" s="78">
+      <c r="L38" s="73">
         <f>K38*5</f>
         <v>20</v>
       </c>
-      <c r="M38" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N38" s="84"/>
-      <c r="O38" s="56">
-        <f>N38*L38</f>
-        <v>0</v>
+      <c r="M38" s="90" t="s">
+        <v>414</v>
+      </c>
+      <c r="N38" s="79" t="s">
+        <v>378</v>
+      </c>
+      <c r="O38" s="56" t="s">
+        <v>378</v>
       </c>
       <c r="P38" s="30"/>
     </row>
     <row r="39" spans="1:16" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A39" s="1"/>
-      <c r="B39" s="67">
+      <c r="B39" s="62">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
@@ -4009,23 +4012,25 @@
       <c r="K39" s="31">
         <v>1</v>
       </c>
-      <c r="L39" s="79">
-        <f t="shared" ref="L39" si="28">K39*5</f>
+      <c r="L39" s="74">
+        <f t="shared" ref="L39" si="22">K39*5</f>
         <v>5</v>
       </c>
-      <c r="M39" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N39" s="85"/>
+      <c r="M39" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N39" s="80">
+        <v>1.46</v>
+      </c>
       <c r="O39" s="55">
-        <f t="shared" ref="O39" si="29">N39*L39</f>
-        <v>0</v>
+        <f t="shared" ref="O39" si="23">N39*L39</f>
+        <v>7.3</v>
       </c>
       <c r="P39" s="31"/>
     </row>
     <row r="40" spans="1:16" ht="36" x14ac:dyDescent="0.25">
       <c r="A40" s="1"/>
-      <c r="B40" s="66">
+      <c r="B40" s="61">
         <f>ROW(B40) - ROW($B$9)</f>
         <v>31</v>
       </c>
@@ -4056,23 +4061,24 @@
       <c r="K40" s="30">
         <v>1</v>
       </c>
-      <c r="L40" s="78">
+      <c r="L40" s="73">
         <f>K40*5</f>
         <v>5</v>
       </c>
-      <c r="M40" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N40" s="84"/>
-      <c r="O40" s="56">
-        <f>N40*L40</f>
-        <v>0</v>
+      <c r="M40" s="90" t="s">
+        <v>414</v>
+      </c>
+      <c r="N40" s="79" t="s">
+        <v>378</v>
+      </c>
+      <c r="O40" s="56" t="s">
+        <v>378</v>
       </c>
       <c r="P40" s="30"/>
     </row>
     <row r="41" spans="1:16" ht="48" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
-      <c r="B41" s="67">
+      <c r="B41" s="62">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
@@ -4101,23 +4107,24 @@
       <c r="K41" s="31">
         <v>1</v>
       </c>
-      <c r="L41" s="79">
-        <f t="shared" ref="L41" si="30">K41*5</f>
+      <c r="L41" s="74">
+        <f t="shared" ref="L41" si="24">K41*5</f>
         <v>5</v>
       </c>
-      <c r="M41" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N41" s="85"/>
-      <c r="O41" s="55">
-        <f t="shared" ref="O41" si="31">N41*L41</f>
-        <v>0</v>
+      <c r="M41" s="90" t="s">
+        <v>414</v>
+      </c>
+      <c r="N41" s="80" t="s">
+        <v>378</v>
+      </c>
+      <c r="O41" s="55" t="s">
+        <v>378</v>
       </c>
       <c r="P41" s="31"/>
     </row>
     <row r="42" spans="1:16" ht="36" x14ac:dyDescent="0.25">
       <c r="A42" s="1"/>
-      <c r="B42" s="66">
+      <c r="B42" s="61">
         <f>ROW(B42) - ROW($B$9)</f>
         <v>33</v>
       </c>
@@ -4148,23 +4155,24 @@
       <c r="K42" s="30">
         <v>2</v>
       </c>
-      <c r="L42" s="78">
+      <c r="L42" s="73">
         <f>K42*5</f>
         <v>10</v>
       </c>
-      <c r="M42" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N42" s="84"/>
-      <c r="O42" s="56">
-        <f>N42*L42</f>
-        <v>0</v>
+      <c r="M42" s="90" t="s">
+        <v>414</v>
+      </c>
+      <c r="N42" s="79" t="s">
+        <v>378</v>
+      </c>
+      <c r="O42" s="56" t="s">
+        <v>378</v>
       </c>
       <c r="P42" s="30"/>
     </row>
     <row r="43" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A43" s="1"/>
-      <c r="B43" s="67">
+      <c r="B43" s="62">
         <f t="shared" si="0"/>
         <v>34</v>
       </c>
@@ -4175,19 +4183,19 @@
         <v>57</v>
       </c>
       <c r="E43" s="31" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="F43" s="31" t="s">
         <v>379</v>
       </c>
       <c r="G43" s="31" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="H43" s="31" t="s">
         <v>378</v>
       </c>
       <c r="I43" s="31" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="J43" s="31" t="s">
         <v>378</v>
@@ -4195,23 +4203,25 @@
       <c r="K43" s="31">
         <v>3</v>
       </c>
-      <c r="L43" s="79">
-        <f t="shared" ref="L43" si="32">K43*5</f>
+      <c r="L43" s="74">
+        <f t="shared" ref="L43" si="25">K43*5</f>
         <v>15</v>
       </c>
-      <c r="M43" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N43" s="85"/>
+      <c r="M43" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N43" s="80">
+        <v>0.90900000000000003</v>
+      </c>
       <c r="O43" s="55">
-        <f t="shared" ref="O43" si="33">N43*L43</f>
-        <v>0</v>
+        <f t="shared" ref="O43" si="26">N43*L43</f>
+        <v>13.635</v>
       </c>
       <c r="P43" s="31"/>
     </row>
-    <row r="44" spans="1:16" ht="24" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A44" s="1"/>
-      <c r="B44" s="66">
+      <c r="B44" s="61">
         <f>ROW(B44) - ROW($B$9)</f>
         <v>35</v>
       </c>
@@ -4242,23 +4252,24 @@
       <c r="K44" s="30">
         <v>1</v>
       </c>
-      <c r="L44" s="78">
+      <c r="L44" s="73">
         <f>K44*5</f>
         <v>5</v>
       </c>
-      <c r="M44" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N44" s="84"/>
-      <c r="O44" s="56">
-        <f>N44*L44</f>
-        <v>0</v>
+      <c r="M44" s="90" t="s">
+        <v>414</v>
+      </c>
+      <c r="N44" s="79" t="s">
+        <v>378</v>
+      </c>
+      <c r="O44" s="56" t="s">
+        <v>378</v>
       </c>
       <c r="P44" s="30"/>
     </row>
-    <row r="45" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A45" s="1"/>
-      <c r="B45" s="67">
+      <c r="B45" s="62">
         <f t="shared" si="0"/>
         <v>36</v>
       </c>
@@ -4289,23 +4300,24 @@
       <c r="K45" s="31">
         <v>1</v>
       </c>
-      <c r="L45" s="79">
-        <f t="shared" ref="L45" si="34">K45*5</f>
+      <c r="L45" s="74">
+        <f t="shared" ref="L45" si="27">K45*5</f>
         <v>5</v>
       </c>
-      <c r="M45" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N45" s="85"/>
-      <c r="O45" s="55">
-        <f t="shared" ref="O45" si="35">N45*L45</f>
-        <v>0</v>
+      <c r="M45" s="90" t="s">
+        <v>414</v>
+      </c>
+      <c r="N45" s="80" t="s">
+        <v>378</v>
+      </c>
+      <c r="O45" s="55" t="s">
+        <v>378</v>
       </c>
       <c r="P45" s="31"/>
     </row>
-    <row r="46" spans="1:16" ht="24" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A46" s="1"/>
-      <c r="B46" s="66">
+      <c r="B46" s="61">
         <f>ROW(B46) - ROW($B$9)</f>
         <v>37</v>
       </c>
@@ -4336,23 +4348,24 @@
       <c r="K46" s="30">
         <v>2</v>
       </c>
-      <c r="L46" s="78">
+      <c r="L46" s="73">
         <f>K46*5</f>
         <v>10</v>
       </c>
-      <c r="M46" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N46" s="84"/>
-      <c r="O46" s="56">
-        <f>N46*L46</f>
-        <v>0</v>
+      <c r="M46" s="90" t="s">
+        <v>414</v>
+      </c>
+      <c r="N46" s="79" t="s">
+        <v>378</v>
+      </c>
+      <c r="O46" s="79" t="s">
+        <v>378</v>
       </c>
       <c r="P46" s="30"/>
     </row>
-    <row r="47" spans="1:16" ht="24" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A47" s="1"/>
-      <c r="B47" s="67">
+      <c r="B47" s="62">
         <f t="shared" si="0"/>
         <v>38</v>
       </c>
@@ -4383,23 +4396,24 @@
       <c r="K47" s="31">
         <v>1</v>
       </c>
-      <c r="L47" s="79">
-        <f t="shared" ref="L47" si="36">K47*5</f>
+      <c r="L47" s="74">
+        <f t="shared" ref="L47" si="28">K47*5</f>
         <v>5</v>
       </c>
-      <c r="M47" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N47" s="85"/>
-      <c r="O47" s="55">
-        <f t="shared" ref="O47" si="37">N47*L47</f>
-        <v>0</v>
+      <c r="M47" s="90" t="s">
+        <v>414</v>
+      </c>
+      <c r="N47" s="80" t="s">
+        <v>378</v>
+      </c>
+      <c r="O47" s="80" t="s">
+        <v>378</v>
       </c>
       <c r="P47" s="31"/>
     </row>
     <row r="48" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A48" s="1"/>
-      <c r="B48" s="66">
+      <c r="B48" s="61">
         <f>ROW(B48) - ROW($B$9)</f>
         <v>39</v>
       </c>
@@ -4430,14 +4444,16 @@
       <c r="K48" s="44">
         <v>10</v>
       </c>
-      <c r="L48" s="80">
+      <c r="L48" s="75">
         <f>K48*5</f>
         <v>50</v>
       </c>
-      <c r="M48" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N48" s="86"/>
+      <c r="M48" s="88" t="s">
+        <v>378</v>
+      </c>
+      <c r="N48" s="81" t="s">
+        <v>378</v>
+      </c>
       <c r="O48" s="44" t="s">
         <v>378</v>
       </c>
@@ -4445,7 +4461,7 @@
     </row>
     <row r="49" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A49" s="1"/>
-      <c r="B49" s="67">
+      <c r="B49" s="62">
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
@@ -4464,7 +4480,9 @@
       <c r="G49" s="31" t="s">
         <v>256</v>
       </c>
-      <c r="H49" s="31"/>
+      <c r="H49" s="31" t="s">
+        <v>378</v>
+      </c>
       <c r="I49" s="31" t="s">
         <v>322</v>
       </c>
@@ -4474,23 +4492,25 @@
       <c r="K49" s="31">
         <v>1</v>
       </c>
-      <c r="L49" s="79">
-        <f t="shared" ref="L49" si="38">K49*5</f>
+      <c r="L49" s="74">
+        <f t="shared" ref="L49" si="29">K49*5</f>
         <v>5</v>
       </c>
-      <c r="M49" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N49" s="85"/>
+      <c r="M49" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N49" s="80">
+        <v>0.14000000000000001</v>
+      </c>
       <c r="O49" s="55">
-        <f t="shared" ref="O49" si="39">N49*L49</f>
-        <v>0</v>
+        <f t="shared" ref="O49" si="30">N49*L49</f>
+        <v>0.70000000000000007</v>
       </c>
       <c r="P49" s="31"/>
     </row>
     <row r="50" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A50" s="1"/>
-      <c r="B50" s="66">
+      <c r="B50" s="61">
         <f>ROW(B50) - ROW($B$9)</f>
         <v>41</v>
       </c>
@@ -4521,23 +4541,25 @@
       <c r="K50" s="30">
         <v>2</v>
       </c>
-      <c r="L50" s="78">
+      <c r="L50" s="73">
         <f>K50*5</f>
         <v>10</v>
       </c>
-      <c r="M50" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N50" s="84"/>
+      <c r="M50" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N50" s="79">
+        <v>0.33600000000000002</v>
+      </c>
       <c r="O50" s="56">
         <f>N50*L50</f>
-        <v>0</v>
+        <v>3.3600000000000003</v>
       </c>
       <c r="P50" s="30"/>
     </row>
     <row r="51" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A51" s="1"/>
-      <c r="B51" s="67">
+      <c r="B51" s="62">
         <f t="shared" si="0"/>
         <v>42</v>
       </c>
@@ -4556,7 +4578,9 @@
       <c r="G51" s="31" t="s">
         <v>207</v>
       </c>
-      <c r="H51" s="31"/>
+      <c r="H51" s="31" t="s">
+        <v>378</v>
+      </c>
       <c r="I51" s="31" t="s">
         <v>324</v>
       </c>
@@ -4566,23 +4590,25 @@
       <c r="K51" s="31">
         <v>1</v>
       </c>
-      <c r="L51" s="79">
-        <f t="shared" ref="L51" si="40">K51*5</f>
+      <c r="L51" s="74">
+        <f t="shared" ref="L51" si="31">K51*5</f>
         <v>5</v>
       </c>
-      <c r="M51" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N51" s="85"/>
+      <c r="M51" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N51" s="80">
+        <v>0.51</v>
+      </c>
       <c r="O51" s="55">
-        <f t="shared" ref="O51" si="41">N51*L51</f>
-        <v>0</v>
+        <f t="shared" ref="O51" si="32">N51*L51</f>
+        <v>2.5499999999999998</v>
       </c>
       <c r="P51" s="31"/>
     </row>
     <row r="52" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A52" s="1"/>
-      <c r="B52" s="66">
+      <c r="B52" s="61">
         <f>ROW(B52) - ROW($B$9)</f>
         <v>43</v>
       </c>
@@ -4601,7 +4627,9 @@
       <c r="G52" s="30" t="s">
         <v>258</v>
       </c>
-      <c r="H52" s="30"/>
+      <c r="H52" s="30" t="s">
+        <v>378</v>
+      </c>
       <c r="I52" s="30" t="s">
         <v>294</v>
       </c>
@@ -4611,23 +4639,25 @@
       <c r="K52" s="30">
         <v>1</v>
       </c>
-      <c r="L52" s="78">
+      <c r="L52" s="73">
         <f>K52*5</f>
         <v>5</v>
       </c>
-      <c r="M52" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N52" s="84"/>
+      <c r="M52" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N52" s="79">
+        <v>0.1</v>
+      </c>
       <c r="O52" s="56">
         <f>N52*L52</f>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="P52" s="30"/>
     </row>
     <row r="53" spans="1:16" ht="24" x14ac:dyDescent="0.25">
       <c r="A53" s="1"/>
-      <c r="B53" s="67">
+      <c r="B53" s="62">
         <f t="shared" si="0"/>
         <v>44</v>
       </c>
@@ -4635,7 +4665,7 @@
         <v>17</v>
       </c>
       <c r="D53" s="31" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="E53" s="31" t="s">
         <v>142</v>
@@ -4646,7 +4676,9 @@
       <c r="G53" s="31" t="s">
         <v>259</v>
       </c>
-      <c r="H53" s="31"/>
+      <c r="H53" s="31" t="s">
+        <v>378</v>
+      </c>
       <c r="I53" s="31" t="s">
         <v>294</v>
       </c>
@@ -4656,23 +4688,25 @@
       <c r="K53" s="31">
         <v>12</v>
       </c>
-      <c r="L53" s="79">
-        <f t="shared" ref="L53" si="42">K53*5</f>
+      <c r="L53" s="74">
+        <f t="shared" ref="L53" si="33">K53*5</f>
         <v>60</v>
       </c>
-      <c r="M53" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N53" s="85"/>
+      <c r="M53" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N53" s="80">
+        <v>1.6199999999999999E-2</v>
+      </c>
       <c r="O53" s="55">
-        <f t="shared" ref="O53" si="43">N53*L53</f>
-        <v>0</v>
+        <f t="shared" ref="O53" si="34">N53*L53</f>
+        <v>0.97199999999999998</v>
       </c>
       <c r="P53" s="31"/>
     </row>
     <row r="54" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A54" s="1"/>
-      <c r="B54" s="66">
+      <c r="B54" s="61">
         <f>ROW(B54) - ROW($B$9)</f>
         <v>45</v>
       </c>
@@ -4703,23 +4737,25 @@
       <c r="K54" s="30">
         <v>7</v>
       </c>
-      <c r="L54" s="78">
+      <c r="L54" s="73">
         <f>K54*5</f>
         <v>35</v>
       </c>
-      <c r="M54" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N54" s="84"/>
+      <c r="M54" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N54" s="79">
+        <v>2.5999999999999999E-2</v>
+      </c>
       <c r="O54" s="56">
         <f>N54*L54</f>
-        <v>0</v>
+        <v>0.90999999999999992</v>
       </c>
       <c r="P54" s="30"/>
     </row>
     <row r="55" spans="1:16" ht="36" x14ac:dyDescent="0.25">
       <c r="A55" s="1"/>
-      <c r="B55" s="67">
+      <c r="B55" s="62">
         <f t="shared" si="0"/>
         <v>46</v>
       </c>
@@ -4750,23 +4786,24 @@
       <c r="K55" s="31">
         <v>1</v>
       </c>
-      <c r="L55" s="79">
-        <f t="shared" ref="L55" si="44">K55*5</f>
+      <c r="L55" s="74">
+        <f t="shared" ref="L55" si="35">K55*5</f>
         <v>5</v>
       </c>
-      <c r="M55" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N55" s="85"/>
-      <c r="O55" s="55">
-        <f t="shared" ref="O55" si="45">N55*L55</f>
-        <v>0</v>
+      <c r="M55" s="90" t="s">
+        <v>414</v>
+      </c>
+      <c r="N55" s="80" t="s">
+        <v>378</v>
+      </c>
+      <c r="O55" s="55" t="s">
+        <v>378</v>
       </c>
       <c r="P55" s="31"/>
     </row>
     <row r="56" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A56" s="1"/>
-      <c r="B56" s="66">
+      <c r="B56" s="61">
         <f>ROW(B56) - ROW($B$9)</f>
         <v>47</v>
       </c>
@@ -4797,23 +4834,25 @@
       <c r="K56" s="30">
         <v>2</v>
       </c>
-      <c r="L56" s="78">
+      <c r="L56" s="73">
         <f>K56*5</f>
         <v>10</v>
       </c>
-      <c r="M56" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N56" s="84"/>
+      <c r="M56" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N56" s="79">
+        <v>0.02</v>
+      </c>
       <c r="O56" s="56">
         <f>N56*L56</f>
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="P56" s="30"/>
     </row>
     <row r="57" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A57" s="1"/>
-      <c r="B57" s="67">
+      <c r="B57" s="62">
         <f t="shared" si="0"/>
         <v>48</v>
       </c>
@@ -4821,7 +4860,7 @@
         <v>17</v>
       </c>
       <c r="D57" s="31" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="E57" s="31" t="s">
         <v>146</v>
@@ -4829,11 +4868,11 @@
       <c r="F57" s="31" t="s">
         <v>208</v>
       </c>
-      <c r="G57" s="44" t="s">
+      <c r="G57" s="91" t="s">
         <v>263</v>
       </c>
       <c r="H57" s="31" t="s">
-        <v>391</v>
+        <v>378</v>
       </c>
       <c r="I57" s="31" t="s">
         <v>294</v>
@@ -4844,23 +4883,25 @@
       <c r="K57" s="31">
         <v>2</v>
       </c>
-      <c r="L57" s="79">
-        <f t="shared" ref="L57" si="46">K57*5</f>
+      <c r="L57" s="74">
+        <f t="shared" ref="L57" si="36">K57*5</f>
         <v>10</v>
       </c>
-      <c r="M57" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N57" s="85"/>
+      <c r="M57" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N57" s="80">
+        <v>0.02</v>
+      </c>
       <c r="O57" s="55">
-        <f t="shared" ref="O57" si="47">N57*L57</f>
-        <v>0</v>
+        <f t="shared" ref="O57" si="37">N57*L57</f>
+        <v>0.2</v>
       </c>
       <c r="P57" s="31"/>
     </row>
     <row r="58" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A58" s="1"/>
-      <c r="B58" s="66">
+      <c r="B58" s="61">
         <f>ROW(B58) - ROW($B$9)</f>
         <v>49</v>
       </c>
@@ -4879,7 +4920,9 @@
       <c r="G58" s="30" t="s">
         <v>264</v>
       </c>
-      <c r="H58" s="30"/>
+      <c r="H58" s="30" t="s">
+        <v>378</v>
+      </c>
       <c r="I58" s="30" t="s">
         <v>294</v>
       </c>
@@ -4889,23 +4932,25 @@
       <c r="K58" s="30">
         <v>2</v>
       </c>
-      <c r="L58" s="78">
+      <c r="L58" s="73">
         <f>K58*5</f>
         <v>10</v>
       </c>
-      <c r="M58" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N58" s="84"/>
+      <c r="M58" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N58" s="79">
+        <v>1.4E-2</v>
+      </c>
       <c r="O58" s="56">
         <f>N58*L58</f>
-        <v>0</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="P58" s="30"/>
     </row>
     <row r="59" spans="1:16" ht="36" x14ac:dyDescent="0.25">
       <c r="A59" s="1"/>
-      <c r="B59" s="67">
+      <c r="B59" s="62">
         <f t="shared" si="0"/>
         <v>50</v>
       </c>
@@ -4924,7 +4969,9 @@
       <c r="G59" s="31" t="s">
         <v>265</v>
       </c>
-      <c r="H59" s="31"/>
+      <c r="H59" s="31" t="s">
+        <v>378</v>
+      </c>
       <c r="I59" s="31" t="s">
         <v>294</v>
       </c>
@@ -4934,23 +4981,25 @@
       <c r="K59" s="31">
         <v>22</v>
       </c>
-      <c r="L59" s="79">
-        <f t="shared" ref="L59" si="48">K59*5</f>
+      <c r="L59" s="74">
+        <f t="shared" ref="L59" si="38">K59*5</f>
         <v>110</v>
       </c>
-      <c r="M59" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N59" s="85"/>
+      <c r="M59" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N59" s="80">
+        <v>7.0000000000000001E-3</v>
+      </c>
       <c r="O59" s="55">
-        <f t="shared" ref="O59" si="49">N59*L59</f>
-        <v>0</v>
+        <f t="shared" ref="O59" si="39">N59*L59</f>
+        <v>0.77</v>
       </c>
       <c r="P59" s="31"/>
     </row>
     <row r="60" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A60" s="1"/>
-      <c r="B60" s="66">
+      <c r="B60" s="61">
         <f>ROW(B60) - ROW($B$9)</f>
         <v>51</v>
       </c>
@@ -4969,7 +5018,9 @@
       <c r="G60" s="30" t="s">
         <v>266</v>
       </c>
-      <c r="H60" s="30"/>
+      <c r="H60" s="30" t="s">
+        <v>378</v>
+      </c>
       <c r="I60" s="30" t="s">
         <v>294</v>
       </c>
@@ -4979,23 +5030,25 @@
       <c r="K60" s="30">
         <v>1</v>
       </c>
-      <c r="L60" s="78">
+      <c r="L60" s="73">
         <f>K60*5</f>
         <v>5</v>
       </c>
-      <c r="M60" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N60" s="84"/>
+      <c r="M60" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N60" s="79">
+        <v>0.1</v>
+      </c>
       <c r="O60" s="56">
         <f>N60*L60</f>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="P60" s="30"/>
     </row>
     <row r="61" spans="1:16" ht="24" x14ac:dyDescent="0.25">
       <c r="A61" s="1"/>
-      <c r="B61" s="66">
+      <c r="B61" s="61">
         <f>ROW(B61) - ROW($B$9)</f>
         <v>52</v>
       </c>
@@ -5003,7 +5056,7 @@
         <v>17</v>
       </c>
       <c r="D61" s="31" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="E61" s="30" t="s">
         <v>154</v>
@@ -5014,7 +5067,9 @@
       <c r="G61" s="30" t="s">
         <v>271</v>
       </c>
-      <c r="H61" s="30"/>
+      <c r="H61" s="30" t="s">
+        <v>378</v>
+      </c>
       <c r="I61" s="30" t="s">
         <v>294</v>
       </c>
@@ -5024,23 +5079,25 @@
       <c r="K61" s="30">
         <v>11</v>
       </c>
-      <c r="L61" s="78">
+      <c r="L61" s="73">
         <f>K61*5</f>
         <v>55</v>
       </c>
-      <c r="M61" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N61" s="84"/>
+      <c r="M61" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N61" s="79">
+        <v>6.4000000000000003E-3</v>
+      </c>
       <c r="O61" s="56">
         <f>N61*L61</f>
-        <v>0</v>
+        <v>0.35200000000000004</v>
       </c>
       <c r="P61" s="31"/>
     </row>
     <row r="62" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A62" s="1"/>
-      <c r="B62" s="66">
+      <c r="B62" s="61">
         <f>ROW(B62) - ROW($B$9)</f>
         <v>53</v>
       </c>
@@ -5059,7 +5116,9 @@
       <c r="G62" s="30" t="s">
         <v>267</v>
       </c>
-      <c r="H62" s="30"/>
+      <c r="H62" s="30" t="s">
+        <v>378</v>
+      </c>
       <c r="I62" s="30" t="s">
         <v>294</v>
       </c>
@@ -5069,23 +5128,25 @@
       <c r="K62" s="30">
         <v>4</v>
       </c>
-      <c r="L62" s="78">
+      <c r="L62" s="73">
         <f>K62*5</f>
         <v>20</v>
       </c>
-      <c r="M62" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N62" s="84"/>
+      <c r="M62" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N62" s="79">
+        <v>1.4E-2</v>
+      </c>
       <c r="O62" s="56">
         <f>N62*L62</f>
-        <v>0</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="P62" s="30"/>
     </row>
     <row r="63" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A63" s="1"/>
-      <c r="B63" s="67">
+      <c r="B63" s="62">
         <f t="shared" si="0"/>
         <v>54</v>
       </c>
@@ -5104,7 +5165,9 @@
       <c r="G63" s="31" t="s">
         <v>268</v>
       </c>
-      <c r="H63" s="31"/>
+      <c r="H63" s="31" t="s">
+        <v>378</v>
+      </c>
       <c r="I63" s="31" t="s">
         <v>294</v>
       </c>
@@ -5114,23 +5177,25 @@
       <c r="K63" s="31">
         <v>1</v>
       </c>
-      <c r="L63" s="79">
-        <f t="shared" ref="L63" si="50">K63*5</f>
+      <c r="L63" s="74">
+        <f t="shared" ref="L63" si="40">K63*5</f>
         <v>5</v>
       </c>
-      <c r="M63" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N63" s="85"/>
+      <c r="M63" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N63" s="80">
+        <v>0.1</v>
+      </c>
       <c r="O63" s="55">
-        <f t="shared" ref="O63" si="51">N63*L63</f>
-        <v>0</v>
+        <f t="shared" ref="O63" si="41">N63*L63</f>
+        <v>0.5</v>
       </c>
       <c r="P63" s="31"/>
     </row>
     <row r="64" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A64" s="1"/>
-      <c r="B64" s="66">
+      <c r="B64" s="61">
         <f>ROW(B64) - ROW($B$9)</f>
         <v>55</v>
       </c>
@@ -5149,7 +5214,9 @@
       <c r="G64" s="30" t="s">
         <v>269</v>
       </c>
-      <c r="H64" s="30"/>
+      <c r="H64" s="30" t="s">
+        <v>378</v>
+      </c>
       <c r="I64" s="30" t="s">
         <v>294</v>
       </c>
@@ -5159,23 +5226,25 @@
       <c r="K64" s="30">
         <v>1</v>
       </c>
-      <c r="L64" s="78">
+      <c r="L64" s="73">
         <f>K64*5</f>
         <v>5</v>
       </c>
-      <c r="M64" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N64" s="84"/>
+      <c r="M64" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N64" s="79">
+        <v>0.1</v>
+      </c>
       <c r="O64" s="56">
         <f>N64*L64</f>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="P64" s="30"/>
     </row>
     <row r="65" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A65" s="1"/>
-      <c r="B65" s="67">
+      <c r="B65" s="62">
         <f t="shared" si="0"/>
         <v>56</v>
       </c>
@@ -5194,7 +5263,9 @@
       <c r="G65" s="31" t="s">
         <v>270</v>
       </c>
-      <c r="H65" s="31"/>
+      <c r="H65" s="31" t="s">
+        <v>378</v>
+      </c>
       <c r="I65" s="31" t="s">
         <v>294</v>
       </c>
@@ -5204,23 +5275,25 @@
       <c r="K65" s="31">
         <v>1</v>
       </c>
-      <c r="L65" s="79">
-        <f t="shared" ref="L65:L66" si="52">K65*5</f>
+      <c r="L65" s="74">
+        <f t="shared" ref="L65:L66" si="42">K65*5</f>
         <v>5</v>
       </c>
-      <c r="M65" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N65" s="85"/>
+      <c r="M65" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N65" s="80">
+        <v>0.34</v>
+      </c>
       <c r="O65" s="55">
-        <f t="shared" ref="O65:O66" si="53">N65*L65</f>
-        <v>0</v>
+        <f t="shared" ref="O65:O66" si="43">N65*L65</f>
+        <v>1.7000000000000002</v>
       </c>
       <c r="P65" s="31"/>
     </row>
     <row r="66" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A66" s="1"/>
-      <c r="B66" s="67">
+      <c r="B66" s="62">
         <f t="shared" si="0"/>
         <v>57</v>
       </c>
@@ -5236,11 +5309,11 @@
       <c r="F66" s="31" t="s">
         <v>206</v>
       </c>
-      <c r="G66" s="44" t="s">
+      <c r="G66" s="91" t="s">
         <v>272</v>
       </c>
       <c r="H66" s="31" t="s">
-        <v>392</v>
+        <v>415</v>
       </c>
       <c r="I66" s="31" t="s">
         <v>326</v>
@@ -5251,23 +5324,25 @@
       <c r="K66" s="31">
         <v>4</v>
       </c>
-      <c r="L66" s="79">
-        <f t="shared" si="52"/>
+      <c r="L66" s="74">
+        <f t="shared" si="42"/>
         <v>20</v>
       </c>
-      <c r="M66" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N66" s="85"/>
+      <c r="M66" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N66" s="80">
+        <v>0.11600000000000001</v>
+      </c>
       <c r="O66" s="55">
-        <f t="shared" si="53"/>
-        <v>0</v>
+        <f t="shared" si="43"/>
+        <v>2.3200000000000003</v>
       </c>
       <c r="P66" s="30"/>
     </row>
     <row r="67" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A67" s="1"/>
-      <c r="B67" s="66">
+      <c r="B67" s="61">
         <f>ROW(B67) - ROW($B$9)</f>
         <v>58</v>
       </c>
@@ -5286,7 +5361,9 @@
       <c r="G67" s="30" t="s">
         <v>273</v>
       </c>
-      <c r="H67" s="30"/>
+      <c r="H67" s="30" t="s">
+        <v>378</v>
+      </c>
       <c r="I67" s="30" t="s">
         <v>294</v>
       </c>
@@ -5296,23 +5373,25 @@
       <c r="K67" s="30">
         <v>1</v>
       </c>
-      <c r="L67" s="78">
+      <c r="L67" s="73">
         <f>K67*5</f>
         <v>5</v>
       </c>
-      <c r="M67" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N67" s="84"/>
+      <c r="M67" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N67" s="79">
+        <v>0.1</v>
+      </c>
       <c r="O67" s="56">
         <f>N67*L67</f>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="P67" s="31"/>
     </row>
     <row r="68" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A68" s="1"/>
-      <c r="B68" s="67">
+      <c r="B68" s="62">
         <f t="shared" si="0"/>
         <v>59</v>
       </c>
@@ -5331,7 +5410,9 @@
       <c r="G68" s="31" t="s">
         <v>274</v>
       </c>
-      <c r="H68" s="31"/>
+      <c r="H68" s="31" t="s">
+        <v>378</v>
+      </c>
       <c r="I68" s="31" t="s">
         <v>323</v>
       </c>
@@ -5341,23 +5422,25 @@
       <c r="K68" s="31">
         <v>1</v>
       </c>
-      <c r="L68" s="79">
-        <f t="shared" ref="L68" si="54">K68*5</f>
+      <c r="L68" s="74">
+        <f t="shared" ref="L68" si="44">K68*5</f>
         <v>5</v>
       </c>
-      <c r="M68" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N68" s="85"/>
+      <c r="M68" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N68" s="80">
+        <v>0.41</v>
+      </c>
       <c r="O68" s="55">
-        <f t="shared" ref="O68" si="55">N68*L68</f>
-        <v>0</v>
+        <f t="shared" ref="O68" si="45">N68*L68</f>
+        <v>2.0499999999999998</v>
       </c>
       <c r="P68" s="30"/>
     </row>
     <row r="69" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A69" s="1"/>
-      <c r="B69" s="66">
+      <c r="B69" s="61">
         <f>ROW(B69) - ROW($B$9)</f>
         <v>60</v>
       </c>
@@ -5376,7 +5459,9 @@
       <c r="G69" s="30" t="s">
         <v>275</v>
       </c>
-      <c r="H69" s="30"/>
+      <c r="H69" s="30" t="s">
+        <v>378</v>
+      </c>
       <c r="I69" s="30" t="s">
         <v>294</v>
       </c>
@@ -5386,23 +5471,25 @@
       <c r="K69" s="30">
         <v>2</v>
       </c>
-      <c r="L69" s="78">
+      <c r="L69" s="73">
         <f>K69*5</f>
         <v>10</v>
       </c>
-      <c r="M69" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N69" s="84"/>
+      <c r="M69" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N69" s="79">
+        <v>1.7999999999999999E-2</v>
+      </c>
       <c r="O69" s="56">
         <f>N69*L69</f>
-        <v>0</v>
+        <v>0.18</v>
       </c>
       <c r="P69" s="31"/>
     </row>
     <row r="70" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A70" s="1"/>
-      <c r="B70" s="67">
+      <c r="B70" s="62">
         <f t="shared" si="0"/>
         <v>61</v>
       </c>
@@ -5421,7 +5508,9 @@
       <c r="G70" s="31" t="s">
         <v>276</v>
       </c>
-      <c r="H70" s="31"/>
+      <c r="H70" s="31" t="s">
+        <v>378</v>
+      </c>
       <c r="I70" s="31" t="s">
         <v>294</v>
       </c>
@@ -5431,40 +5520,42 @@
       <c r="K70" s="31">
         <v>1</v>
       </c>
-      <c r="L70" s="79">
-        <f t="shared" ref="L70:L71" si="56">K70*5</f>
+      <c r="L70" s="74">
+        <f t="shared" ref="L70:L71" si="46">K70*5</f>
         <v>5</v>
       </c>
-      <c r="M70" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N70" s="85"/>
+      <c r="M70" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N70" s="80">
+        <v>0.1</v>
+      </c>
       <c r="O70" s="55">
-        <f t="shared" ref="O70:O71" si="57">N70*L70</f>
-        <v>0</v>
+        <f t="shared" ref="O70:O71" si="47">N70*L70</f>
+        <v>0.5</v>
       </c>
       <c r="P70" s="30"/>
     </row>
     <row r="71" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A71" s="1"/>
-      <c r="B71" s="67">
+      <c r="B71" s="62">
         <f t="shared" si="0"/>
         <v>62</v>
       </c>
       <c r="C71" s="45" t="s">
+        <v>404</v>
+      </c>
+      <c r="D71" s="31" t="s">
+        <v>405</v>
+      </c>
+      <c r="E71" s="31" t="s">
         <v>406</v>
-      </c>
-      <c r="D71" s="31" t="s">
-        <v>407</v>
-      </c>
-      <c r="E71" s="31" t="s">
-        <v>408</v>
       </c>
       <c r="F71" s="31" t="s">
         <v>379</v>
       </c>
       <c r="G71" s="31" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="H71" s="31" t="s">
         <v>378</v>
@@ -5478,23 +5569,25 @@
       <c r="K71" s="31">
         <v>5</v>
       </c>
-      <c r="L71" s="79">
-        <f t="shared" si="56"/>
+      <c r="L71" s="74">
+        <f t="shared" si="46"/>
         <v>25</v>
       </c>
-      <c r="M71" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N71" s="85"/>
+      <c r="M71" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N71" s="80">
+        <v>8.9599999999999999E-2</v>
+      </c>
       <c r="O71" s="55">
-        <f t="shared" si="57"/>
-        <v>0</v>
+        <f t="shared" si="47"/>
+        <v>2.2399999999999998</v>
       </c>
       <c r="P71" s="31"/>
     </row>
     <row r="72" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A72" s="1"/>
-      <c r="B72" s="66">
+      <c r="B72" s="61">
         <f>ROW(B72) - ROW($B$9)</f>
         <v>63</v>
       </c>
@@ -5525,14 +5618,16 @@
       <c r="K72" s="46">
         <v>2</v>
       </c>
-      <c r="L72" s="81">
+      <c r="L72" s="76">
         <f>K72*5</f>
         <v>10</v>
       </c>
-      <c r="M72" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N72" s="87"/>
+      <c r="M72" s="88" t="s">
+        <v>378</v>
+      </c>
+      <c r="N72" s="82" t="s">
+        <v>378</v>
+      </c>
       <c r="O72" s="46" t="s">
         <v>378</v>
       </c>
@@ -5540,7 +5635,7 @@
     </row>
     <row r="73" spans="1:16" ht="24" x14ac:dyDescent="0.25">
       <c r="A73" s="1"/>
-      <c r="B73" s="67">
+      <c r="B73" s="62">
         <f t="shared" si="0"/>
         <v>64</v>
       </c>
@@ -5571,23 +5666,25 @@
       <c r="K73" s="31">
         <v>1</v>
       </c>
-      <c r="L73" s="79">
-        <f t="shared" ref="L73" si="58">K73*5</f>
+      <c r="L73" s="74">
+        <f t="shared" ref="L73" si="48">K73*5</f>
         <v>5</v>
       </c>
-      <c r="M73" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N73" s="85"/>
+      <c r="M73" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N73" s="80">
+        <v>0.14000000000000001</v>
+      </c>
       <c r="O73" s="55">
-        <f t="shared" ref="O73" si="59">N73*L73</f>
-        <v>0</v>
+        <f t="shared" ref="O73" si="49">N73*L73</f>
+        <v>0.70000000000000007</v>
       </c>
       <c r="P73" s="31"/>
     </row>
     <row r="74" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A74" s="1"/>
-      <c r="B74" s="66">
+      <c r="B74" s="61">
         <f>ROW(B74) - ROW($B$9)</f>
         <v>65</v>
       </c>
@@ -5618,23 +5715,25 @@
       <c r="K74" s="30">
         <v>1</v>
       </c>
-      <c r="L74" s="78">
+      <c r="L74" s="73">
         <f>K74*5</f>
         <v>5</v>
       </c>
-      <c r="M74" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N74" s="84"/>
+      <c r="M74" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N74" s="79">
+        <v>5.28</v>
+      </c>
       <c r="O74" s="56">
         <f>N74*L74</f>
-        <v>0</v>
+        <v>26.400000000000002</v>
       </c>
       <c r="P74" s="30"/>
     </row>
     <row r="75" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A75" s="1"/>
-      <c r="B75" s="67">
+      <c r="B75" s="62">
         <f t="shared" si="0"/>
         <v>66</v>
       </c>
@@ -5665,23 +5764,25 @@
       <c r="K75" s="31">
         <v>1</v>
       </c>
-      <c r="L75" s="79">
-        <f t="shared" ref="L75" si="60">K75*5</f>
+      <c r="L75" s="74">
+        <f t="shared" ref="L75" si="50">K75*5</f>
         <v>5</v>
       </c>
-      <c r="M75" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N75" s="85"/>
+      <c r="M75" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N75" s="80">
+        <v>0.88</v>
+      </c>
       <c r="O75" s="55">
-        <f t="shared" ref="O75" si="61">N75*L75</f>
-        <v>0</v>
+        <f t="shared" ref="O75" si="51">N75*L75</f>
+        <v>4.4000000000000004</v>
       </c>
       <c r="P75" s="31"/>
     </row>
     <row r="76" spans="1:16" ht="36" x14ac:dyDescent="0.25">
       <c r="A76" s="1"/>
-      <c r="B76" s="66">
+      <c r="B76" s="61">
         <f>ROW(B76) - ROW($B$9)</f>
         <v>67</v>
       </c>
@@ -5712,23 +5813,24 @@
       <c r="K76" s="30">
         <v>1</v>
       </c>
-      <c r="L76" s="78">
+      <c r="L76" s="73">
         <f>K76*5</f>
         <v>5</v>
       </c>
-      <c r="M76" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N76" s="84"/>
-      <c r="O76" s="56">
-        <f>N76*L76</f>
-        <v>0</v>
+      <c r="M76" s="90" t="s">
+        <v>414</v>
+      </c>
+      <c r="N76" s="80" t="s">
+        <v>378</v>
+      </c>
+      <c r="O76" s="55" t="s">
+        <v>378</v>
       </c>
       <c r="P76" s="30"/>
     </row>
     <row r="77" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A77" s="1"/>
-      <c r="B77" s="67">
+      <c r="B77" s="62">
         <f t="shared" si="0"/>
         <v>68</v>
       </c>
@@ -5759,23 +5861,25 @@
       <c r="K77" s="31">
         <v>1</v>
       </c>
-      <c r="L77" s="79">
-        <f t="shared" ref="L77" si="62">K77*5</f>
+      <c r="L77" s="74">
+        <f t="shared" ref="L77" si="52">K77*5</f>
         <v>5</v>
       </c>
-      <c r="M77" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N77" s="85"/>
+      <c r="M77" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N77" s="80">
+        <v>2.89</v>
+      </c>
       <c r="O77" s="55">
-        <f t="shared" ref="O77" si="63">N77*L77</f>
-        <v>0</v>
+        <f t="shared" ref="O77" si="53">N77*L77</f>
+        <v>14.450000000000001</v>
       </c>
       <c r="P77" s="31"/>
     </row>
     <row r="78" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A78" s="1"/>
-      <c r="B78" s="66">
+      <c r="B78" s="61">
         <f>ROW(B78) - ROW($B$9)</f>
         <v>69</v>
       </c>
@@ -5804,23 +5908,25 @@
       <c r="K78" s="30">
         <v>1</v>
       </c>
-      <c r="L78" s="78">
+      <c r="L78" s="73">
         <f>K78*5</f>
         <v>5</v>
       </c>
-      <c r="M78" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N78" s="84"/>
+      <c r="M78" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N78" s="79">
+        <v>1.1499999999999999</v>
+      </c>
       <c r="O78" s="56">
         <f>N78*L78</f>
-        <v>0</v>
+        <v>5.75</v>
       </c>
       <c r="P78" s="30"/>
     </row>
     <row r="79" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A79" s="1"/>
-      <c r="B79" s="68">
+      <c r="B79" s="63">
         <f t="shared" si="0"/>
         <v>70</v>
       </c>
@@ -5851,23 +5957,25 @@
       <c r="K79" s="49">
         <v>1</v>
       </c>
-      <c r="L79" s="82">
-        <f t="shared" ref="L79" si="64">K79*5</f>
+      <c r="L79" s="77">
+        <f t="shared" ref="L79" si="54">K79*5</f>
         <v>5</v>
       </c>
-      <c r="M79" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N79" s="88"/>
+      <c r="M79" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N79" s="83">
+        <v>2.5099999999999998</v>
+      </c>
       <c r="O79" s="57">
-        <f t="shared" ref="O79" si="65">N79*L79</f>
-        <v>0</v>
+        <f t="shared" ref="O79" si="55">N79*L79</f>
+        <v>12.549999999999999</v>
       </c>
       <c r="P79" s="31"/>
     </row>
     <row r="80" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A80" s="1"/>
-      <c r="B80" s="69">
+      <c r="B80" s="64">
         <f>ROW(B80) - ROW($B$9)</f>
         <v>71</v>
       </c>
@@ -5898,23 +6006,25 @@
       <c r="K80" s="51">
         <v>1</v>
       </c>
-      <c r="L80" s="83">
+      <c r="L80" s="78">
         <f>K80*5</f>
         <v>5</v>
       </c>
-      <c r="M80" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N80" s="89"/>
+      <c r="M80" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N80" s="84">
+        <v>0.9</v>
+      </c>
       <c r="O80" s="58">
         <f>N80*L80</f>
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="P80" s="30"/>
     </row>
     <row r="81" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A81" s="1"/>
-      <c r="B81" s="67">
+      <c r="B81" s="62">
         <f t="shared" si="0"/>
         <v>72</v>
       </c>
@@ -5943,23 +6053,25 @@
       <c r="K81" s="31">
         <v>1</v>
       </c>
-      <c r="L81" s="79">
-        <f t="shared" ref="L81" si="66">K81*5</f>
+      <c r="L81" s="74">
+        <f t="shared" ref="L81" si="56">K81*5</f>
         <v>5</v>
       </c>
-      <c r="M81" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N81" s="85"/>
+      <c r="M81" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N81" s="80">
+        <v>1.53</v>
+      </c>
       <c r="O81" s="55">
-        <f t="shared" ref="O81" si="67">N81*L81</f>
-        <v>0</v>
+        <f t="shared" ref="O81" si="57">N81*L81</f>
+        <v>7.65</v>
       </c>
       <c r="P81" s="31"/>
     </row>
     <row r="82" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A82" s="1"/>
-      <c r="B82" s="69">
+      <c r="B82" s="64">
         <f>ROW(B82) - ROW($B$9)</f>
         <v>73</v>
       </c>
@@ -5990,23 +6102,25 @@
       <c r="K82" s="51">
         <v>1</v>
       </c>
-      <c r="L82" s="83">
+      <c r="L82" s="78">
         <f>K82*5</f>
         <v>5</v>
       </c>
-      <c r="M82" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N82" s="89"/>
+      <c r="M82" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N82" s="84">
+        <v>3.54</v>
+      </c>
       <c r="O82" s="58">
         <f>N82*L82</f>
-        <v>0</v>
+        <v>17.7</v>
       </c>
       <c r="P82" s="30"/>
     </row>
     <row r="83" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A83" s="1"/>
-      <c r="B83" s="67">
+      <c r="B83" s="62">
         <f t="shared" si="0"/>
         <v>74</v>
       </c>
@@ -6037,23 +6151,25 @@
       <c r="K83" s="31">
         <v>3</v>
       </c>
-      <c r="L83" s="79">
-        <f t="shared" ref="L83" si="68">K83*5</f>
+      <c r="L83" s="74">
+        <f t="shared" ref="L83" si="58">K83*5</f>
         <v>15</v>
       </c>
-      <c r="M83" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N83" s="85"/>
+      <c r="M83" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N83" s="80">
+        <v>1.69</v>
+      </c>
       <c r="O83" s="55">
-        <f t="shared" ref="O83" si="69">N83*L83</f>
-        <v>0</v>
+        <f t="shared" ref="O83" si="59">N83*L83</f>
+        <v>25.349999999999998</v>
       </c>
       <c r="P83" s="31"/>
     </row>
     <row r="84" spans="1:16" ht="60" x14ac:dyDescent="0.25">
       <c r="A84" s="1"/>
-      <c r="B84" s="66">
+      <c r="B84" s="61">
         <f>ROW(B84) - ROW($B$9)</f>
         <v>75</v>
       </c>
@@ -6084,23 +6200,24 @@
       <c r="K84" s="30">
         <v>1</v>
       </c>
-      <c r="L84" s="78">
+      <c r="L84" s="73">
         <f>K84*5</f>
         <v>5</v>
       </c>
-      <c r="M84" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N84" s="84"/>
-      <c r="O84" s="56">
-        <f>N84*L84</f>
-        <v>0</v>
+      <c r="M84" s="90" t="s">
+        <v>414</v>
+      </c>
+      <c r="N84" s="80" t="s">
+        <v>378</v>
+      </c>
+      <c r="O84" s="55" t="s">
+        <v>378</v>
       </c>
       <c r="P84" s="30"/>
     </row>
     <row r="85" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A85" s="1"/>
-      <c r="B85" s="67">
+      <c r="B85" s="62">
         <f t="shared" si="0"/>
         <v>76</v>
       </c>
@@ -6131,23 +6248,25 @@
       <c r="K85" s="31">
         <v>1</v>
       </c>
-      <c r="L85" s="79">
-        <f t="shared" ref="L85" si="70">K85*5</f>
+      <c r="L85" s="74">
+        <f t="shared" ref="L85" si="60">K85*5</f>
         <v>5</v>
       </c>
-      <c r="M85" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N85" s="85"/>
+      <c r="M85" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N85" s="80">
+        <v>2.14</v>
+      </c>
       <c r="O85" s="55">
-        <f t="shared" ref="O85" si="71">N85*L85</f>
-        <v>0</v>
+        <f t="shared" ref="O85" si="61">N85*L85</f>
+        <v>10.700000000000001</v>
       </c>
       <c r="P85" s="31"/>
     </row>
-    <row r="86" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A86" s="1"/>
-      <c r="B86" s="66">
+      <c r="B86" s="61">
         <f>ROW(B86) - ROW($B$9)</f>
         <v>77</v>
       </c>
@@ -6178,23 +6297,24 @@
       <c r="K86" s="30">
         <v>1</v>
       </c>
-      <c r="L86" s="78">
+      <c r="L86" s="73">
         <f>K86*5</f>
         <v>5</v>
       </c>
-      <c r="M86" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N86" s="84"/>
-      <c r="O86" s="56">
-        <f>N86*L86</f>
-        <v>0</v>
+      <c r="M86" s="90" t="s">
+        <v>414</v>
+      </c>
+      <c r="N86" s="80" t="s">
+        <v>378</v>
+      </c>
+      <c r="O86" s="55" t="s">
+        <v>378</v>
       </c>
       <c r="P86" s="30"/>
     </row>
     <row r="87" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A87" s="1"/>
-      <c r="B87" s="67">
+      <c r="B87" s="62">
         <f t="shared" si="0"/>
         <v>78</v>
       </c>
@@ -6225,23 +6345,25 @@
       <c r="K87" s="31">
         <v>1</v>
       </c>
-      <c r="L87" s="79">
-        <f t="shared" ref="L87" si="72">K87*5</f>
+      <c r="L87" s="74">
+        <f t="shared" ref="L87" si="62">K87*5</f>
         <v>5</v>
       </c>
-      <c r="M87" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N87" s="85"/>
+      <c r="M87" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N87" s="80">
+        <v>4</v>
+      </c>
       <c r="O87" s="55">
-        <f t="shared" ref="O87" si="73">N87*L87</f>
-        <v>0</v>
+        <f t="shared" ref="O87" si="63">N87*L87</f>
+        <v>20</v>
       </c>
       <c r="P87" s="31"/>
     </row>
     <row r="88" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A88" s="1"/>
-      <c r="B88" s="66">
+      <c r="B88" s="61">
         <f>ROW(B88) - ROW($B$9)</f>
         <v>79</v>
       </c>
@@ -6272,23 +6394,25 @@
       <c r="K88" s="30">
         <v>1</v>
       </c>
-      <c r="L88" s="78">
+      <c r="L88" s="73">
         <f>K88*5</f>
         <v>5</v>
       </c>
-      <c r="M88" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N88" s="84"/>
+      <c r="M88" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="N88" s="79">
+        <v>4.17</v>
+      </c>
       <c r="O88" s="56">
         <f>N88*L88</f>
-        <v>0</v>
+        <v>20.85</v>
       </c>
       <c r="P88" s="30"/>
     </row>
-    <row r="89" spans="1:16" ht="24" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A89" s="1"/>
-      <c r="B89" s="67">
+      <c r="B89" s="62">
         <f t="shared" si="0"/>
         <v>80</v>
       </c>
@@ -6319,23 +6443,24 @@
       <c r="K89" s="31">
         <v>1</v>
       </c>
-      <c r="L89" s="79">
-        <f t="shared" ref="L89" si="74">K89*5</f>
+      <c r="L89" s="74">
+        <f t="shared" ref="L89" si="64">K89*5</f>
         <v>5</v>
       </c>
-      <c r="M89" s="94" t="s">
-        <v>415</v>
-      </c>
-      <c r="N89" s="85"/>
-      <c r="O89" s="55">
-        <f t="shared" ref="O89" si="75">N89*L89</f>
-        <v>0</v>
+      <c r="M89" s="90" t="s">
+        <v>414</v>
+      </c>
+      <c r="N89" s="80" t="s">
+        <v>378</v>
+      </c>
+      <c r="O89" s="55" t="s">
+        <v>378</v>
       </c>
       <c r="P89" s="31"/>
     </row>
-    <row r="90" spans="1:16" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:16" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A90" s="1"/>
-      <c r="B90" s="66">
+      <c r="B90" s="61">
         <f>ROW(B90) - ROW($B$9)</f>
         <v>81</v>
       </c>
@@ -6346,17 +6471,19 @@
         <v>99</v>
       </c>
       <c r="E90" s="30" t="s">
+        <v>408</v>
+      </c>
+      <c r="F90" s="30" t="s">
+        <v>409</v>
+      </c>
+      <c r="G90" s="30" t="s">
         <v>410</v>
       </c>
-      <c r="F90" s="30" t="s">
-        <v>411</v>
-      </c>
-      <c r="G90" s="30" t="s">
+      <c r="H90" s="30" t="s">
+        <v>378</v>
+      </c>
+      <c r="I90" s="30" t="s">
         <v>412</v>
-      </c>
-      <c r="H90" s="30"/>
-      <c r="I90" s="30" t="s">
-        <v>414</v>
       </c>
       <c r="J90" s="30" t="s">
         <v>374</v>
@@ -6364,42 +6491,43 @@
       <c r="K90" s="30">
         <v>1</v>
       </c>
-      <c r="L90" s="78">
+      <c r="L90" s="73">
         <f>K90*5</f>
         <v>5</v>
       </c>
-      <c r="M90" s="95" t="s">
-        <v>415</v>
-      </c>
-      <c r="N90" s="84"/>
-      <c r="O90" s="56">
-        <f>N90*L90</f>
-        <v>0</v>
+      <c r="M90" s="90" t="s">
+        <v>414</v>
+      </c>
+      <c r="N90" s="80" t="s">
+        <v>378</v>
+      </c>
+      <c r="O90" s="55" t="s">
+        <v>378</v>
       </c>
       <c r="P90" s="31"/>
     </row>
     <row r="91" spans="1:16" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A91" s="1"/>
-      <c r="B91" s="70"/>
-      <c r="C91" s="71"/>
-      <c r="D91" s="72"/>
-      <c r="E91" s="73"/>
-      <c r="F91" s="74"/>
-      <c r="G91" s="75"/>
-      <c r="H91" s="75"/>
-      <c r="I91" s="74"/>
-      <c r="J91" s="75"/>
-      <c r="K91" s="75"/>
-      <c r="L91" s="64" t="s">
-        <v>399</v>
-      </c>
-      <c r="M91" s="90"/>
-      <c r="N91" s="65"/>
+      <c r="B91" s="65"/>
+      <c r="C91" s="66"/>
+      <c r="D91" s="67"/>
+      <c r="E91" s="68"/>
+      <c r="F91" s="69"/>
+      <c r="G91" s="70"/>
+      <c r="H91" s="70"/>
+      <c r="I91" s="69"/>
+      <c r="J91" s="70"/>
+      <c r="K91" s="70"/>
+      <c r="L91" s="95" t="s">
+        <v>397</v>
+      </c>
+      <c r="M91" s="96"/>
+      <c r="N91" s="97"/>
       <c r="O91" s="59">
         <f>SUM(O10:O90)</f>
-        <v>32.387500000000003</v>
-      </c>
-      <c r="P91" s="76"/>
+        <v>271.6465</v>
+      </c>
+      <c r="P91" s="71"/>
     </row>
     <row r="92" spans="1:16" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B92" s="24"/>
@@ -6412,16 +6540,16 @@
       <c r="I92" s="9"/>
       <c r="J92" s="9"/>
       <c r="K92" s="9"/>
-      <c r="L92" s="64" t="s">
-        <v>400</v>
-      </c>
-      <c r="M92" s="65"/>
-      <c r="N92" s="65"/>
+      <c r="L92" s="95" t="s">
+        <v>398</v>
+      </c>
+      <c r="M92" s="97"/>
+      <c r="N92" s="97"/>
       <c r="O92" s="60">
         <f>O91/5</f>
-        <v>6.4775000000000009</v>
-      </c>
-      <c r="P92" s="77"/>
+        <v>54.329300000000003</v>
+      </c>
+      <c r="P92" s="72"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -6437,9 +6565,55 @@
     <hyperlink ref="M15" r:id="rId4"/>
     <hyperlink ref="M18" r:id="rId5"/>
     <hyperlink ref="M19" r:id="rId6"/>
+    <hyperlink ref="M20" r:id="rId7"/>
+    <hyperlink ref="M21" r:id="rId8"/>
+    <hyperlink ref="M22" r:id="rId9"/>
+    <hyperlink ref="M23" r:id="rId10"/>
+    <hyperlink ref="M24" r:id="rId11"/>
+    <hyperlink ref="M28" r:id="rId12"/>
+    <hyperlink ref="M30" r:id="rId13"/>
+    <hyperlink ref="M32" r:id="rId14"/>
+    <hyperlink ref="M35" r:id="rId15"/>
+    <hyperlink ref="M39" r:id="rId16"/>
+    <hyperlink ref="M43" r:id="rId17"/>
+    <hyperlink ref="M49" r:id="rId18"/>
+    <hyperlink ref="M50" r:id="rId19"/>
+    <hyperlink ref="M51" r:id="rId20"/>
+    <hyperlink ref="M52" r:id="rId21"/>
+    <hyperlink ref="M53" r:id="rId22"/>
+    <hyperlink ref="M54" r:id="rId23"/>
+    <hyperlink ref="M56" r:id="rId24"/>
+    <hyperlink ref="M57" r:id="rId25"/>
+    <hyperlink ref="M58" r:id="rId26"/>
+    <hyperlink ref="M59" r:id="rId27"/>
+    <hyperlink ref="M60" r:id="rId28"/>
+    <hyperlink ref="M61" r:id="rId29"/>
+    <hyperlink ref="M62" r:id="rId30"/>
+    <hyperlink ref="M63" r:id="rId31"/>
+    <hyperlink ref="M64" r:id="rId32"/>
+    <hyperlink ref="M65" r:id="rId33"/>
+    <hyperlink ref="M66" r:id="rId34"/>
+    <hyperlink ref="M67" r:id="rId35"/>
+    <hyperlink ref="M68" r:id="rId36"/>
+    <hyperlink ref="M69" r:id="rId37"/>
+    <hyperlink ref="M70" r:id="rId38"/>
+    <hyperlink ref="M71" r:id="rId39"/>
+    <hyperlink ref="M73" r:id="rId40"/>
+    <hyperlink ref="M74" r:id="rId41"/>
+    <hyperlink ref="M75" r:id="rId42"/>
+    <hyperlink ref="M77" r:id="rId43"/>
+    <hyperlink ref="M78" r:id="rId44"/>
+    <hyperlink ref="M79" r:id="rId45"/>
+    <hyperlink ref="M80" r:id="rId46"/>
+    <hyperlink ref="M81" r:id="rId47"/>
+    <hyperlink ref="M82" r:id="rId48"/>
+    <hyperlink ref="M83" r:id="rId49"/>
+    <hyperlink ref="M85" r:id="rId50"/>
+    <hyperlink ref="M87" r:id="rId51"/>
+    <hyperlink ref="M88" r:id="rId52"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId7"/>
-  <drawing r:id="rId8"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId53"/>
+  <drawing r:id="rId54"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
#29 Antenna change in BOM.
</commit_message>
<xml_diff>
--- a/Design Files/Baseboard-v2.0/BOM/Client_BOM_Baseboard-v2.0.xlsx
+++ b/Design Files/Baseboard-v2.0/BOM/Client_BOM_Baseboard-v2.0.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="827" uniqueCount="422">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="827" uniqueCount="424">
   <si>
     <t>Component list</t>
   </si>
@@ -1284,7 +1284,13 @@
     <t>peripheral</t>
   </si>
   <si>
-    <t>RF2111027</t>
+    <t>1.8 8dBi Vertical 50W - Antennas ROHS</t>
+  </si>
+  <si>
+    <t>BW2.4JWX195-13KJ</t>
+  </si>
+  <si>
+    <t>BAT WIRELESS</t>
   </si>
 </sst>
 </file>
@@ -2030,6 +2036,15 @@
     <xf numFmtId="0" fontId="24" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2050,15 +2065,6 @@
     <xf numFmtId="0" fontId="22" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2432,13 +2438,13 @@
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
-      <c r="J1" s="95"/>
-      <c r="K1" s="95"/>
-      <c r="L1" s="95"/>
-      <c r="M1" s="95"/>
-      <c r="N1" s="95"/>
-      <c r="O1" s="95"/>
-      <c r="P1" s="95"/>
+      <c r="J1" s="98"/>
+      <c r="K1" s="98"/>
+      <c r="L1" s="98"/>
+      <c r="M1" s="98"/>
+      <c r="N1" s="98"/>
+      <c r="O1" s="98"/>
+      <c r="P1" s="98"/>
     </row>
     <row r="2" spans="1:16" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -2482,7 +2488,7 @@
       <c r="M3" s="4"/>
       <c r="N3" s="4"/>
       <c r="O3" s="4"/>
-      <c r="P3" s="96"/>
+      <c r="P3" s="99"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -2504,7 +2510,7 @@
       <c r="M4" s="5"/>
       <c r="N4" s="5"/>
       <c r="O4" s="5"/>
-      <c r="P4" s="97"/>
+      <c r="P4" s="100"/>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -2526,7 +2532,7 @@
       <c r="M5" s="5"/>
       <c r="N5" s="5"/>
       <c r="O5" s="5"/>
-      <c r="P5" s="97"/>
+      <c r="P5" s="100"/>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -2544,7 +2550,7 @@
       <c r="M6" s="5"/>
       <c r="N6" s="5"/>
       <c r="O6" s="5"/>
-      <c r="P6" s="97"/>
+      <c r="P6" s="100"/>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -2562,7 +2568,7 @@
       <c r="M7" s="7"/>
       <c r="N7" s="7"/>
       <c r="O7" s="7"/>
-      <c r="P7" s="97"/>
+      <c r="P7" s="100"/>
     </row>
     <row r="8" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -2580,7 +2586,7 @@
       <c r="M8" s="7"/>
       <c r="N8" s="7"/>
       <c r="O8" s="7"/>
-      <c r="P8" s="97"/>
+      <c r="P8" s="100"/>
     </row>
     <row r="9" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -22976,31 +22982,31 @@
       <c r="C92" s="43" t="s">
         <v>420</v>
       </c>
-      <c r="D92" s="30" t="s">
+      <c r="D92" s="51" t="s">
         <v>373</v>
       </c>
-      <c r="E92" s="30" t="s">
+      <c r="E92" s="51" t="s">
+        <v>421</v>
+      </c>
+      <c r="F92" s="51" t="s">
         <v>373</v>
       </c>
-      <c r="F92" s="30" t="s">
+      <c r="G92" s="51" t="s">
+        <v>422</v>
+      </c>
+      <c r="H92" s="95" t="s">
         <v>373</v>
       </c>
-      <c r="G92" s="30" t="s">
-        <v>421</v>
-      </c>
-      <c r="H92" s="101" t="s">
-        <v>373</v>
-      </c>
-      <c r="I92" s="30" t="s">
-        <v>312</v>
+      <c r="I92" s="51" t="s">
+        <v>423</v>
       </c>
       <c r="J92" s="30" t="s">
         <v>373</v>
       </c>
-      <c r="K92" s="101">
+      <c r="K92" s="95">
         <v>1</v>
       </c>
-      <c r="L92" s="102">
+      <c r="L92" s="96">
         <f>K92*5</f>
         <v>5</v>
       </c>
@@ -23013,7 +23019,7 @@
       <c r="O92" s="55" t="s">
         <v>373</v>
       </c>
-      <c r="P92" s="103"/>
+      <c r="P92" s="97"/>
     </row>
     <row r="93" spans="1:16" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A93" s="1"/>
@@ -23027,11 +23033,11 @@
       <c r="I93" s="69"/>
       <c r="J93" s="70"/>
       <c r="K93" s="70"/>
-      <c r="L93" s="98" t="s">
+      <c r="L93" s="101" t="s">
         <v>391</v>
       </c>
-      <c r="M93" s="99"/>
-      <c r="N93" s="100"/>
+      <c r="M93" s="102"/>
+      <c r="N93" s="103"/>
       <c r="O93" s="59">
         <f>SUM(O10:O91)</f>
         <v>262.72650000000004</v>
@@ -23049,11 +23055,11 @@
       <c r="I94" s="9"/>
       <c r="J94" s="9"/>
       <c r="K94" s="9"/>
-      <c r="L94" s="98" t="s">
+      <c r="L94" s="101" t="s">
         <v>392</v>
       </c>
-      <c r="M94" s="100"/>
-      <c r="N94" s="100"/>
+      <c r="M94" s="103"/>
+      <c r="N94" s="103"/>
       <c r="O94" s="60">
         <f>O93/5</f>
         <v>52.545300000000012</v>

</xml_diff>

<commit_message>
#29 Client BOM Updated.
</commit_message>
<xml_diff>
--- a/Design Files/Baseboard-v2.0/BOM/Client_BOM_Baseboard-v2.0.xlsx
+++ b/Design Files/Baseboard-v2.0/BOM/Client_BOM_Baseboard-v2.0.xlsx
@@ -408,9 +408,6 @@
     <t>1x6P SH 1 1mm 6 SMD,P=1mm Wire To Board / Wire To Wire Connector ROHS</t>
   </si>
   <si>
-    <t>1 Inner bore SMA Board Edge Bend -55℃~+155℃ 50Ω Plugin RF Connectors / Coaxial Connectors ROHS</t>
-  </si>
-  <si>
     <t>0.8mm mPCI-E Surface Mount 52 SMD,P=0.8mm Card Edge Connectors ROHS</t>
   </si>
   <si>
@@ -765,9 +762,6 @@
     <t>C145963</t>
   </si>
   <si>
-    <t>HJ-SMA508</t>
-  </si>
-  <si>
     <t>SDCL1608C2N0STDF</t>
   </si>
   <si>
@@ -1146,9 +1140,6 @@
     <t>Custom</t>
   </si>
   <si>
-    <t>UFL Connector</t>
-  </si>
-  <si>
     <t>Relay</t>
   </si>
   <si>
@@ -1291,6 +1282,15 @@
   </si>
   <si>
     <t>BAT WIRELESS</t>
+  </si>
+  <si>
+    <t>SMA Connector</t>
+  </si>
+  <si>
+    <t>1 Inner bore SMA Board Edge Bend 11mm 5.35mm Plugin RF Connectors / Coaxial Connectors ROHS</t>
+  </si>
+  <si>
+    <t>HJ-SMA175</t>
   </si>
 </sst>
 </file>
@@ -2455,7 +2455,7 @@
       </c>
       <c r="E2" s="10"/>
       <c r="F2" s="39" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="G2" s="11"/>
       <c r="H2" s="11"/>
@@ -2477,7 +2477,7 @@
       </c>
       <c r="E3" s="12"/>
       <c r="F3" s="40" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="G3" s="12"/>
       <c r="H3" s="12"/>
@@ -2499,7 +2499,7 @@
       </c>
       <c r="E4" s="12"/>
       <c r="F4" s="41" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="G4" s="13"/>
       <c r="H4" s="13"/>
@@ -2603,37 +2603,37 @@
         <v>99</v>
       </c>
       <c r="F9" s="29" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="G9" s="29" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="H9" s="29" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
       <c r="I9" s="29" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="J9" s="29" t="s">
+        <v>382</v>
+      </c>
+      <c r="K9" s="29" t="s">
+        <v>368</v>
+      </c>
+      <c r="L9" s="85" t="s">
+        <v>383</v>
+      </c>
+      <c r="M9" s="29" t="s">
+        <v>384</v>
+      </c>
+      <c r="N9" s="86" t="s">
         <v>385</v>
       </c>
-      <c r="K9" s="29" t="s">
-        <v>370</v>
-      </c>
-      <c r="L9" s="85" t="s">
+      <c r="O9" s="29" t="s">
         <v>386</v>
       </c>
-      <c r="M9" s="29" t="s">
+      <c r="P9" s="29" t="s">
         <v>387</v>
-      </c>
-      <c r="N9" s="86" t="s">
-        <v>388</v>
-      </c>
-      <c r="O9" s="29" t="s">
-        <v>389</v>
-      </c>
-      <c r="P9" s="29" t="s">
-        <v>390</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
@@ -2643,28 +2643,28 @@
         <v>1</v>
       </c>
       <c r="C10" s="43" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="D10" s="44" t="s">
         <v>24</v>
       </c>
       <c r="E10" s="44" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="F10" s="44" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="G10" s="44" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="H10" s="52" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I10" s="52" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="J10" s="44" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="K10" s="44">
         <v>1</v>
@@ -2674,13 +2674,13 @@
         <v>5</v>
       </c>
       <c r="M10" s="44" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="N10" s="87" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="O10" s="52" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="P10" s="30"/>
     </row>
@@ -2700,19 +2700,19 @@
         <v>100</v>
       </c>
       <c r="F11" s="31" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G11" s="31" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H11" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I11" s="31" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="J11" s="31" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="K11" s="31">
         <v>1</v>
@@ -2722,7 +2722,7 @@
         <v>5</v>
       </c>
       <c r="M11" s="54" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N11" s="80">
         <v>0.48</v>
@@ -2749,19 +2749,19 @@
         <v>101</v>
       </c>
       <c r="F12" s="30" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="G12" s="30" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="H12" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I12" s="30" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="J12" s="30" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="K12" s="30">
         <v>25</v>
@@ -2771,7 +2771,7 @@
         <v>125</v>
       </c>
       <c r="M12" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N12" s="79">
         <v>1.03E-2</v>
@@ -2798,19 +2798,19 @@
         <v>102</v>
       </c>
       <c r="F13" s="31" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="G13" s="31" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="H13" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I13" s="31" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="J13" s="31" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="K13" s="31">
         <v>3</v>
@@ -2820,7 +2820,7 @@
         <v>15</v>
       </c>
       <c r="M13" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N13" s="80">
         <v>1.6E-2</v>
@@ -2847,19 +2847,19 @@
         <v>103</v>
       </c>
       <c r="F14" s="30" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="G14" s="30" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="H14" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I14" s="30" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="J14" s="30" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="K14" s="30">
         <v>3</v>
@@ -2869,13 +2869,13 @@
         <v>15</v>
       </c>
       <c r="M14" s="90" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="N14" s="79" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="O14" s="56" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="P14" s="30"/>
     </row>
@@ -2895,19 +2895,19 @@
         <v>104</v>
       </c>
       <c r="F15" s="31" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G15" s="31" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="H15" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I15" s="31" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="J15" s="31" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="K15" s="31">
         <v>2</v>
@@ -2917,7 +2917,7 @@
         <v>10</v>
       </c>
       <c r="M15" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N15" s="80">
         <v>0.72599999999999998</v>
@@ -2944,19 +2944,19 @@
         <v>105</v>
       </c>
       <c r="F16" s="30" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="G16" s="30" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="H16" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I16" s="30" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="J16" s="30" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="K16" s="30">
         <v>1</v>
@@ -2966,13 +2966,13 @@
         <v>5</v>
       </c>
       <c r="M16" s="90" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="N16" s="79" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="O16" s="56" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="P16" s="30"/>
     </row>
@@ -2992,19 +2992,19 @@
         <v>106</v>
       </c>
       <c r="F17" s="31" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="G17" s="31" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="H17" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I17" s="31" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="J17" s="31" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="K17" s="31">
         <v>1</v>
@@ -3014,13 +3014,13 @@
         <v>5</v>
       </c>
       <c r="M17" s="90" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="N17" s="80" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="O17" s="55" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="P17" s="31"/>
     </row>
@@ -3040,19 +3040,19 @@
         <v>107</v>
       </c>
       <c r="F18" s="30" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="G18" s="30" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="H18" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I18" s="30" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="J18" s="30" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="K18" s="30">
         <v>1</v>
@@ -3062,7 +3062,7 @@
         <v>5</v>
       </c>
       <c r="M18" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N18" s="79">
         <v>3.42</v>
@@ -3089,19 +3089,19 @@
         <v>108</v>
       </c>
       <c r="F19" s="31" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G19" s="31" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="H19" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I19" s="31" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="J19" s="31" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="K19" s="31">
         <v>1</v>
@@ -3111,7 +3111,7 @@
         <v>5</v>
       </c>
       <c r="M19" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N19" s="80">
         <v>0.68</v>
@@ -3138,19 +3138,19 @@
         <v>109</v>
       </c>
       <c r="F20" s="30" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="G20" s="44" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H20" s="30" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
       <c r="I20" s="30" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="J20" s="30" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="K20" s="30">
         <v>4</v>
@@ -3160,7 +3160,7 @@
         <v>20</v>
       </c>
       <c r="M20" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N20" s="79">
         <v>6.2E-2</v>
@@ -3187,19 +3187,19 @@
         <v>110</v>
       </c>
       <c r="F21" s="31" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="G21" s="31" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="H21" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I21" s="31" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="J21" s="31" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="K21" s="31">
         <v>2</v>
@@ -3209,7 +3209,7 @@
         <v>10</v>
       </c>
       <c r="M21" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N21" s="80">
         <v>0.121</v>
@@ -3236,19 +3236,19 @@
         <v>111</v>
       </c>
       <c r="F22" s="30" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="G22" s="30" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="H22" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I22" s="30" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="J22" s="30" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="K22" s="30">
         <v>2</v>
@@ -3258,7 +3258,7 @@
         <v>10</v>
       </c>
       <c r="M22" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N22" s="79">
         <v>1.9E-2</v>
@@ -3285,19 +3285,19 @@
         <v>112</v>
       </c>
       <c r="F23" s="31" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G23" s="31" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="H23" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I23" s="31" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="J23" s="31" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="K23" s="31">
         <v>3</v>
@@ -3307,7 +3307,7 @@
         <v>15</v>
       </c>
       <c r="M23" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N23" s="80">
         <v>7.3999999999999996E-2</v>
@@ -3334,19 +3334,19 @@
         <v>113</v>
       </c>
       <c r="F24" s="30" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G24" s="30" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="H24" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I24" s="30" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="J24" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="K24" s="30">
         <v>1</v>
@@ -3356,7 +3356,7 @@
         <v>5</v>
       </c>
       <c r="M24" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N24" s="79">
         <v>0.44</v>
@@ -3383,19 +3383,19 @@
         <v>114</v>
       </c>
       <c r="F25" s="31" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="G25" s="31" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="H25" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I25" s="31" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="J25" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="K25" s="31">
         <v>1</v>
@@ -3405,11 +3405,11 @@
         <v>5</v>
       </c>
       <c r="M25" s="90" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="N25" s="80"/>
       <c r="O25" s="55" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="P25" s="31"/>
     </row>
@@ -3429,19 +3429,19 @@
         <v>115</v>
       </c>
       <c r="F26" s="30" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="G26" s="30" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="H26" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I26" s="30" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="J26" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="K26" s="30">
         <v>1</v>
@@ -3451,11 +3451,11 @@
         <v>5</v>
       </c>
       <c r="M26" s="90" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="N26" s="79"/>
       <c r="O26" s="56" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="P26" s="30"/>
     </row>
@@ -3475,19 +3475,19 @@
         <v>116</v>
       </c>
       <c r="F27" s="31" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="G27" s="31" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H27" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I27" s="31" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="J27" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="K27" s="31">
         <v>1</v>
@@ -3497,11 +3497,11 @@
         <v>5</v>
       </c>
       <c r="M27" s="90" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="N27" s="80"/>
       <c r="O27" s="55" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="P27" s="31"/>
     </row>
@@ -3521,19 +3521,19 @@
         <v>117</v>
       </c>
       <c r="F28" s="30" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="G28" s="30" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="H28" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I28" s="30" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="J28" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="K28" s="30">
         <v>3</v>
@@ -3543,7 +3543,7 @@
         <v>15</v>
       </c>
       <c r="M28" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N28" s="79">
         <v>0.184</v>
@@ -3570,19 +3570,19 @@
         <v>118</v>
       </c>
       <c r="F29" s="31" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="G29" s="31" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="H29" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I29" s="31" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="J29" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="K29" s="31">
         <v>2</v>
@@ -3592,11 +3592,11 @@
         <v>10</v>
       </c>
       <c r="M29" s="90" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="N29" s="80"/>
       <c r="O29" s="55" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="P29" s="31"/>
     </row>
@@ -3616,19 +3616,19 @@
         <v>119</v>
       </c>
       <c r="F30" s="30" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="G30" s="30" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="H30" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I30" s="30" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="J30" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="K30" s="30">
         <v>4</v>
@@ -3638,7 +3638,7 @@
         <v>20</v>
       </c>
       <c r="M30" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N30" s="79">
         <v>0.32300000000000001</v>
@@ -3665,19 +3665,19 @@
         <v>120</v>
       </c>
       <c r="F31" s="31" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="G31" s="31" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="H31" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I31" s="31" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="J31" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="K31" s="31">
         <v>4</v>
@@ -3687,11 +3687,11 @@
         <v>20</v>
       </c>
       <c r="M31" s="90" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="N31" s="80"/>
       <c r="O31" s="55" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="P31" s="31"/>
     </row>
@@ -3711,19 +3711,19 @@
         <v>121</v>
       </c>
       <c r="F32" s="30" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G32" s="30" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="H32" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I32" s="30" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="J32" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="K32" s="30">
         <v>1</v>
@@ -3733,7 +3733,7 @@
         <v>5</v>
       </c>
       <c r="M32" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N32" s="79">
         <v>1.766</v>
@@ -3760,19 +3760,19 @@
         <v>122</v>
       </c>
       <c r="F33" s="31" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="G33" s="31" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="H33" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I33" s="31" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="J33" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="K33" s="31">
         <v>1</v>
@@ -3782,11 +3782,11 @@
         <v>5</v>
       </c>
       <c r="M33" s="90" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="N33" s="80"/>
       <c r="O33" s="55" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="P33" s="31"/>
     </row>
@@ -3806,19 +3806,19 @@
         <v>123</v>
       </c>
       <c r="F34" s="30" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="G34" s="30" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="H34" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I34" s="30" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="J34" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="K34" s="30">
         <v>4</v>
@@ -3828,11 +3828,11 @@
         <v>20</v>
       </c>
       <c r="M34" s="90" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="N34" s="79"/>
       <c r="O34" s="56" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="P34" s="30"/>
     </row>
@@ -3852,19 +3852,19 @@
         <v>124</v>
       </c>
       <c r="F35" s="31" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="G35" s="31" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="H35" s="53" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="I35" s="31" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="J35" s="31" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="K35" s="31">
         <v>1</v>
@@ -3874,7 +3874,7 @@
         <v>5</v>
       </c>
       <c r="M35" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N35" s="80">
         <v>0.28000000000000003</v>
@@ -3901,19 +3901,19 @@
         <v>125</v>
       </c>
       <c r="F36" s="31" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="G36" s="30" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="H36" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I36" s="30" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="J36" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="K36" s="30">
         <v>8</v>
@@ -3923,13 +3923,13 @@
         <v>40</v>
       </c>
       <c r="M36" s="90" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="N36" s="79" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="O36" s="56" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="P36" s="30"/>
     </row>
@@ -3949,19 +3949,19 @@
         <v>126</v>
       </c>
       <c r="F37" s="31" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="G37" s="31" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="H37" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I37" s="31" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="J37" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="K37" s="31">
         <v>1</v>
@@ -3971,13 +3971,13 @@
         <v>5</v>
       </c>
       <c r="M37" s="90" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="N37" s="80" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="O37" s="55" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="P37" s="31"/>
     </row>
@@ -3997,19 +3997,19 @@
         <v>127</v>
       </c>
       <c r="F38" s="31" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="G38" s="30" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="H38" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I38" s="30" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="J38" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="K38" s="30">
         <v>4</v>
@@ -4019,13 +4019,13 @@
         <v>20</v>
       </c>
       <c r="M38" s="90" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="N38" s="79" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="O38" s="56" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="P38" s="30"/>
     </row>
@@ -4036,28 +4036,28 @@
         <v>30</v>
       </c>
       <c r="C39" s="45" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="D39" s="92" t="s">
         <v>53</v>
       </c>
       <c r="E39" s="31" t="s">
-        <v>412</v>
+        <v>409</v>
       </c>
       <c r="F39" s="31" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="G39" s="31" t="s">
-        <v>413</v>
+        <v>410</v>
       </c>
       <c r="H39" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I39" s="31" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
       <c r="J39" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="K39" s="31">
         <v>1</v>
@@ -4067,13 +4067,13 @@
         <v>5</v>
       </c>
       <c r="M39" s="90" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="N39" s="79" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="O39" s="56" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="P39" s="31"/>
     </row>
@@ -4093,19 +4093,19 @@
         <v>128</v>
       </c>
       <c r="F40" s="31" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="G40" s="30" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="H40" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I40" s="30" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="J40" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="K40" s="30">
         <v>1</v>
@@ -4115,43 +4115,43 @@
         <v>5</v>
       </c>
       <c r="M40" s="90" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="N40" s="79" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="O40" s="56" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="P40" s="30"/>
     </row>
-    <row r="41" spans="1:16" ht="48" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:16" ht="36" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
       <c r="B41" s="62">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
       <c r="C41" s="45" t="s">
-        <v>375</v>
+        <v>421</v>
       </c>
       <c r="D41" s="31" t="s">
         <v>55</v>
       </c>
       <c r="E41" s="31" t="s">
-        <v>129</v>
+        <v>422</v>
       </c>
       <c r="F41" s="31" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="G41" s="31" t="s">
-        <v>248</v>
+        <v>423</v>
       </c>
       <c r="H41" s="31"/>
       <c r="I41" s="31" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="J41" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="K41" s="31">
         <v>1</v>
@@ -4161,13 +4161,13 @@
         <v>5</v>
       </c>
       <c r="M41" s="90" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="N41" s="80" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="O41" s="55" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="P41" s="31"/>
     </row>
@@ -4184,22 +4184,22 @@
         <v>56</v>
       </c>
       <c r="E42" s="30" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F42" s="31" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="G42" s="30" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="H42" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I42" s="30" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="J42" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="K42" s="30">
         <v>2</v>
@@ -4209,13 +4209,13 @@
         <v>10</v>
       </c>
       <c r="M42" s="90" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="N42" s="79" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="O42" s="56" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="P42" s="30"/>
     </row>
@@ -4226,28 +4226,28 @@
         <v>34</v>
       </c>
       <c r="C43" s="45" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="D43" s="31" t="s">
         <v>57</v>
       </c>
       <c r="E43" s="31" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
       <c r="F43" s="31" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="G43" s="31" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
       <c r="H43" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I43" s="31" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
       <c r="J43" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="K43" s="31">
         <v>3</v>
@@ -4257,7 +4257,7 @@
         <v>15</v>
       </c>
       <c r="M43" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N43" s="80">
         <v>0.90900000000000003</v>
@@ -4281,22 +4281,22 @@
         <v>58</v>
       </c>
       <c r="E44" s="30" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F44" s="31" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="G44" s="30" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="H44" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I44" s="30" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="J44" s="30" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="K44" s="30">
         <v>1</v>
@@ -4306,13 +4306,13 @@
         <v>5</v>
       </c>
       <c r="M44" s="90" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="N44" s="79" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="O44" s="56" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="P44" s="30"/>
     </row>
@@ -4329,22 +4329,22 @@
         <v>59</v>
       </c>
       <c r="E45" s="31" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F45" s="31" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="G45" s="31" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="H45" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I45" s="31" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="J45" s="31" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="K45" s="31">
         <v>1</v>
@@ -4354,13 +4354,13 @@
         <v>5</v>
       </c>
       <c r="M45" s="90" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="N45" s="80" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="O45" s="55" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="P45" s="31"/>
     </row>
@@ -4377,22 +4377,22 @@
         <v>60</v>
       </c>
       <c r="E46" s="30" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F46" s="30" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G46" s="30" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="H46" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I46" s="30" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="J46" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="K46" s="30">
         <v>2</v>
@@ -4402,13 +4402,13 @@
         <v>10</v>
       </c>
       <c r="M46" s="90" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="N46" s="79" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="O46" s="79" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="P46" s="30"/>
     </row>
@@ -4425,22 +4425,22 @@
         <v>61</v>
       </c>
       <c r="E47" s="31" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F47" s="31" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G47" s="31" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="H47" s="53" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="I47" s="31" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="J47" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="K47" s="31">
         <v>1</v>
@@ -4450,13 +4450,13 @@
         <v>5</v>
       </c>
       <c r="M47" s="90" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="N47" s="80" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="O47" s="80" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="P47" s="31"/>
     </row>
@@ -4467,28 +4467,28 @@
         <v>39</v>
       </c>
       <c r="C48" s="43" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="D48" s="44" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
       <c r="E48" s="44" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F48" s="44" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="G48" s="44" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="H48" s="44" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I48" s="44" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="J48" s="44" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="K48" s="44">
         <v>10</v>
@@ -4498,13 +4498,13 @@
         <v>50</v>
       </c>
       <c r="M48" s="88" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="N48" s="81" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="O48" s="44" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="P48" s="30"/>
     </row>
@@ -4515,28 +4515,28 @@
         <v>40</v>
       </c>
       <c r="C49" s="45" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
       <c r="D49" s="31" t="s">
         <v>62</v>
       </c>
       <c r="E49" s="31" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F49" s="31" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="G49" s="31" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="H49" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I49" s="31" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="J49" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="K49" s="31">
         <v>1</v>
@@ -4546,7 +4546,7 @@
         <v>5</v>
       </c>
       <c r="M49" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N49" s="80">
         <v>0.14000000000000001</v>
@@ -4570,22 +4570,22 @@
         <v>63</v>
       </c>
       <c r="E50" s="30" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F50" s="30" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="G50" s="44" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="H50" s="30" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
       <c r="I50" s="30" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="J50" s="30" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="K50" s="30">
         <v>2</v>
@@ -4595,7 +4595,7 @@
         <v>10</v>
       </c>
       <c r="M50" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N50" s="79">
         <v>0.33600000000000002</v>
@@ -4619,22 +4619,22 @@
         <v>64</v>
       </c>
       <c r="E51" s="31" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F51" s="31" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="G51" s="31" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="H51" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I51" s="31" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="J51" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="K51" s="31">
         <v>1</v>
@@ -4644,16 +4644,16 @@
         <v>5</v>
       </c>
       <c r="M51" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N51" s="80" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="O51" s="55" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="P51" s="94" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
     </row>
     <row r="52" spans="1:16384" x14ac:dyDescent="0.25">
@@ -4669,22 +4669,22 @@
         <v>65</v>
       </c>
       <c r="E52" s="30" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F52" s="30" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="G52" s="30" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="H52" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I52" s="30" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="J52" s="30" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="K52" s="30">
         <v>1</v>
@@ -4694,7 +4694,7 @@
         <v>5</v>
       </c>
       <c r="M52" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N52" s="79">
         <v>0.1</v>
@@ -4715,25 +4715,25 @@
         <v>17</v>
       </c>
       <c r="D53" s="31" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
       <c r="E53" s="31" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F53" s="31" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="G53" s="31" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="H53" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I53" s="31" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="J53" s="31" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="K53" s="31">
         <v>12</v>
@@ -4743,7 +4743,7 @@
         <v>60</v>
       </c>
       <c r="M53" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N53" s="80">
         <v>1.6199999999999999E-2</v>
@@ -4764,25 +4764,25 @@
         <v>17</v>
       </c>
       <c r="D54" s="91" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="E54" s="30" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F54" s="30" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="G54" s="44" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="H54" s="30" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
       <c r="I54" s="30" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="J54" s="30" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="K54" s="30">
         <v>8</v>
@@ -4792,7 +4792,7 @@
         <v>40</v>
       </c>
       <c r="M54" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N54" s="79">
         <v>2.5999999999999999E-2</v>
@@ -4816,22 +4816,22 @@
         <v>66</v>
       </c>
       <c r="E55" s="31" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="F55" s="31" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="G55" s="31" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="H55" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I55" s="31" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="J55" s="31" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="K55" s="31">
         <v>1</v>
@@ -4841,13 +4841,13 @@
         <v>5</v>
       </c>
       <c r="M55" s="90" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="N55" s="80" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="O55" s="55" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="P55" s="31"/>
     </row>
@@ -4864,22 +4864,22 @@
         <v>67</v>
       </c>
       <c r="E56" s="30" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F56" s="30" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="G56" s="30" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="H56" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I56" s="30" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="J56" s="30" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="K56" s="30">
         <v>2</v>
@@ -4889,7 +4889,7 @@
         <v>10</v>
       </c>
       <c r="M56" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N56" s="79">
         <v>0.02</v>
@@ -4910,25 +4910,25 @@
         <v>17</v>
       </c>
       <c r="D57" s="31" t="s">
-        <v>396</v>
+        <v>393</v>
       </c>
       <c r="E57" s="31" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F57" s="31" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="G57" s="91" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="H57" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I57" s="31" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="J57" s="31" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="K57" s="31">
         <v>2</v>
@@ -4938,7 +4938,7 @@
         <v>10</v>
       </c>
       <c r="M57" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N57" s="80">
         <v>0.02</v>
@@ -4962,22 +4962,22 @@
         <v>68</v>
       </c>
       <c r="E58" s="30" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F58" s="30" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="G58" s="30" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="H58" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I58" s="30" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="J58" s="30" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="K58" s="30">
         <v>2</v>
@@ -4987,7 +4987,7 @@
         <v>10</v>
       </c>
       <c r="M58" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N58" s="79">
         <v>1.4E-2</v>
@@ -5011,22 +5011,22 @@
         <v>69</v>
       </c>
       <c r="E59" s="31" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F59" s="31" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="G59" s="31" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="H59" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I59" s="31" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="J59" s="31" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="K59" s="31">
         <v>22</v>
@@ -5036,7 +5036,7 @@
         <v>110</v>
       </c>
       <c r="M59" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N59" s="80">
         <v>7.0000000000000001E-3</v>
@@ -5060,22 +5060,22 @@
         <v>70</v>
       </c>
       <c r="E60" s="30" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="F60" s="30" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="G60" s="30" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="H60" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I60" s="30" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="J60" s="30" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="K60" s="30">
         <v>1</v>
@@ -5085,7 +5085,7 @@
         <v>5</v>
       </c>
       <c r="M60" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N60" s="79">
         <v>0.1</v>
@@ -5106,25 +5106,25 @@
         <v>17</v>
       </c>
       <c r="D61" s="31" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="E61" s="30" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F61" s="30" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="G61" s="30" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="H61" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I61" s="30" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="J61" s="30" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="K61" s="30">
         <v>11</v>
@@ -5134,7 +5134,7 @@
         <v>55</v>
       </c>
       <c r="M61" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N61" s="79">
         <v>6.4000000000000003E-3</v>
@@ -5152,28 +5152,28 @@
         <v>53</v>
       </c>
       <c r="C62" s="45" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
       <c r="D62" s="91" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="E62" s="30" t="s">
-        <v>417</v>
+        <v>414</v>
       </c>
       <c r="F62" s="30" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="G62" s="30" t="s">
-        <v>418</v>
+        <v>415</v>
       </c>
       <c r="H62" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I62" s="30" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="J62" s="30" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="K62" s="30">
         <v>3</v>
@@ -5183,7 +5183,7 @@
         <v>15</v>
       </c>
       <c r="M62" s="93" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N62" s="79">
         <v>0.1</v>
@@ -21575,22 +21575,22 @@
         <v>71</v>
       </c>
       <c r="E63" s="30" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F63" s="30" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="G63" s="30" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="H63" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I63" s="30" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="J63" s="30" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="K63" s="30">
         <v>4</v>
@@ -21600,7 +21600,7 @@
         <v>20</v>
       </c>
       <c r="M63" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N63" s="79">
         <v>1.4E-2</v>
@@ -21624,22 +21624,22 @@
         <v>72</v>
       </c>
       <c r="E64" s="31" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F64" s="31" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="G64" s="31" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="H64" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I64" s="31" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="J64" s="31" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="K64" s="31">
         <v>1</v>
@@ -21649,7 +21649,7 @@
         <v>5</v>
       </c>
       <c r="M64" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N64" s="80">
         <v>0.1</v>
@@ -21673,22 +21673,22 @@
         <v>73</v>
       </c>
       <c r="E65" s="30" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="F65" s="30" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="G65" s="30" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="H65" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I65" s="30" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="J65" s="30" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="K65" s="30">
         <v>1</v>
@@ -21698,7 +21698,7 @@
         <v>5</v>
       </c>
       <c r="M65" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N65" s="79">
         <v>0.1</v>
@@ -21722,22 +21722,22 @@
         <v>74</v>
       </c>
       <c r="E66" s="31" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="F66" s="31" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="G66" s="31" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="H66" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I66" s="31" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="J66" s="31" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="K66" s="31">
         <v>1</v>
@@ -21747,7 +21747,7 @@
         <v>5</v>
       </c>
       <c r="M66" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N66" s="80">
         <v>0.34</v>
@@ -21771,22 +21771,22 @@
         <v>75</v>
       </c>
       <c r="E67" s="31" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="F67" s="31" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="G67" s="91" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="H67" s="31" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
       <c r="I67" s="31" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="J67" s="31" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="K67" s="31">
         <v>4</v>
@@ -21796,7 +21796,7 @@
         <v>20</v>
       </c>
       <c r="M67" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N67" s="80">
         <v>0.11600000000000001</v>
@@ -21820,22 +21820,22 @@
         <v>76</v>
       </c>
       <c r="E68" s="30" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F68" s="30" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="G68" s="30" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="H68" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I68" s="30" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="J68" s="30" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="K68" s="30">
         <v>1</v>
@@ -21845,7 +21845,7 @@
         <v>5</v>
       </c>
       <c r="M68" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N68" s="79">
         <v>0.1</v>
@@ -21869,22 +21869,22 @@
         <v>77</v>
       </c>
       <c r="E69" s="31" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F69" s="31" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="G69" s="31" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="H69" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I69" s="31" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="J69" s="31" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="K69" s="31">
         <v>1</v>
@@ -21894,7 +21894,7 @@
         <v>5</v>
       </c>
       <c r="M69" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N69" s="80">
         <v>0.41</v>
@@ -21918,22 +21918,22 @@
         <v>78</v>
       </c>
       <c r="E70" s="30" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F70" s="30" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="G70" s="30" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="H70" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I70" s="30" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="J70" s="30" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="K70" s="30">
         <v>2</v>
@@ -21943,7 +21943,7 @@
         <v>10</v>
       </c>
       <c r="M70" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N70" s="79">
         <v>1.7999999999999999E-2</v>
@@ -21967,22 +21967,22 @@
         <v>79</v>
       </c>
       <c r="E71" s="31" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="F71" s="31" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="G71" s="31" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="H71" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I71" s="31" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="J71" s="31" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="K71" s="31">
         <v>1</v>
@@ -21992,7 +21992,7 @@
         <v>5</v>
       </c>
       <c r="M71" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N71" s="80">
         <v>0.1</v>
@@ -22010,28 +22010,28 @@
         <v>63</v>
       </c>
       <c r="C72" s="45" t="s">
+        <v>395</v>
+      </c>
+      <c r="D72" s="31" t="s">
+        <v>396</v>
+      </c>
+      <c r="E72" s="31" t="s">
+        <v>397</v>
+      </c>
+      <c r="F72" s="31" t="s">
+        <v>372</v>
+      </c>
+      <c r="G72" s="31" t="s">
         <v>398</v>
       </c>
-      <c r="D72" s="31" t="s">
-        <v>399</v>
-      </c>
-      <c r="E72" s="31" t="s">
-        <v>400</v>
-      </c>
-      <c r="F72" s="31" t="s">
-        <v>374</v>
-      </c>
-      <c r="G72" s="31" t="s">
-        <v>401</v>
-      </c>
       <c r="H72" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I72" s="31" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="J72" s="31" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="K72" s="31">
         <v>5</v>
@@ -22041,7 +22041,7 @@
         <v>25</v>
       </c>
       <c r="M72" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N72" s="80">
         <v>8.9599999999999999E-2</v>
@@ -22065,22 +22065,22 @@
         <v>80</v>
       </c>
       <c r="E73" s="46" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="F73" s="47" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="G73" s="46" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="H73" s="46" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I73" s="46" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="J73" s="46" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="K73" s="46">
         <v>2</v>
@@ -22090,13 +22090,13 @@
         <v>10</v>
       </c>
       <c r="M73" s="88" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="N73" s="82" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="O73" s="46" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="P73" s="30"/>
     </row>
@@ -22113,22 +22113,22 @@
         <v>81</v>
       </c>
       <c r="E74" s="31" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="F74" s="31" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="G74" s="31" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="H74" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I74" s="31" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="J74" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="K74" s="31">
         <v>1</v>
@@ -22138,7 +22138,7 @@
         <v>5</v>
       </c>
       <c r="M74" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N74" s="80">
         <v>0.14000000000000001</v>
@@ -22162,22 +22162,22 @@
         <v>82</v>
       </c>
       <c r="E75" s="30" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F75" s="30" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="G75" s="30" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="H75" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I75" s="30" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="J75" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="K75" s="30">
         <v>1</v>
@@ -22187,7 +22187,7 @@
         <v>5</v>
       </c>
       <c r="M75" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N75" s="79">
         <v>5.28</v>
@@ -22211,22 +22211,22 @@
         <v>83</v>
       </c>
       <c r="E76" s="31" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F76" s="31" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="G76" s="31" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="H76" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I76" s="31" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="J76" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="K76" s="31">
         <v>1</v>
@@ -22236,7 +22236,7 @@
         <v>5</v>
       </c>
       <c r="M76" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N76" s="80">
         <v>0.88</v>
@@ -22260,22 +22260,22 @@
         <v>84</v>
       </c>
       <c r="E77" s="30" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F77" s="30" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="G77" s="30" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="H77" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I77" s="30" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="J77" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="K77" s="30">
         <v>1</v>
@@ -22285,13 +22285,13 @@
         <v>5</v>
       </c>
       <c r="M77" s="90" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="N77" s="80" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="O77" s="55" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="P77" s="30"/>
     </row>
@@ -22308,22 +22308,22 @@
         <v>85</v>
       </c>
       <c r="E78" s="31" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F78" s="31" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="G78" s="31" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="H78" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I78" s="31" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="J78" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="K78" s="31">
         <v>1</v>
@@ -22333,7 +22333,7 @@
         <v>5</v>
       </c>
       <c r="M78" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N78" s="80">
         <v>2.89</v>
@@ -22357,20 +22357,20 @@
         <v>86</v>
       </c>
       <c r="E79" s="30" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F79" s="30" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="G79" s="30" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="H79" s="30"/>
       <c r="I79" s="30" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="J79" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="K79" s="30">
         <v>1</v>
@@ -22380,7 +22380,7 @@
         <v>5</v>
       </c>
       <c r="M79" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N79" s="79">
         <v>1.1499999999999999</v>
@@ -22404,22 +22404,22 @@
         <v>87</v>
       </c>
       <c r="E80" s="49" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F80" s="49" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="G80" s="49" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="H80" s="49" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I80" s="49" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="J80" s="49" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="K80" s="49">
         <v>1</v>
@@ -22429,7 +22429,7 @@
         <v>5</v>
       </c>
       <c r="M80" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N80" s="83">
         <v>2.5099999999999998</v>
@@ -22453,22 +22453,22 @@
         <v>88</v>
       </c>
       <c r="E81" s="51" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F81" s="51" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="G81" s="51" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="H81" s="51" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I81" s="51" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="J81" s="51" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="K81" s="51">
         <v>1</v>
@@ -22478,7 +22478,7 @@
         <v>5</v>
       </c>
       <c r="M81" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N81" s="84">
         <v>0.9</v>
@@ -22502,20 +22502,20 @@
         <v>89</v>
       </c>
       <c r="E82" s="31" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="F82" s="31" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="G82" s="31" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="H82" s="31"/>
       <c r="I82" s="31" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="J82" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="K82" s="31">
         <v>1</v>
@@ -22525,7 +22525,7 @@
         <v>5</v>
       </c>
       <c r="M82" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N82" s="80">
         <v>1.53</v>
@@ -22549,22 +22549,22 @@
         <v>90</v>
       </c>
       <c r="E83" s="51" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F83" s="51" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="G83" s="51" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="H83" s="51" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I83" s="51" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="J83" s="51" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="K83" s="51">
         <v>1</v>
@@ -22574,7 +22574,7 @@
         <v>5</v>
       </c>
       <c r="M83" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N83" s="84">
         <v>3.54</v>
@@ -22598,22 +22598,22 @@
         <v>91</v>
       </c>
       <c r="E84" s="31" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F84" s="31" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="G84" s="31" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="H84" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I84" s="31" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="J84" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="K84" s="31">
         <v>3</v>
@@ -22623,7 +22623,7 @@
         <v>15</v>
       </c>
       <c r="M84" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N84" s="80">
         <v>1.69</v>
@@ -22647,22 +22647,22 @@
         <v>92</v>
       </c>
       <c r="E85" s="30" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F85" s="30" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="G85" s="30" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="H85" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I85" s="30" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="J85" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="K85" s="30">
         <v>1</v>
@@ -22672,13 +22672,13 @@
         <v>5</v>
       </c>
       <c r="M85" s="90" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="N85" s="80" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="O85" s="55" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="P85" s="30"/>
     </row>
@@ -22695,22 +22695,22 @@
         <v>93</v>
       </c>
       <c r="E86" s="31" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F86" s="31" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G86" s="31" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="H86" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I86" s="31" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="J86" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="K86" s="31">
         <v>1</v>
@@ -22720,7 +22720,7 @@
         <v>5</v>
       </c>
       <c r="M86" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N86" s="80">
         <v>2.14</v>
@@ -22744,22 +22744,22 @@
         <v>94</v>
       </c>
       <c r="E87" s="30" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F87" s="30" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="G87" s="30" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="H87" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I87" s="30" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="J87" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="K87" s="30">
         <v>1</v>
@@ -22769,13 +22769,13 @@
         <v>5</v>
       </c>
       <c r="M87" s="90" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="N87" s="80" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="O87" s="55" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="P87" s="30"/>
     </row>
@@ -22792,22 +22792,22 @@
         <v>95</v>
       </c>
       <c r="E88" s="31" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F88" s="31" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="G88" s="31" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="H88" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I88" s="31" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="J88" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="K88" s="31">
         <v>1</v>
@@ -22817,7 +22817,7 @@
         <v>5</v>
       </c>
       <c r="M88" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N88" s="80">
         <v>4</v>
@@ -22841,22 +22841,22 @@
         <v>96</v>
       </c>
       <c r="E89" s="30" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F89" s="30" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="G89" s="30" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="H89" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I89" s="30" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="J89" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="K89" s="30">
         <v>1</v>
@@ -22866,7 +22866,7 @@
         <v>5</v>
       </c>
       <c r="M89" s="89" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N89" s="79">
         <v>4.17</v>
@@ -22890,22 +22890,22 @@
         <v>97</v>
       </c>
       <c r="E90" s="31" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="F90" s="31" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="G90" s="31" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="H90" s="31" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I90" s="31" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="J90" s="31" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="K90" s="31">
         <v>1</v>
@@ -22915,13 +22915,13 @@
         <v>5</v>
       </c>
       <c r="M90" s="90" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="N90" s="80" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="O90" s="55" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="P90" s="31"/>
     </row>
@@ -22938,22 +22938,22 @@
         <v>98</v>
       </c>
       <c r="E91" s="30" t="s">
-        <v>402</v>
+        <v>399</v>
       </c>
       <c r="F91" s="30" t="s">
+        <v>400</v>
+      </c>
+      <c r="G91" s="30" t="s">
+        <v>401</v>
+      </c>
+      <c r="H91" s="30" t="s">
+        <v>371</v>
+      </c>
+      <c r="I91" s="30" t="s">
         <v>403</v>
       </c>
-      <c r="G91" s="30" t="s">
-        <v>404</v>
-      </c>
-      <c r="H91" s="30" t="s">
-        <v>373</v>
-      </c>
-      <c r="I91" s="30" t="s">
-        <v>406</v>
-      </c>
       <c r="J91" s="30" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="K91" s="30">
         <v>1</v>
@@ -22963,13 +22963,13 @@
         <v>5</v>
       </c>
       <c r="M91" s="90" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="N91" s="80" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="O91" s="55" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="P91" s="31"/>
     </row>
@@ -22980,28 +22980,28 @@
         <v>83</v>
       </c>
       <c r="C92" s="43" t="s">
+        <v>417</v>
+      </c>
+      <c r="D92" s="51" t="s">
+        <v>371</v>
+      </c>
+      <c r="E92" s="51" t="s">
+        <v>418</v>
+      </c>
+      <c r="F92" s="51" t="s">
+        <v>371</v>
+      </c>
+      <c r="G92" s="51" t="s">
+        <v>419</v>
+      </c>
+      <c r="H92" s="95" t="s">
+        <v>371</v>
+      </c>
+      <c r="I92" s="51" t="s">
         <v>420</v>
       </c>
-      <c r="D92" s="51" t="s">
-        <v>373</v>
-      </c>
-      <c r="E92" s="51" t="s">
-        <v>421</v>
-      </c>
-      <c r="F92" s="51" t="s">
-        <v>373</v>
-      </c>
-      <c r="G92" s="51" t="s">
-        <v>422</v>
-      </c>
-      <c r="H92" s="95" t="s">
-        <v>373</v>
-      </c>
-      <c r="I92" s="51" t="s">
-        <v>423</v>
-      </c>
       <c r="J92" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="K92" s="95">
         <v>1</v>
@@ -23011,13 +23011,13 @@
         <v>5</v>
       </c>
       <c r="M92" s="90" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="N92" s="80" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="O92" s="55" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="P92" s="97"/>
     </row>
@@ -23034,7 +23034,7 @@
       <c r="J93" s="70"/>
       <c r="K93" s="70"/>
       <c r="L93" s="101" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
       <c r="M93" s="102"/>
       <c r="N93" s="103"/>
@@ -23056,7 +23056,7 @@
       <c r="J94" s="9"/>
       <c r="K94" s="9"/>
       <c r="L94" s="101" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
       <c r="M94" s="103"/>
       <c r="N94" s="103"/>

</xml_diff>

<commit_message>
#29 eSpark And Client BOM Updated.
</commit_message>
<xml_diff>
--- a/Design Files/Baseboard-v2.0/BOM/Client_BOM_Baseboard-v2.0.xlsx
+++ b/Design Files/Baseboard-v2.0/BOM/Client_BOM_Baseboard-v2.0.xlsx
@@ -102,9 +102,6 @@
     <t>C2, C9, C10, C13, C16, C17, C22, C23, C24, C27, C28, C32, C33, C34, C35, C36, C37, C38, C40, C41, C42, C43, C44, C45, C54</t>
   </si>
   <si>
-    <t>C3, C19, C20</t>
-  </si>
-  <si>
     <t>C4, C5, C6</t>
   </si>
   <si>
@@ -126,9 +123,6 @@
     <t>C18, C21, C26, C39</t>
   </si>
   <si>
-    <t>C25, C48</t>
-  </si>
-  <si>
     <t>C29, C30</t>
   </si>
   <si>
@@ -1291,6 +1285,12 @@
   </si>
   <si>
     <t>HJ-SMA175</t>
+  </si>
+  <si>
+    <t>C3, C19</t>
+  </si>
+  <si>
+    <t>C20, C25, C48</t>
   </si>
 </sst>
 </file>
@@ -2455,7 +2455,7 @@
       </c>
       <c r="E2" s="10"/>
       <c r="F2" s="39" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="G2" s="11"/>
       <c r="H2" s="11"/>
@@ -2477,7 +2477,7 @@
       </c>
       <c r="E3" s="12"/>
       <c r="F3" s="40" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="G3" s="12"/>
       <c r="H3" s="12"/>
@@ -2499,7 +2499,7 @@
       </c>
       <c r="E4" s="12"/>
       <c r="F4" s="41" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="G4" s="13"/>
       <c r="H4" s="13"/>
@@ -2600,40 +2600,40 @@
         <v>23</v>
       </c>
       <c r="E9" s="29" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="F9" s="29" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="G9" s="29" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="H9" s="29" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="I9" s="29" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="J9" s="29" t="s">
+        <v>380</v>
+      </c>
+      <c r="K9" s="29" t="s">
+        <v>366</v>
+      </c>
+      <c r="L9" s="85" t="s">
+        <v>381</v>
+      </c>
+      <c r="M9" s="29" t="s">
         <v>382</v>
       </c>
-      <c r="K9" s="29" t="s">
-        <v>368</v>
-      </c>
-      <c r="L9" s="85" t="s">
+      <c r="N9" s="86" t="s">
         <v>383</v>
       </c>
-      <c r="M9" s="29" t="s">
+      <c r="O9" s="29" t="s">
         <v>384</v>
       </c>
-      <c r="N9" s="86" t="s">
+      <c r="P9" s="29" t="s">
         <v>385</v>
-      </c>
-      <c r="O9" s="29" t="s">
-        <v>386</v>
-      </c>
-      <c r="P9" s="29" t="s">
-        <v>387</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
@@ -2643,28 +2643,28 @@
         <v>1</v>
       </c>
       <c r="C10" s="43" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="D10" s="44" t="s">
         <v>24</v>
       </c>
       <c r="E10" s="44" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="F10" s="44" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="G10" s="44" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="H10" s="52" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I10" s="52" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="J10" s="44" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K10" s="44">
         <v>1</v>
@@ -2674,13 +2674,13 @@
         <v>5</v>
       </c>
       <c r="M10" s="44" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="N10" s="87" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="O10" s="52" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="P10" s="30"/>
     </row>
@@ -2697,22 +2697,22 @@
         <v>25</v>
       </c>
       <c r="E11" s="31" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="F11" s="31" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="G11" s="31" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="H11" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I11" s="31" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="J11" s="31" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="K11" s="31">
         <v>1</v>
@@ -2722,7 +2722,7 @@
         <v>5</v>
       </c>
       <c r="M11" s="54" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N11" s="80">
         <v>0.48</v>
@@ -2746,22 +2746,22 @@
         <v>26</v>
       </c>
       <c r="E12" s="30" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="F12" s="30" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="G12" s="30" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="H12" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I12" s="30" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="J12" s="30" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="K12" s="30">
         <v>25</v>
@@ -2771,7 +2771,7 @@
         <v>125</v>
       </c>
       <c r="M12" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N12" s="79">
         <v>1.03E-2</v>
@@ -2792,42 +2792,42 @@
         <v>7</v>
       </c>
       <c r="D13" s="31" t="s">
-        <v>27</v>
+        <v>422</v>
       </c>
       <c r="E13" s="31" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="F13" s="31" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="G13" s="31" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="H13" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I13" s="31" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="J13" s="31" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="K13" s="31">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L13" s="74">
         <f t="shared" ref="L13" si="3">K13*5</f>
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="M13" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N13" s="80">
         <v>1.6E-2</v>
       </c>
       <c r="O13" s="55">
         <f t="shared" ref="O13" si="4">N13*L13</f>
-        <v>0.24</v>
+        <v>0.16</v>
       </c>
       <c r="P13" s="31"/>
     </row>
@@ -2841,25 +2841,25 @@
         <v>7</v>
       </c>
       <c r="D14" s="30" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E14" s="30" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="F14" s="30" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="G14" s="30" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="H14" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I14" s="30" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="J14" s="30" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="K14" s="30">
         <v>3</v>
@@ -2869,13 +2869,13 @@
         <v>15</v>
       </c>
       <c r="M14" s="90" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="N14" s="79" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="O14" s="56" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="P14" s="30"/>
     </row>
@@ -2889,25 +2889,25 @@
         <v>7</v>
       </c>
       <c r="D15" s="31" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E15" s="31" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="F15" s="31" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="G15" s="31" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="H15" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I15" s="31" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="J15" s="31" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="K15" s="31">
         <v>2</v>
@@ -2917,7 +2917,7 @@
         <v>10</v>
       </c>
       <c r="M15" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N15" s="80">
         <v>0.72599999999999998</v>
@@ -2938,25 +2938,25 @@
         <v>7</v>
       </c>
       <c r="D16" s="30" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E16" s="30" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="F16" s="30" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="G16" s="30" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="H16" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I16" s="30" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="J16" s="30" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="K16" s="30">
         <v>1</v>
@@ -2966,13 +2966,13 @@
         <v>5</v>
       </c>
       <c r="M16" s="90" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="N16" s="79" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="O16" s="56" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="P16" s="30"/>
     </row>
@@ -2986,25 +2986,25 @@
         <v>7</v>
       </c>
       <c r="D17" s="31" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E17" s="31" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="F17" s="31" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="G17" s="31" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="H17" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I17" s="31" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="J17" s="31" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="K17" s="31">
         <v>1</v>
@@ -3014,13 +3014,13 @@
         <v>5</v>
       </c>
       <c r="M17" s="90" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="N17" s="80" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="O17" s="55" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="P17" s="31"/>
     </row>
@@ -3034,25 +3034,25 @@
         <v>7</v>
       </c>
       <c r="D18" s="30" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E18" s="30" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="F18" s="30" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="G18" s="30" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="H18" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I18" s="30" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="J18" s="30" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="K18" s="30">
         <v>1</v>
@@ -3062,7 +3062,7 @@
         <v>5</v>
       </c>
       <c r="M18" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N18" s="79">
         <v>3.42</v>
@@ -3083,25 +3083,25 @@
         <v>7</v>
       </c>
       <c r="D19" s="31" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E19" s="31" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="F19" s="31" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G19" s="31" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="H19" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I19" s="31" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="J19" s="31" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="K19" s="31">
         <v>1</v>
@@ -3111,7 +3111,7 @@
         <v>5</v>
       </c>
       <c r="M19" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N19" s="80">
         <v>0.68</v>
@@ -3132,25 +3132,25 @@
         <v>7</v>
       </c>
       <c r="D20" s="30" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E20" s="30" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="F20" s="30" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="G20" s="44" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="H20" s="30" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="I20" s="30" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="J20" s="30" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="K20" s="30">
         <v>4</v>
@@ -3160,7 +3160,7 @@
         <v>20</v>
       </c>
       <c r="M20" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N20" s="79">
         <v>6.2E-2</v>
@@ -3181,42 +3181,42 @@
         <v>7</v>
       </c>
       <c r="D21" s="31" t="s">
-        <v>35</v>
+        <v>423</v>
       </c>
       <c r="E21" s="31" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="F21" s="31" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="G21" s="31" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="H21" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I21" s="31" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="J21" s="31" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="K21" s="31">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L21" s="74">
         <f t="shared" ref="L21" si="10">K21*5</f>
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="M21" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N21" s="80">
         <v>0.121</v>
       </c>
       <c r="O21" s="55">
         <f t="shared" ref="O21" si="11">N21*L21</f>
-        <v>1.21</v>
+        <v>1.8149999999999999</v>
       </c>
       <c r="P21" s="31"/>
     </row>
@@ -3230,25 +3230,25 @@
         <v>7</v>
       </c>
       <c r="D22" s="30" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E22" s="30" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F22" s="30" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="G22" s="30" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="H22" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I22" s="30" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="J22" s="30" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="K22" s="30">
         <v>2</v>
@@ -3258,7 +3258,7 @@
         <v>10</v>
       </c>
       <c r="M22" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N22" s="79">
         <v>1.9E-2</v>
@@ -3279,25 +3279,25 @@
         <v>7</v>
       </c>
       <c r="D23" s="31" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E23" s="31" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F23" s="31" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="G23" s="31" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="H23" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I23" s="31" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="J23" s="31" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="K23" s="31">
         <v>3</v>
@@ -3307,7 +3307,7 @@
         <v>15</v>
       </c>
       <c r="M23" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N23" s="80">
         <v>7.3999999999999996E-2</v>
@@ -3328,25 +3328,25 @@
         <v>8</v>
       </c>
       <c r="D24" s="30" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E24" s="30" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F24" s="30" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="G24" s="30" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="H24" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I24" s="30" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="J24" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K24" s="30">
         <v>1</v>
@@ -3356,7 +3356,7 @@
         <v>5</v>
       </c>
       <c r="M24" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N24" s="79">
         <v>0.44</v>
@@ -3377,25 +3377,25 @@
         <v>8</v>
       </c>
       <c r="D25" s="31" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E25" s="31" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="F25" s="31" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="G25" s="31" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="H25" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I25" s="31" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="J25" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K25" s="31">
         <v>1</v>
@@ -3405,11 +3405,11 @@
         <v>5</v>
       </c>
       <c r="M25" s="90" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="N25" s="80"/>
       <c r="O25" s="55" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="P25" s="31"/>
     </row>
@@ -3423,25 +3423,25 @@
         <v>8</v>
       </c>
       <c r="D26" s="30" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E26" s="30" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="F26" s="30" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="G26" s="30" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="H26" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I26" s="30" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="J26" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K26" s="30">
         <v>1</v>
@@ -3451,11 +3451,11 @@
         <v>5</v>
       </c>
       <c r="M26" s="90" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="N26" s="79"/>
       <c r="O26" s="56" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="P26" s="30"/>
     </row>
@@ -3469,25 +3469,25 @@
         <v>8</v>
       </c>
       <c r="D27" s="31" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E27" s="31" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F27" s="31" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="G27" s="31" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="H27" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I27" s="31" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="J27" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K27" s="31">
         <v>1</v>
@@ -3497,11 +3497,11 @@
         <v>5</v>
       </c>
       <c r="M27" s="90" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="N27" s="80"/>
       <c r="O27" s="55" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="P27" s="31"/>
     </row>
@@ -3515,25 +3515,25 @@
         <v>8</v>
       </c>
       <c r="D28" s="30" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E28" s="30" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="F28" s="30" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="G28" s="30" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="H28" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I28" s="30" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="J28" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K28" s="30">
         <v>3</v>
@@ -3543,7 +3543,7 @@
         <v>15</v>
       </c>
       <c r="M28" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N28" s="79">
         <v>0.184</v>
@@ -3564,25 +3564,25 @@
         <v>8</v>
       </c>
       <c r="D29" s="31" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="E29" s="31" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="F29" s="31" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="G29" s="31" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="H29" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I29" s="31" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="J29" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K29" s="31">
         <v>2</v>
@@ -3592,11 +3592,11 @@
         <v>10</v>
       </c>
       <c r="M29" s="90" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="N29" s="80"/>
       <c r="O29" s="55" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="P29" s="31"/>
     </row>
@@ -3610,25 +3610,25 @@
         <v>8</v>
       </c>
       <c r="D30" s="30" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E30" s="30" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="F30" s="30" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="G30" s="30" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="H30" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I30" s="30" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="J30" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K30" s="30">
         <v>4</v>
@@ -3638,7 +3638,7 @@
         <v>20</v>
       </c>
       <c r="M30" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N30" s="79">
         <v>0.32300000000000001</v>
@@ -3659,25 +3659,25 @@
         <v>8</v>
       </c>
       <c r="D31" s="31" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E31" s="31" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="F31" s="31" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="G31" s="31" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="H31" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I31" s="31" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="J31" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K31" s="31">
         <v>4</v>
@@ -3687,11 +3687,11 @@
         <v>20</v>
       </c>
       <c r="M31" s="90" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="N31" s="80"/>
       <c r="O31" s="55" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="P31" s="31"/>
     </row>
@@ -3705,25 +3705,25 @@
         <v>9</v>
       </c>
       <c r="D32" s="30" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E32" s="30" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="F32" s="30" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="G32" s="30" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="H32" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I32" s="30" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="J32" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K32" s="30">
         <v>1</v>
@@ -3733,7 +3733,7 @@
         <v>5</v>
       </c>
       <c r="M32" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N32" s="79">
         <v>1.766</v>
@@ -3754,25 +3754,25 @@
         <v>9</v>
       </c>
       <c r="D33" s="31" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E33" s="31" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="F33" s="31" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="G33" s="31" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="H33" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I33" s="31" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="J33" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K33" s="31">
         <v>1</v>
@@ -3782,11 +3782,11 @@
         <v>5</v>
       </c>
       <c r="M33" s="90" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="N33" s="80"/>
       <c r="O33" s="55" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="P33" s="31"/>
     </row>
@@ -3800,25 +3800,25 @@
         <v>9</v>
       </c>
       <c r="D34" s="30" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E34" s="30" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="F34" s="30" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="G34" s="30" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="H34" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I34" s="30" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="J34" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K34" s="30">
         <v>4</v>
@@ -3828,11 +3828,11 @@
         <v>20</v>
       </c>
       <c r="M34" s="90" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="N34" s="79"/>
       <c r="O34" s="56" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="P34" s="30"/>
     </row>
@@ -3846,25 +3846,25 @@
         <v>10</v>
       </c>
       <c r="D35" s="31" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E35" s="31" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="F35" s="31" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="G35" s="31" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="H35" s="53" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="I35" s="31" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="J35" s="31" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="K35" s="31">
         <v>1</v>
@@ -3874,7 +3874,7 @@
         <v>5</v>
       </c>
       <c r="M35" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N35" s="80">
         <v>0.28000000000000003</v>
@@ -3895,25 +3895,25 @@
         <v>11</v>
       </c>
       <c r="D36" s="30" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E36" s="30" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="F36" s="31" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="G36" s="30" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="H36" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I36" s="30" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="J36" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K36" s="30">
         <v>8</v>
@@ -3923,13 +3923,13 @@
         <v>40</v>
       </c>
       <c r="M36" s="90" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="N36" s="79" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="O36" s="56" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="P36" s="30"/>
     </row>
@@ -3943,25 +3943,25 @@
         <v>12</v>
       </c>
       <c r="D37" s="31" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E37" s="31" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="F37" s="31" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="G37" s="31" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="H37" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I37" s="31" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="J37" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K37" s="31">
         <v>1</v>
@@ -3971,13 +3971,13 @@
         <v>5</v>
       </c>
       <c r="M37" s="90" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="N37" s="80" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="O37" s="55" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="P37" s="31"/>
     </row>
@@ -3991,25 +3991,25 @@
         <v>11</v>
       </c>
       <c r="D38" s="30" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E38" s="30" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="F38" s="31" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="G38" s="30" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="H38" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I38" s="30" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="J38" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K38" s="30">
         <v>4</v>
@@ -4019,13 +4019,13 @@
         <v>20</v>
       </c>
       <c r="M38" s="90" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="N38" s="79" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="O38" s="56" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="P38" s="30"/>
     </row>
@@ -4036,28 +4036,28 @@
         <v>30</v>
       </c>
       <c r="C39" s="45" t="s">
+        <v>406</v>
+      </c>
+      <c r="D39" s="92" t="s">
+        <v>51</v>
+      </c>
+      <c r="E39" s="31" t="s">
+        <v>407</v>
+      </c>
+      <c r="F39" s="31" t="s">
+        <v>370</v>
+      </c>
+      <c r="G39" s="31" t="s">
         <v>408</v>
       </c>
-      <c r="D39" s="92" t="s">
-        <v>53</v>
-      </c>
-      <c r="E39" s="31" t="s">
+      <c r="H39" s="31" t="s">
+        <v>369</v>
+      </c>
+      <c r="I39" s="31" t="s">
         <v>409</v>
       </c>
-      <c r="F39" s="31" t="s">
-        <v>372</v>
-      </c>
-      <c r="G39" s="31" t="s">
-        <v>410</v>
-      </c>
-      <c r="H39" s="31" t="s">
-        <v>371</v>
-      </c>
-      <c r="I39" s="31" t="s">
-        <v>411</v>
-      </c>
       <c r="J39" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K39" s="31">
         <v>1</v>
@@ -4067,13 +4067,13 @@
         <v>5</v>
       </c>
       <c r="M39" s="90" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="N39" s="79" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="O39" s="56" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="P39" s="31"/>
     </row>
@@ -4087,25 +4087,25 @@
         <v>13</v>
       </c>
       <c r="D40" s="30" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E40" s="30" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="F40" s="31" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="G40" s="30" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="H40" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I40" s="30" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="J40" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K40" s="30">
         <v>1</v>
@@ -4115,13 +4115,13 @@
         <v>5</v>
       </c>
       <c r="M40" s="90" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="N40" s="79" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="O40" s="56" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="P40" s="30"/>
     </row>
@@ -4132,26 +4132,26 @@
         <v>32</v>
       </c>
       <c r="C41" s="45" t="s">
+        <v>419</v>
+      </c>
+      <c r="D41" s="31" t="s">
+        <v>53</v>
+      </c>
+      <c r="E41" s="31" t="s">
+        <v>420</v>
+      </c>
+      <c r="F41" s="31" t="s">
+        <v>370</v>
+      </c>
+      <c r="G41" s="31" t="s">
         <v>421</v>
-      </c>
-      <c r="D41" s="31" t="s">
-        <v>55</v>
-      </c>
-      <c r="E41" s="31" t="s">
-        <v>422</v>
-      </c>
-      <c r="F41" s="31" t="s">
-        <v>372</v>
-      </c>
-      <c r="G41" s="31" t="s">
-        <v>423</v>
       </c>
       <c r="H41" s="31"/>
       <c r="I41" s="31" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="J41" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K41" s="31">
         <v>1</v>
@@ -4161,13 +4161,13 @@
         <v>5</v>
       </c>
       <c r="M41" s="90" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="N41" s="80" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="O41" s="55" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="P41" s="31"/>
     </row>
@@ -4181,25 +4181,25 @@
         <v>14</v>
       </c>
       <c r="D42" s="30" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E42" s="30" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="F42" s="31" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="G42" s="30" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="H42" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I42" s="30" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="J42" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K42" s="30">
         <v>2</v>
@@ -4209,13 +4209,13 @@
         <v>10</v>
       </c>
       <c r="M42" s="90" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="N42" s="79" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="O42" s="56" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="P42" s="30"/>
     </row>
@@ -4226,28 +4226,28 @@
         <v>34</v>
       </c>
       <c r="C43" s="45" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="D43" s="31" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E43" s="31" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="F43" s="31" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="G43" s="31" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="H43" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I43" s="31" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="J43" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K43" s="31">
         <v>3</v>
@@ -4257,7 +4257,7 @@
         <v>15</v>
       </c>
       <c r="M43" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N43" s="80">
         <v>0.90900000000000003</v>
@@ -4278,25 +4278,25 @@
         <v>15</v>
       </c>
       <c r="D44" s="30" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E44" s="30" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="F44" s="31" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="G44" s="30" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="H44" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I44" s="30" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="J44" s="30" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="K44" s="30">
         <v>1</v>
@@ -4306,13 +4306,13 @@
         <v>5</v>
       </c>
       <c r="M44" s="90" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="N44" s="79" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="O44" s="56" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="P44" s="30"/>
     </row>
@@ -4326,25 +4326,25 @@
         <v>15</v>
       </c>
       <c r="D45" s="31" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E45" s="31" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="F45" s="31" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="G45" s="31" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="H45" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I45" s="31" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="J45" s="31" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="K45" s="31">
         <v>1</v>
@@ -4354,13 +4354,13 @@
         <v>5</v>
       </c>
       <c r="M45" s="90" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="N45" s="80" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="O45" s="55" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="P45" s="31"/>
     </row>
@@ -4374,25 +4374,25 @@
         <v>16</v>
       </c>
       <c r="D46" s="30" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E46" s="30" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="F46" s="30" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="G46" s="30" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="H46" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I46" s="30" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="J46" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K46" s="30">
         <v>2</v>
@@ -4402,13 +4402,13 @@
         <v>10</v>
       </c>
       <c r="M46" s="90" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="N46" s="79" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="O46" s="79" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="P46" s="30"/>
     </row>
@@ -4422,25 +4422,25 @@
         <v>16</v>
       </c>
       <c r="D47" s="31" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E47" s="31" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="F47" s="31" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="G47" s="31" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="H47" s="53" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="I47" s="31" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="J47" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K47" s="31">
         <v>1</v>
@@ -4450,13 +4450,13 @@
         <v>5</v>
       </c>
       <c r="M47" s="90" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="N47" s="80" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="O47" s="80" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="P47" s="31"/>
     </row>
@@ -4467,28 +4467,28 @@
         <v>39</v>
       </c>
       <c r="C48" s="43" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="D48" s="44" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="E48" s="44" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="F48" s="44" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="G48" s="44" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="H48" s="44" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I48" s="44" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="J48" s="44" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K48" s="44">
         <v>10</v>
@@ -4498,13 +4498,13 @@
         <v>50</v>
       </c>
       <c r="M48" s="88" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="N48" s="81" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="O48" s="44" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="P48" s="30"/>
     </row>
@@ -4515,28 +4515,28 @@
         <v>40</v>
       </c>
       <c r="C49" s="45" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="D49" s="31" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E49" s="31" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="F49" s="31" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="G49" s="31" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="H49" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I49" s="31" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="J49" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K49" s="31">
         <v>1</v>
@@ -4546,7 +4546,7 @@
         <v>5</v>
       </c>
       <c r="M49" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N49" s="80">
         <v>0.14000000000000001</v>
@@ -4567,25 +4567,25 @@
         <v>17</v>
       </c>
       <c r="D50" s="30" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E50" s="30" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="F50" s="30" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="G50" s="44" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="H50" s="30" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="I50" s="30" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="J50" s="30" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="K50" s="30">
         <v>2</v>
@@ -4595,7 +4595,7 @@
         <v>10</v>
       </c>
       <c r="M50" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N50" s="79">
         <v>0.33600000000000002</v>
@@ -4616,25 +4616,25 @@
         <v>18</v>
       </c>
       <c r="D51" s="31" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E51" s="31" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="F51" s="31" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="G51" s="31" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="H51" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I51" s="31" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="J51" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K51" s="31">
         <v>1</v>
@@ -4644,16 +4644,16 @@
         <v>5</v>
       </c>
       <c r="M51" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N51" s="80" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="O51" s="55" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="P51" s="94" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
     </row>
     <row r="52" spans="1:16384" x14ac:dyDescent="0.25">
@@ -4666,25 +4666,25 @@
         <v>17</v>
       </c>
       <c r="D52" s="30" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E52" s="30" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="F52" s="30" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="G52" s="30" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="H52" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I52" s="30" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="J52" s="30" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="K52" s="30">
         <v>1</v>
@@ -4694,7 +4694,7 @@
         <v>5</v>
       </c>
       <c r="M52" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N52" s="79">
         <v>0.1</v>
@@ -4715,25 +4715,25 @@
         <v>17</v>
       </c>
       <c r="D53" s="31" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="E53" s="31" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="F53" s="31" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="G53" s="31" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="H53" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I53" s="31" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="J53" s="31" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="K53" s="31">
         <v>12</v>
@@ -4743,7 +4743,7 @@
         <v>60</v>
       </c>
       <c r="M53" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N53" s="80">
         <v>1.6199999999999999E-2</v>
@@ -4764,25 +4764,25 @@
         <v>17</v>
       </c>
       <c r="D54" s="91" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="E54" s="30" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="F54" s="30" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="G54" s="44" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="H54" s="30" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="I54" s="30" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="J54" s="30" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="K54" s="30">
         <v>8</v>
@@ -4792,7 +4792,7 @@
         <v>40</v>
       </c>
       <c r="M54" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N54" s="79">
         <v>2.5999999999999999E-2</v>
@@ -4813,25 +4813,25 @@
         <v>17</v>
       </c>
       <c r="D55" s="31" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="E55" s="31" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="F55" s="31" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="G55" s="31" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="H55" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I55" s="31" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="J55" s="31" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="K55" s="31">
         <v>1</v>
@@ -4841,13 +4841,13 @@
         <v>5</v>
       </c>
       <c r="M55" s="90" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="N55" s="80" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="O55" s="55" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="P55" s="31"/>
     </row>
@@ -4861,25 +4861,25 @@
         <v>17</v>
       </c>
       <c r="D56" s="30" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E56" s="30" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="F56" s="30" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="G56" s="30" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="H56" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I56" s="30" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="J56" s="30" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="K56" s="30">
         <v>2</v>
@@ -4889,7 +4889,7 @@
         <v>10</v>
       </c>
       <c r="M56" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N56" s="79">
         <v>0.02</v>
@@ -4910,25 +4910,25 @@
         <v>17</v>
       </c>
       <c r="D57" s="31" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="E57" s="31" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="F57" s="31" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="G57" s="91" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="H57" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I57" s="31" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="J57" s="31" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="K57" s="31">
         <v>2</v>
@@ -4938,7 +4938,7 @@
         <v>10</v>
       </c>
       <c r="M57" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N57" s="80">
         <v>0.02</v>
@@ -4959,25 +4959,25 @@
         <v>17</v>
       </c>
       <c r="D58" s="30" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E58" s="30" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="F58" s="30" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="G58" s="30" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="H58" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I58" s="30" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="J58" s="30" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="K58" s="30">
         <v>2</v>
@@ -4987,7 +4987,7 @@
         <v>10</v>
       </c>
       <c r="M58" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N58" s="79">
         <v>1.4E-2</v>
@@ -5008,25 +5008,25 @@
         <v>17</v>
       </c>
       <c r="D59" s="31" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="E59" s="31" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="F59" s="31" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="G59" s="31" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="H59" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I59" s="31" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="J59" s="31" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="K59" s="31">
         <v>22</v>
@@ -5036,7 +5036,7 @@
         <v>110</v>
       </c>
       <c r="M59" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N59" s="80">
         <v>7.0000000000000001E-3</v>
@@ -5057,25 +5057,25 @@
         <v>17</v>
       </c>
       <c r="D60" s="30" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E60" s="30" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="F60" s="30" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="G60" s="30" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="H60" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I60" s="30" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="J60" s="30" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="K60" s="30">
         <v>1</v>
@@ -5085,7 +5085,7 @@
         <v>5</v>
       </c>
       <c r="M60" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N60" s="79">
         <v>0.1</v>
@@ -5106,25 +5106,25 @@
         <v>17</v>
       </c>
       <c r="D61" s="31" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="E61" s="30" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="F61" s="30" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="G61" s="30" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="H61" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I61" s="30" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="J61" s="30" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="K61" s="30">
         <v>11</v>
@@ -5134,7 +5134,7 @@
         <v>55</v>
       </c>
       <c r="M61" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N61" s="79">
         <v>6.4000000000000003E-3</v>
@@ -5152,28 +5152,28 @@
         <v>53</v>
       </c>
       <c r="C62" s="45" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="D62" s="91" t="s">
+        <v>411</v>
+      </c>
+      <c r="E62" s="30" t="s">
+        <v>412</v>
+      </c>
+      <c r="F62" s="30" t="s">
+        <v>370</v>
+      </c>
+      <c r="G62" s="30" t="s">
         <v>413</v>
       </c>
-      <c r="E62" s="30" t="s">
-        <v>414</v>
-      </c>
-      <c r="F62" s="30" t="s">
-        <v>372</v>
-      </c>
-      <c r="G62" s="30" t="s">
-        <v>415</v>
-      </c>
       <c r="H62" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I62" s="30" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="J62" s="30" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="K62" s="30">
         <v>3</v>
@@ -5183,7 +5183,7 @@
         <v>15</v>
       </c>
       <c r="M62" s="93" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N62" s="79">
         <v>0.1</v>
@@ -21572,25 +21572,25 @@
         <v>17</v>
       </c>
       <c r="D63" s="30" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E63" s="30" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F63" s="30" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="G63" s="30" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="H63" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I63" s="30" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="J63" s="30" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="K63" s="30">
         <v>4</v>
@@ -21600,7 +21600,7 @@
         <v>20</v>
       </c>
       <c r="M63" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N63" s="79">
         <v>1.4E-2</v>
@@ -21621,25 +21621,25 @@
         <v>17</v>
       </c>
       <c r="D64" s="31" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E64" s="31" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="F64" s="31" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="G64" s="31" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="H64" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I64" s="31" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="J64" s="31" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="K64" s="31">
         <v>1</v>
@@ -21649,7 +21649,7 @@
         <v>5</v>
       </c>
       <c r="M64" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N64" s="80">
         <v>0.1</v>
@@ -21670,25 +21670,25 @@
         <v>17</v>
       </c>
       <c r="D65" s="30" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E65" s="30" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="F65" s="30" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="G65" s="30" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="H65" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I65" s="30" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="J65" s="30" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="K65" s="30">
         <v>1</v>
@@ -21698,7 +21698,7 @@
         <v>5</v>
       </c>
       <c r="M65" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N65" s="79">
         <v>0.1</v>
@@ -21719,25 +21719,25 @@
         <v>17</v>
       </c>
       <c r="D66" s="31" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="E66" s="31" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="F66" s="31" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="G66" s="31" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="H66" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I66" s="31" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="J66" s="31" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="K66" s="31">
         <v>1</v>
@@ -21747,7 +21747,7 @@
         <v>5</v>
       </c>
       <c r="M66" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N66" s="80">
         <v>0.34</v>
@@ -21768,25 +21768,25 @@
         <v>17</v>
       </c>
       <c r="D67" s="31" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="E67" s="31" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="F67" s="31" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="G67" s="91" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="H67" s="31" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="I67" s="31" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="J67" s="31" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="K67" s="31">
         <v>4</v>
@@ -21796,7 +21796,7 @@
         <v>20</v>
       </c>
       <c r="M67" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N67" s="80">
         <v>0.11600000000000001</v>
@@ -21817,25 +21817,25 @@
         <v>17</v>
       </c>
       <c r="D68" s="30" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="E68" s="30" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="F68" s="30" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="G68" s="30" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="H68" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I68" s="30" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="J68" s="30" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="K68" s="30">
         <v>1</v>
@@ -21845,7 +21845,7 @@
         <v>5</v>
       </c>
       <c r="M68" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N68" s="79">
         <v>0.1</v>
@@ -21866,25 +21866,25 @@
         <v>17</v>
       </c>
       <c r="D69" s="31" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="E69" s="31" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="F69" s="31" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="G69" s="31" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="H69" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I69" s="31" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="J69" s="31" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="K69" s="31">
         <v>1</v>
@@ -21894,7 +21894,7 @@
         <v>5</v>
       </c>
       <c r="M69" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N69" s="80">
         <v>0.41</v>
@@ -21915,25 +21915,25 @@
         <v>17</v>
       </c>
       <c r="D70" s="30" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="E70" s="30" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="F70" s="30" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="G70" s="30" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="H70" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I70" s="30" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="J70" s="30" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="K70" s="30">
         <v>2</v>
@@ -21943,7 +21943,7 @@
         <v>10</v>
       </c>
       <c r="M70" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N70" s="79">
         <v>1.7999999999999999E-2</v>
@@ -21964,25 +21964,25 @@
         <v>17</v>
       </c>
       <c r="D71" s="31" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="E71" s="31" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="F71" s="31" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="G71" s="31" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="H71" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I71" s="31" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="J71" s="31" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="K71" s="31">
         <v>1</v>
@@ -21992,7 +21992,7 @@
         <v>5</v>
       </c>
       <c r="M71" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N71" s="80">
         <v>0.1</v>
@@ -22010,28 +22010,28 @@
         <v>63</v>
       </c>
       <c r="C72" s="45" t="s">
+        <v>393</v>
+      </c>
+      <c r="D72" s="31" t="s">
+        <v>394</v>
+      </c>
+      <c r="E72" s="31" t="s">
         <v>395</v>
       </c>
-      <c r="D72" s="31" t="s">
+      <c r="F72" s="31" t="s">
+        <v>370</v>
+      </c>
+      <c r="G72" s="31" t="s">
         <v>396</v>
       </c>
-      <c r="E72" s="31" t="s">
-        <v>397</v>
-      </c>
-      <c r="F72" s="31" t="s">
-        <v>372</v>
-      </c>
-      <c r="G72" s="31" t="s">
-        <v>398</v>
-      </c>
       <c r="H72" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I72" s="31" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="J72" s="31" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="K72" s="31">
         <v>5</v>
@@ -22041,7 +22041,7 @@
         <v>25</v>
       </c>
       <c r="M72" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N72" s="80">
         <v>8.9599999999999999E-2</v>
@@ -22062,25 +22062,25 @@
         <v>19</v>
       </c>
       <c r="D73" s="46" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="E73" s="46" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="F73" s="47" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="G73" s="46" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="H73" s="46" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I73" s="46" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="J73" s="46" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K73" s="46">
         <v>2</v>
@@ -22090,13 +22090,13 @@
         <v>10</v>
       </c>
       <c r="M73" s="88" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="N73" s="82" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="O73" s="46" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="P73" s="30"/>
     </row>
@@ -22110,25 +22110,25 @@
         <v>20</v>
       </c>
       <c r="D74" s="31" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="E74" s="31" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="F74" s="31" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="G74" s="31" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="H74" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I74" s="31" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="J74" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K74" s="31">
         <v>1</v>
@@ -22138,7 +22138,7 @@
         <v>5</v>
       </c>
       <c r="M74" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N74" s="80">
         <v>0.14000000000000001</v>
@@ -22159,25 +22159,25 @@
         <v>21</v>
       </c>
       <c r="D75" s="30" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="E75" s="30" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="F75" s="30" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="G75" s="30" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="H75" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I75" s="30" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="J75" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K75" s="30">
         <v>1</v>
@@ -22187,7 +22187,7 @@
         <v>5</v>
       </c>
       <c r="M75" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N75" s="79">
         <v>5.28</v>
@@ -22208,25 +22208,25 @@
         <v>21</v>
       </c>
       <c r="D76" s="31" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="E76" s="31" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="F76" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="G76" s="31" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="H76" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I76" s="31" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="J76" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K76" s="31">
         <v>1</v>
@@ -22236,7 +22236,7 @@
         <v>5</v>
       </c>
       <c r="M76" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N76" s="80">
         <v>0.88</v>
@@ -22257,25 +22257,25 @@
         <v>21</v>
       </c>
       <c r="D77" s="30" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="E77" s="30" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="F77" s="30" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="G77" s="30" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="H77" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I77" s="30" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="J77" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K77" s="30">
         <v>1</v>
@@ -22285,13 +22285,13 @@
         <v>5</v>
       </c>
       <c r="M77" s="90" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="N77" s="80" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="O77" s="55" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="P77" s="30"/>
     </row>
@@ -22305,25 +22305,25 @@
         <v>21</v>
       </c>
       <c r="D78" s="31" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="E78" s="31" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="F78" s="31" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="G78" s="31" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="H78" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I78" s="31" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="J78" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K78" s="31">
         <v>1</v>
@@ -22333,7 +22333,7 @@
         <v>5</v>
       </c>
       <c r="M78" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N78" s="80">
         <v>2.89</v>
@@ -22354,23 +22354,23 @@
         <v>21</v>
       </c>
       <c r="D79" s="30" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E79" s="30" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="F79" s="30" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="G79" s="30" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="H79" s="30"/>
       <c r="I79" s="30" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="J79" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K79" s="30">
         <v>1</v>
@@ -22380,7 +22380,7 @@
         <v>5</v>
       </c>
       <c r="M79" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N79" s="79">
         <v>1.1499999999999999</v>
@@ -22401,25 +22401,25 @@
         <v>21</v>
       </c>
       <c r="D80" s="49" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="E80" s="49" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="F80" s="49" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="G80" s="49" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="H80" s="49" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I80" s="49" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="J80" s="49" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K80" s="49">
         <v>1</v>
@@ -22429,7 +22429,7 @@
         <v>5</v>
       </c>
       <c r="M80" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N80" s="83">
         <v>2.5099999999999998</v>
@@ -22450,25 +22450,25 @@
         <v>21</v>
       </c>
       <c r="D81" s="51" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="E81" s="51" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="F81" s="51" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="G81" s="51" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="H81" s="51" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I81" s="51" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="J81" s="51" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K81" s="51">
         <v>1</v>
@@ -22478,7 +22478,7 @@
         <v>5</v>
       </c>
       <c r="M81" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N81" s="84">
         <v>0.9</v>
@@ -22499,23 +22499,23 @@
         <v>21</v>
       </c>
       <c r="D82" s="31" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E82" s="31" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="F82" s="31" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="G82" s="31" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="H82" s="31"/>
       <c r="I82" s="31" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="J82" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K82" s="31">
         <v>1</v>
@@ -22525,7 +22525,7 @@
         <v>5</v>
       </c>
       <c r="M82" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N82" s="80">
         <v>1.53</v>
@@ -22546,25 +22546,25 @@
         <v>21</v>
       </c>
       <c r="D83" s="51" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="E83" s="51" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="F83" s="51" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="G83" s="51" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="H83" s="51" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I83" s="51" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="J83" s="51" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K83" s="51">
         <v>1</v>
@@ -22574,7 +22574,7 @@
         <v>5</v>
       </c>
       <c r="M83" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N83" s="84">
         <v>3.54</v>
@@ -22595,25 +22595,25 @@
         <v>21</v>
       </c>
       <c r="D84" s="31" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E84" s="31" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="F84" s="31" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="G84" s="31" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="H84" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I84" s="31" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="J84" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K84" s="31">
         <v>3</v>
@@ -22623,7 +22623,7 @@
         <v>15</v>
       </c>
       <c r="M84" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N84" s="80">
         <v>1.69</v>
@@ -22644,25 +22644,25 @@
         <v>21</v>
       </c>
       <c r="D85" s="30" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="E85" s="30" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="F85" s="30" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="G85" s="30" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="H85" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I85" s="30" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="J85" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K85" s="30">
         <v>1</v>
@@ -22672,13 +22672,13 @@
         <v>5</v>
       </c>
       <c r="M85" s="90" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="N85" s="80" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="O85" s="55" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="P85" s="30"/>
     </row>
@@ -22692,25 +22692,25 @@
         <v>21</v>
       </c>
       <c r="D86" s="31" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="E86" s="31" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="F86" s="31" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="G86" s="31" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="H86" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I86" s="31" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="J86" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K86" s="31">
         <v>1</v>
@@ -22720,7 +22720,7 @@
         <v>5</v>
       </c>
       <c r="M86" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N86" s="80">
         <v>2.14</v>
@@ -22741,25 +22741,25 @@
         <v>21</v>
       </c>
       <c r="D87" s="30" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E87" s="30" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="F87" s="30" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="G87" s="30" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="H87" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I87" s="30" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="J87" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K87" s="30">
         <v>1</v>
@@ -22769,13 +22769,13 @@
         <v>5</v>
       </c>
       <c r="M87" s="90" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="N87" s="80" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="O87" s="55" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="P87" s="30"/>
     </row>
@@ -22789,25 +22789,25 @@
         <v>21</v>
       </c>
       <c r="D88" s="31" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E88" s="31" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="F88" s="31" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="G88" s="31" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="H88" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I88" s="31" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="J88" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K88" s="31">
         <v>1</v>
@@ -22817,7 +22817,7 @@
         <v>5</v>
       </c>
       <c r="M88" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N88" s="80">
         <v>4</v>
@@ -22838,25 +22838,25 @@
         <v>21</v>
       </c>
       <c r="D89" s="30" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="E89" s="30" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="F89" s="30" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="G89" s="30" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="H89" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I89" s="30" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="J89" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K89" s="30">
         <v>1</v>
@@ -22866,7 +22866,7 @@
         <v>5</v>
       </c>
       <c r="M89" s="89" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N89" s="79">
         <v>4.17</v>
@@ -22887,25 +22887,25 @@
         <v>22</v>
       </c>
       <c r="D90" s="31" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="E90" s="31" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="F90" s="31" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="G90" s="31" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="H90" s="31" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I90" s="31" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="J90" s="31" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="K90" s="31">
         <v>1</v>
@@ -22915,13 +22915,13 @@
         <v>5</v>
       </c>
       <c r="M90" s="90" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="N90" s="80" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="O90" s="55" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="P90" s="31"/>
     </row>
@@ -22935,25 +22935,25 @@
         <v>22</v>
       </c>
       <c r="D91" s="30" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="E91" s="30" t="s">
+        <v>397</v>
+      </c>
+      <c r="F91" s="30" t="s">
+        <v>398</v>
+      </c>
+      <c r="G91" s="30" t="s">
         <v>399</v>
       </c>
-      <c r="F91" s="30" t="s">
-        <v>400</v>
-      </c>
-      <c r="G91" s="30" t="s">
+      <c r="H91" s="30" t="s">
+        <v>369</v>
+      </c>
+      <c r="I91" s="30" t="s">
         <v>401</v>
       </c>
-      <c r="H91" s="30" t="s">
-        <v>371</v>
-      </c>
-      <c r="I91" s="30" t="s">
-        <v>403</v>
-      </c>
       <c r="J91" s="30" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="K91" s="30">
         <v>1</v>
@@ -22963,13 +22963,13 @@
         <v>5</v>
       </c>
       <c r="M91" s="90" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="N91" s="80" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="O91" s="55" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="P91" s="31"/>
     </row>
@@ -22980,28 +22980,28 @@
         <v>83</v>
       </c>
       <c r="C92" s="43" t="s">
+        <v>415</v>
+      </c>
+      <c r="D92" s="51" t="s">
+        <v>369</v>
+      </c>
+      <c r="E92" s="51" t="s">
+        <v>416</v>
+      </c>
+      <c r="F92" s="51" t="s">
+        <v>369</v>
+      </c>
+      <c r="G92" s="51" t="s">
         <v>417</v>
       </c>
-      <c r="D92" s="51" t="s">
-        <v>371</v>
-      </c>
-      <c r="E92" s="51" t="s">
+      <c r="H92" s="95" t="s">
+        <v>369</v>
+      </c>
+      <c r="I92" s="51" t="s">
         <v>418</v>
       </c>
-      <c r="F92" s="51" t="s">
-        <v>371</v>
-      </c>
-      <c r="G92" s="51" t="s">
-        <v>419</v>
-      </c>
-      <c r="H92" s="95" t="s">
-        <v>371</v>
-      </c>
-      <c r="I92" s="51" t="s">
-        <v>420</v>
-      </c>
       <c r="J92" s="30" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K92" s="95">
         <v>1</v>
@@ -23011,13 +23011,13 @@
         <v>5</v>
       </c>
       <c r="M92" s="90" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="N92" s="80" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="O92" s="55" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="P92" s="97"/>
     </row>
@@ -23034,13 +23034,13 @@
       <c r="J93" s="70"/>
       <c r="K93" s="70"/>
       <c r="L93" s="101" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="M93" s="102"/>
       <c r="N93" s="103"/>
       <c r="O93" s="59">
         <f>SUM(O10:O91)</f>
-        <v>262.72650000000004</v>
+        <v>263.25150000000002</v>
       </c>
       <c r="P93" s="71"/>
     </row>
@@ -23056,13 +23056,13 @@
       <c r="J94" s="9"/>
       <c r="K94" s="9"/>
       <c r="L94" s="101" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="M94" s="103"/>
       <c r="N94" s="103"/>
       <c r="O94" s="60">
         <f>O93/5</f>
-        <v>52.545300000000012</v>
+        <v>52.650300000000001</v>
       </c>
       <c r="P94" s="72"/>
     </row>

</xml_diff>

<commit_message>
#29 Glass Pipe added
</commit_message>
<xml_diff>
--- a/Design Files/Baseboard-v2.0/BOM/Client_BOM_Baseboard-v2.0.xlsx
+++ b/Design Files/Baseboard-v2.0/BOM/Client_BOM_Baseboard-v2.0.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="827" uniqueCount="424">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="835" uniqueCount="426">
   <si>
     <t>Component list</t>
   </si>
@@ -1291,6 +1291,24 @@
   </si>
   <si>
     <t>C20, C25, C48</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">DIA 2mm Light Pipe Plastic LED Light Pipe RoHS Light Pipe Guide PDPLC-2.0-Series </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(PDPLC-2.0-2.54)</t>
+    </r>
+  </si>
+  <si>
+    <t>PDPLC-2.0-2.54</t>
   </si>
 </sst>
 </file>
@@ -1302,7 +1320,7 @@
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0000"/>
     <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="25" x14ac:knownFonts="1">
+  <fonts count="26" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1476,6 +1494,13 @@
       <b/>
       <sz val="9"/>
       <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -2408,7 +2433,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:XFD94"/>
+  <dimension ref="A1:XFD95"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="25" customWidth="1"/>
@@ -22973,7 +22998,7 @@
       </c>
       <c r="P91" s="31"/>
     </row>
-    <row r="92" spans="1:16" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A92" s="1"/>
       <c r="B92" s="61">
         <f>ROW(B92) - ROW($B$9)</f>
@@ -23021,57 +23046,99 @@
       </c>
       <c r="P92" s="97"/>
     </row>
-    <row r="93" spans="1:16" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:16" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A93" s="1"/>
-      <c r="B93" s="65"/>
-      <c r="C93" s="66"/>
-      <c r="D93" s="67"/>
-      <c r="E93" s="68"/>
-      <c r="F93" s="69"/>
-      <c r="G93" s="70"/>
-      <c r="H93" s="70"/>
-      <c r="I93" s="69"/>
-      <c r="J93" s="70"/>
-      <c r="K93" s="70"/>
-      <c r="L93" s="101" t="s">
+      <c r="B93" s="64">
+        <f>ROW(B93) - ROW($B$9)</f>
+        <v>84</v>
+      </c>
+      <c r="C93" s="50" t="s">
+        <v>415</v>
+      </c>
+      <c r="D93" s="51"/>
+      <c r="E93" s="30" t="s">
+        <v>424</v>
+      </c>
+      <c r="F93" s="51" t="s">
+        <v>369</v>
+      </c>
+      <c r="G93" s="51" t="s">
+        <v>425</v>
+      </c>
+      <c r="H93" s="95" t="s">
+        <v>369</v>
+      </c>
+      <c r="I93" s="51" t="s">
+        <v>369</v>
+      </c>
+      <c r="J93" s="30" t="s">
+        <v>369</v>
+      </c>
+      <c r="K93" s="95">
+        <v>1</v>
+      </c>
+      <c r="L93" s="96">
+        <f>K93*5</f>
+        <v>5</v>
+      </c>
+      <c r="M93" s="90" t="s">
+        <v>403</v>
+      </c>
+      <c r="N93" s="80"/>
+      <c r="O93" s="55"/>
+      <c r="P93" s="97"/>
+    </row>
+    <row r="94" spans="1:16" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A94" s="1"/>
+      <c r="B94" s="65"/>
+      <c r="C94" s="66"/>
+      <c r="D94" s="67"/>
+      <c r="E94" s="68"/>
+      <c r="F94" s="69"/>
+      <c r="G94" s="70"/>
+      <c r="H94" s="70"/>
+      <c r="I94" s="69"/>
+      <c r="J94" s="70"/>
+      <c r="K94" s="70"/>
+      <c r="L94" s="101" t="s">
         <v>386</v>
       </c>
-      <c r="M93" s="102"/>
-      <c r="N93" s="103"/>
-      <c r="O93" s="59">
+      <c r="M94" s="102"/>
+      <c r="N94" s="103"/>
+      <c r="O94" s="59">
         <f>SUM(O10:O91)</f>
         <v>263.25150000000002</v>
       </c>
-      <c r="P93" s="71"/>
+      <c r="P94" s="71"/>
     </row>
-    <row r="94" spans="1:16" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B94" s="24"/>
-      <c r="C94" s="38"/>
-      <c r="D94" s="8"/>
-      <c r="E94" s="9"/>
-      <c r="F94" s="9"/>
-      <c r="G94" s="9"/>
-      <c r="H94" s="9"/>
-      <c r="I94" s="9"/>
-      <c r="J94" s="9"/>
-      <c r="K94" s="9"/>
-      <c r="L94" s="101" t="s">
+    <row r="95" spans="1:16" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B95" s="24"/>
+      <c r="C95" s="38"/>
+      <c r="D95" s="8"/>
+      <c r="E95" s="9"/>
+      <c r="F95" s="9"/>
+      <c r="G95" s="9"/>
+      <c r="H95" s="9"/>
+      <c r="I95" s="9"/>
+      <c r="J95" s="9"/>
+      <c r="K95" s="9"/>
+      <c r="L95" s="101" t="s">
         <v>387</v>
       </c>
-      <c r="M94" s="103"/>
-      <c r="N94" s="103"/>
-      <c r="O94" s="60">
-        <f>O93/5</f>
+      <c r="M95" s="103"/>
+      <c r="N95" s="103"/>
+      <c r="O95" s="60">
+        <f>O94/5</f>
         <v>52.650300000000001</v>
       </c>
-      <c r="P94" s="72"/>
+      <c r="P95" s="72"/>
     </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="J1:P1"/>
     <mergeCell ref="P3:P8"/>
-    <mergeCell ref="L93:N93"/>
     <mergeCell ref="L94:N94"/>
+    <mergeCell ref="L95:N95"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="M11" r:id="rId1"/>

</xml_diff>

<commit_message>
#29 Client BOM Final
</commit_message>
<xml_diff>
--- a/Design Files/Baseboard-v2.0/BOM/Client_BOM_Baseboard-v2.0.xlsx
+++ b/Design Files/Baseboard-v2.0/BOM/Client_BOM_Baseboard-v2.0.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="835" uniqueCount="426">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="691" uniqueCount="419">
   <si>
     <t>Component list</t>
   </si>
@@ -1167,24 +1167,9 @@
     <t>Quantity (5 Boards)</t>
   </si>
   <si>
-    <t>Links</t>
-  </si>
-  <si>
-    <t>Unit Cost (5 Boards)</t>
-  </si>
-  <si>
-    <t>Total Cost (5 Boards)</t>
-  </si>
-  <si>
     <t>Remarks</t>
   </si>
   <si>
-    <t xml:space="preserve">Total Component Cost </t>
-  </si>
-  <si>
-    <t>Single Board Cost</t>
-  </si>
-  <si>
     <t>RELAY GEN PURPOSE SPDT 3A 5V</t>
   </si>
   <si>
@@ -1225,12 +1210,6 @@
   </si>
   <si>
     <t>TAE</t>
-  </si>
-  <si>
-    <t>Digikey</t>
-  </si>
-  <si>
-    <t>Custom Supplier</t>
   </si>
   <si>
     <t>CRCW040222R0FKEDHP</t>
@@ -1315,12 +1294,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="3">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
-    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0000"/>
-    <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="26" x14ac:knownFonts="1">
+  <fonts count="24" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1469,21 +1446,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="14"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="9"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1532,7 +1494,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="23">
+  <borders count="21">
     <border>
       <left/>
       <right/>
@@ -1766,36 +1728,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="104">
+  <cellXfs count="82">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1936,27 +1873,6 @@
     <xf numFmtId="0" fontId="17" fillId="2" borderId="16" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="17" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="17" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="17" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="17" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="14" fillId="3" borderId="14" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="14" fillId="3" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2013,52 +1929,16 @@
     <xf numFmtId="0" fontId="17" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="17" fillId="2" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="17" fillId="2" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="17" fillId="2" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="17" fillId="2" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="16" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="16" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="16" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2079,21 +1959,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -2119,13 +1986,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>15</xdr:col>
+      <xdr:col>12</xdr:col>
       <xdr:colOff>47625</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>19942</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
+      <xdr:col>12</xdr:col>
       <xdr:colOff>1905000</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>171450</xdr:rowOff>
@@ -2433,7 +2300,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:XFD95"/>
+  <dimension ref="A1:XFA95"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="25" customWidth="1"/>
@@ -2447,13 +2314,12 @@
     <col min="10" max="10" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="9.28515625" customWidth="1"/>
-    <col min="14" max="14" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="29.42578125" customWidth="1"/>
+    <col min="13" max="13" width="29.42578125" customWidth="1"/>
+    <col min="15" max="15" width="16.85546875" customWidth="1"/>
+    <col min="16" max="16" width="5.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -2463,15 +2329,12 @@
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
-      <c r="J1" s="98"/>
-      <c r="K1" s="98"/>
-      <c r="L1" s="98"/>
-      <c r="M1" s="98"/>
-      <c r="N1" s="98"/>
-      <c r="O1" s="98"/>
-      <c r="P1" s="98"/>
+      <c r="J1" s="79"/>
+      <c r="K1" s="79"/>
+      <c r="L1" s="79"/>
+      <c r="M1" s="79"/>
     </row>
-    <row r="2" spans="1:16" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
       <c r="B2" s="20"/>
       <c r="C2" s="33"/>
@@ -2488,12 +2351,9 @@
       <c r="J2" s="3"/>
       <c r="K2" s="3"/>
       <c r="L2" s="3"/>
-      <c r="M2" s="3"/>
-      <c r="N2" s="3"/>
-      <c r="O2" s="3"/>
-      <c r="P2" s="32"/>
+      <c r="M2" s="32"/>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="21"/>
       <c r="C3" s="34"/>
@@ -2510,12 +2370,9 @@
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
       <c r="L3" s="4"/>
-      <c r="M3" s="4"/>
-      <c r="N3" s="4"/>
-      <c r="O3" s="4"/>
-      <c r="P3" s="99"/>
+      <c r="M3" s="80"/>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="21"/>
       <c r="C4" s="34"/>
@@ -2532,12 +2389,9 @@
       <c r="J4" s="6"/>
       <c r="K4" s="6"/>
       <c r="L4" s="5"/>
-      <c r="M4" s="5"/>
-      <c r="N4" s="5"/>
-      <c r="O4" s="5"/>
-      <c r="P4" s="100"/>
+      <c r="M4" s="81"/>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="21"/>
       <c r="C5" s="34"/>
@@ -2554,12 +2408,9 @@
       <c r="J5" s="5"/>
       <c r="K5" s="5"/>
       <c r="L5" s="5"/>
-      <c r="M5" s="5"/>
-      <c r="N5" s="5"/>
-      <c r="O5" s="5"/>
-      <c r="P5" s="100"/>
+      <c r="M5" s="81"/>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="22"/>
       <c r="C6" s="35"/>
@@ -2572,12 +2423,9 @@
       <c r="J6" s="5"/>
       <c r="K6" s="5"/>
       <c r="L6" s="5"/>
-      <c r="M6" s="5"/>
-      <c r="N6" s="5"/>
-      <c r="O6" s="5"/>
-      <c r="P6" s="100"/>
+      <c r="M6" s="81"/>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
       <c r="B7" s="23"/>
       <c r="C7" s="36"/>
@@ -2590,12 +2438,9 @@
       <c r="J7" s="7"/>
       <c r="K7" s="7"/>
       <c r="L7" s="7"/>
-      <c r="M7" s="7"/>
-      <c r="N7" s="7"/>
-      <c r="O7" s="7"/>
-      <c r="P7" s="100"/>
+      <c r="M7" s="81"/>
     </row>
-    <row r="8" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="B8" s="26"/>
       <c r="C8" s="37"/>
@@ -2608,12 +2453,9 @@
       <c r="J8" s="7"/>
       <c r="K8" s="7"/>
       <c r="L8" s="7"/>
-      <c r="M8" s="7"/>
-      <c r="N8" s="7"/>
-      <c r="O8" s="7"/>
-      <c r="P8" s="100"/>
+      <c r="M8" s="81"/>
     </row>
-    <row r="9" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
       <c r="B9" s="29" t="s">
         <v>4</v>
@@ -2645,25 +2487,16 @@
       <c r="K9" s="29" t="s">
         <v>366</v>
       </c>
-      <c r="L9" s="85" t="s">
+      <c r="L9" s="72" t="s">
         <v>381</v>
       </c>
       <c r="M9" s="29" t="s">
         <v>382</v>
       </c>
-      <c r="N9" s="86" t="s">
-        <v>383</v>
-      </c>
-      <c r="O9" s="29" t="s">
-        <v>384</v>
-      </c>
-      <c r="P9" s="29" t="s">
-        <v>385</v>
-      </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
-      <c r="B10" s="61">
+      <c r="B10" s="54">
         <f>ROW(B10) - ROW($B$9)</f>
         <v>1</v>
       </c>
@@ -2694,24 +2527,17 @@
       <c r="K10" s="44">
         <v>1</v>
       </c>
-      <c r="L10" s="75">
+      <c r="L10" s="68">
         <f>K10*5</f>
         <v>5</v>
       </c>
-      <c r="M10" s="44" t="s">
-        <v>369</v>
-      </c>
-      <c r="N10" s="87" t="s">
-        <v>369</v>
-      </c>
-      <c r="O10" s="52" t="s">
-        <v>369</v>
-      </c>
-      <c r="P10" s="30"/>
+      <c r="M10" s="75" t="s">
+        <v>407</v>
+      </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
-      <c r="B11" s="62">
+      <c r="B11" s="55">
         <f t="shared" ref="B11:B90" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
@@ -2742,25 +2568,15 @@
       <c r="K11" s="31">
         <v>1</v>
       </c>
-      <c r="L11" s="74">
+      <c r="L11" s="67">
         <f t="shared" ref="L11" si="1">K11*5</f>
         <v>5</v>
       </c>
-      <c r="M11" s="54" t="s">
-        <v>402</v>
-      </c>
-      <c r="N11" s="80">
-        <v>0.48</v>
-      </c>
-      <c r="O11" s="55">
-        <f t="shared" ref="O11" si="2">N11*L11</f>
-        <v>2.4</v>
-      </c>
-      <c r="P11" s="31"/>
+      <c r="M11" s="31"/>
     </row>
-    <row r="12" spans="1:16" ht="36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" ht="36" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
-      <c r="B12" s="61">
+      <c r="B12" s="54">
         <f>ROW(B12) - ROW($B$9)</f>
         <v>3</v>
       </c>
@@ -2791,25 +2607,15 @@
       <c r="K12" s="30">
         <v>25</v>
       </c>
-      <c r="L12" s="73">
+      <c r="L12" s="66">
         <f>K12*5</f>
         <v>125</v>
       </c>
-      <c r="M12" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N12" s="79">
-        <v>1.03E-2</v>
-      </c>
-      <c r="O12" s="56">
-        <f>N12*L12</f>
-        <v>1.2875000000000001</v>
-      </c>
-      <c r="P12" s="30"/>
+      <c r="M12" s="30"/>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" s="1"/>
-      <c r="B13" s="62">
+      <c r="B13" s="55">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
@@ -2817,7 +2623,7 @@
         <v>7</v>
       </c>
       <c r="D13" s="31" t="s">
-        <v>422</v>
+        <v>415</v>
       </c>
       <c r="E13" s="31" t="s">
         <v>100</v>
@@ -2840,25 +2646,15 @@
       <c r="K13" s="31">
         <v>2</v>
       </c>
-      <c r="L13" s="74">
-        <f t="shared" ref="L13" si="3">K13*5</f>
+      <c r="L13" s="67">
+        <f t="shared" ref="L13" si="2">K13*5</f>
         <v>10</v>
       </c>
-      <c r="M13" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N13" s="80">
-        <v>1.6E-2</v>
-      </c>
-      <c r="O13" s="55">
-        <f t="shared" ref="O13" si="4">N13*L13</f>
-        <v>0.16</v>
-      </c>
-      <c r="P13" s="31"/>
+      <c r="M13" s="31"/>
     </row>
-    <row r="14" spans="1:16" ht="36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" ht="36" x14ac:dyDescent="0.25">
       <c r="A14" s="1"/>
-      <c r="B14" s="61">
+      <c r="B14" s="54">
         <f>ROW(B14) - ROW($B$9)</f>
         <v>5</v>
       </c>
@@ -2889,24 +2685,15 @@
       <c r="K14" s="30">
         <v>3</v>
       </c>
-      <c r="L14" s="73">
+      <c r="L14" s="66">
         <f>K14*5</f>
         <v>15</v>
       </c>
-      <c r="M14" s="90" t="s">
-        <v>403</v>
-      </c>
-      <c r="N14" s="79" t="s">
-        <v>369</v>
-      </c>
-      <c r="O14" s="56" t="s">
-        <v>369</v>
-      </c>
-      <c r="P14" s="30"/>
+      <c r="M14" s="30"/>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="1"/>
-      <c r="B15" s="62">
+      <c r="B15" s="55">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
@@ -2923,7 +2710,7 @@
         <v>177</v>
       </c>
       <c r="G15" s="31" t="s">
-        <v>405</v>
+        <v>398</v>
       </c>
       <c r="H15" s="31" t="s">
         <v>369</v>
@@ -2937,25 +2724,15 @@
       <c r="K15" s="31">
         <v>2</v>
       </c>
-      <c r="L15" s="74">
-        <f t="shared" ref="L15" si="5">K15*5</f>
+      <c r="L15" s="67">
+        <f t="shared" ref="L15" si="3">K15*5</f>
         <v>10</v>
       </c>
-      <c r="M15" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N15" s="80">
-        <v>0.72599999999999998</v>
-      </c>
-      <c r="O15" s="55">
-        <f t="shared" ref="O15" si="6">N15*L15</f>
-        <v>7.26</v>
-      </c>
-      <c r="P15" s="31"/>
+      <c r="M15" s="31"/>
     </row>
-    <row r="16" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" ht="24" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
-      <c r="B16" s="61">
+      <c r="B16" s="54">
         <f>ROW(B16) - ROW($B$9)</f>
         <v>7</v>
       </c>
@@ -2986,24 +2763,15 @@
       <c r="K16" s="30">
         <v>1</v>
       </c>
-      <c r="L16" s="73">
+      <c r="L16" s="66">
         <f>K16*5</f>
         <v>5</v>
       </c>
-      <c r="M16" s="90" t="s">
-        <v>403</v>
-      </c>
-      <c r="N16" s="79" t="s">
-        <v>369</v>
-      </c>
-      <c r="O16" s="56" t="s">
-        <v>369</v>
-      </c>
-      <c r="P16" s="30"/>
+      <c r="M16" s="30"/>
     </row>
-    <row r="17" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" ht="24" x14ac:dyDescent="0.25">
       <c r="A17" s="1"/>
-      <c r="B17" s="62">
+      <c r="B17" s="55">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
@@ -3034,24 +2802,15 @@
       <c r="K17" s="31">
         <v>1</v>
       </c>
-      <c r="L17" s="74">
-        <f t="shared" ref="L17" si="7">K17*5</f>
+      <c r="L17" s="67">
+        <f t="shared" ref="L17" si="4">K17*5</f>
         <v>5</v>
       </c>
-      <c r="M17" s="90" t="s">
-        <v>403</v>
-      </c>
-      <c r="N17" s="80" t="s">
-        <v>369</v>
-      </c>
-      <c r="O17" s="55" t="s">
-        <v>369</v>
-      </c>
-      <c r="P17" s="31"/>
+      <c r="M17" s="31"/>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" s="1"/>
-      <c r="B18" s="61">
+      <c r="B18" s="54">
         <f>ROW(B18) - ROW($B$9)</f>
         <v>9</v>
       </c>
@@ -3082,25 +2841,15 @@
       <c r="K18" s="30">
         <v>1</v>
       </c>
-      <c r="L18" s="73">
+      <c r="L18" s="66">
         <f>K18*5</f>
         <v>5</v>
       </c>
-      <c r="M18" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N18" s="79">
-        <v>3.42</v>
-      </c>
-      <c r="O18" s="56">
-        <f>N18*L18</f>
-        <v>17.100000000000001</v>
-      </c>
-      <c r="P18" s="30"/>
+      <c r="M18" s="30"/>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" s="1"/>
-      <c r="B19" s="62">
+      <c r="B19" s="55">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
@@ -3131,25 +2880,15 @@
       <c r="K19" s="31">
         <v>1</v>
       </c>
-      <c r="L19" s="74">
-        <f t="shared" ref="L19" si="8">K19*5</f>
+      <c r="L19" s="67">
+        <f t="shared" ref="L19" si="5">K19*5</f>
         <v>5</v>
       </c>
-      <c r="M19" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N19" s="80">
-        <v>0.68</v>
-      </c>
-      <c r="O19" s="55">
-        <f t="shared" ref="O19" si="9">N19*L19</f>
-        <v>3.4000000000000004</v>
-      </c>
-      <c r="P19" s="31"/>
+      <c r="M19" s="31"/>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" s="1"/>
-      <c r="B20" s="61">
+      <c r="B20" s="54">
         <f>ROW(B20) - ROW($B$9)</f>
         <v>11</v>
       </c>
@@ -3180,25 +2919,15 @@
       <c r="K20" s="30">
         <v>4</v>
       </c>
-      <c r="L20" s="73">
+      <c r="L20" s="66">
         <f>K20*5</f>
         <v>20</v>
       </c>
-      <c r="M20" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N20" s="79">
-        <v>6.2E-2</v>
-      </c>
-      <c r="O20" s="56">
-        <f>N20*L20</f>
-        <v>1.24</v>
-      </c>
-      <c r="P20" s="30"/>
+      <c r="M20" s="30"/>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" s="1"/>
-      <c r="B21" s="62">
+      <c r="B21" s="55">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
@@ -3206,7 +2935,7 @@
         <v>7</v>
       </c>
       <c r="D21" s="31" t="s">
-        <v>423</v>
+        <v>416</v>
       </c>
       <c r="E21" s="31" t="s">
         <v>108</v>
@@ -3229,25 +2958,15 @@
       <c r="K21" s="31">
         <v>3</v>
       </c>
-      <c r="L21" s="74">
-        <f t="shared" ref="L21" si="10">K21*5</f>
+      <c r="L21" s="67">
+        <f t="shared" ref="L21" si="6">K21*5</f>
         <v>15</v>
       </c>
-      <c r="M21" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N21" s="80">
-        <v>0.121</v>
-      </c>
-      <c r="O21" s="55">
-        <f t="shared" ref="O21" si="11">N21*L21</f>
-        <v>1.8149999999999999</v>
-      </c>
-      <c r="P21" s="31"/>
+      <c r="M21" s="31"/>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>
-      <c r="B22" s="61">
+      <c r="B22" s="54">
         <f>ROW(B22) - ROW($B$9)</f>
         <v>13</v>
       </c>
@@ -3278,25 +2997,15 @@
       <c r="K22" s="30">
         <v>2</v>
       </c>
-      <c r="L22" s="73">
+      <c r="L22" s="66">
         <f>K22*5</f>
         <v>10</v>
       </c>
-      <c r="M22" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N22" s="79">
-        <v>1.9E-2</v>
-      </c>
-      <c r="O22" s="56">
-        <f>N22*L22</f>
-        <v>0.19</v>
-      </c>
-      <c r="P22" s="30"/>
+      <c r="M22" s="30"/>
     </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
-      <c r="B23" s="62">
+      <c r="B23" s="55">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
@@ -3327,25 +3036,15 @@
       <c r="K23" s="31">
         <v>3</v>
       </c>
-      <c r="L23" s="74">
-        <f t="shared" ref="L23" si="12">K23*5</f>
+      <c r="L23" s="67">
+        <f t="shared" ref="L23" si="7">K23*5</f>
         <v>15</v>
       </c>
-      <c r="M23" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N23" s="80">
-        <v>7.3999999999999996E-2</v>
-      </c>
-      <c r="O23" s="55">
-        <f t="shared" ref="O23" si="13">N23*L23</f>
-        <v>1.1099999999999999</v>
-      </c>
-      <c r="P23" s="31"/>
+      <c r="M23" s="31"/>
     </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" s="1"/>
-      <c r="B24" s="61">
+      <c r="B24" s="54">
         <f>ROW(B24) - ROW($B$9)</f>
         <v>15</v>
       </c>
@@ -3376,25 +3075,15 @@
       <c r="K24" s="30">
         <v>1</v>
       </c>
-      <c r="L24" s="73">
+      <c r="L24" s="66">
         <f>K24*5</f>
         <v>5</v>
       </c>
-      <c r="M24" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N24" s="79">
-        <v>0.44</v>
-      </c>
-      <c r="O24" s="56">
-        <f>N24*L24</f>
-        <v>2.2000000000000002</v>
-      </c>
-      <c r="P24" s="30"/>
+      <c r="M24" s="30"/>
     </row>
-    <row r="25" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:13" ht="24" x14ac:dyDescent="0.25">
       <c r="A25" s="1"/>
-      <c r="B25" s="62">
+      <c r="B25" s="55">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
@@ -3425,22 +3114,15 @@
       <c r="K25" s="31">
         <v>1</v>
       </c>
-      <c r="L25" s="74">
-        <f t="shared" ref="L25" si="14">K25*5</f>
+      <c r="L25" s="67">
+        <f t="shared" ref="L25" si="8">K25*5</f>
         <v>5</v>
       </c>
-      <c r="M25" s="90" t="s">
-        <v>403</v>
-      </c>
-      <c r="N25" s="80"/>
-      <c r="O25" s="55" t="s">
-        <v>369</v>
-      </c>
-      <c r="P25" s="31"/>
+      <c r="M25" s="31"/>
     </row>
-    <row r="26" spans="1:16" ht="36" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:13" ht="36" x14ac:dyDescent="0.25">
       <c r="A26" s="1"/>
-      <c r="B26" s="61">
+      <c r="B26" s="54">
         <f>ROW(B26) - ROW($B$9)</f>
         <v>17</v>
       </c>
@@ -3471,22 +3153,15 @@
       <c r="K26" s="30">
         <v>1</v>
       </c>
-      <c r="L26" s="73">
+      <c r="L26" s="66">
         <f>K26*5</f>
         <v>5</v>
       </c>
-      <c r="M26" s="90" t="s">
-        <v>403</v>
-      </c>
-      <c r="N26" s="79"/>
-      <c r="O26" s="56" t="s">
-        <v>369</v>
-      </c>
-      <c r="P26" s="30"/>
+      <c r="M26" s="30"/>
     </row>
-    <row r="27" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:13" ht="24" x14ac:dyDescent="0.25">
       <c r="A27" s="1"/>
-      <c r="B27" s="62">
+      <c r="B27" s="55">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
@@ -3517,22 +3192,15 @@
       <c r="K27" s="31">
         <v>1</v>
       </c>
-      <c r="L27" s="74">
-        <f t="shared" ref="L27" si="15">K27*5</f>
+      <c r="L27" s="67">
+        <f t="shared" ref="L27" si="9">K27*5</f>
         <v>5</v>
       </c>
-      <c r="M27" s="90" t="s">
-        <v>403</v>
-      </c>
-      <c r="N27" s="80"/>
-      <c r="O27" s="55" t="s">
-        <v>369</v>
-      </c>
-      <c r="P27" s="31"/>
+      <c r="M27" s="31"/>
     </row>
-    <row r="28" spans="1:16" ht="24" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:13" ht="24" x14ac:dyDescent="0.25">
       <c r="A28" s="1"/>
-      <c r="B28" s="61">
+      <c r="B28" s="54">
         <f>ROW(B28) - ROW($B$9)</f>
         <v>19</v>
       </c>
@@ -3563,25 +3231,15 @@
       <c r="K28" s="30">
         <v>3</v>
       </c>
-      <c r="L28" s="73">
+      <c r="L28" s="66">
         <f>K28*5</f>
         <v>15</v>
       </c>
-      <c r="M28" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N28" s="79">
-        <v>0.184</v>
-      </c>
-      <c r="O28" s="56">
-        <f>N28*L28</f>
-        <v>2.76</v>
-      </c>
-      <c r="P28" s="30"/>
+      <c r="M28" s="30"/>
     </row>
-    <row r="29" spans="1:16" ht="36" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:13" ht="36" x14ac:dyDescent="0.25">
       <c r="A29" s="1"/>
-      <c r="B29" s="62">
+      <c r="B29" s="55">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
@@ -3612,22 +3270,15 @@
       <c r="K29" s="31">
         <v>2</v>
       </c>
-      <c r="L29" s="74">
-        <f t="shared" ref="L29" si="16">K29*5</f>
+      <c r="L29" s="67">
+        <f t="shared" ref="L29" si="10">K29*5</f>
         <v>10</v>
       </c>
-      <c r="M29" s="90" t="s">
-        <v>403</v>
-      </c>
-      <c r="N29" s="80"/>
-      <c r="O29" s="55" t="s">
-        <v>369</v>
-      </c>
-      <c r="P29" s="31"/>
+      <c r="M29" s="31"/>
     </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" s="1"/>
-      <c r="B30" s="61">
+      <c r="B30" s="54">
         <f>ROW(B30) - ROW($B$9)</f>
         <v>21</v>
       </c>
@@ -3658,25 +3309,15 @@
       <c r="K30" s="30">
         <v>4</v>
       </c>
-      <c r="L30" s="73">
+      <c r="L30" s="66">
         <f>K30*5</f>
         <v>20</v>
       </c>
-      <c r="M30" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N30" s="79">
-        <v>0.32300000000000001</v>
-      </c>
-      <c r="O30" s="56">
-        <f>N30*L30</f>
-        <v>6.46</v>
-      </c>
-      <c r="P30" s="30"/>
+      <c r="M30" s="30"/>
     </row>
-    <row r="31" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" s="1"/>
-      <c r="B31" s="62">
+      <c r="B31" s="55">
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
@@ -3707,22 +3348,15 @@
       <c r="K31" s="31">
         <v>4</v>
       </c>
-      <c r="L31" s="74">
-        <f t="shared" ref="L31" si="17">K31*5</f>
+      <c r="L31" s="67">
+        <f t="shared" ref="L31" si="11">K31*5</f>
         <v>20</v>
       </c>
-      <c r="M31" s="90" t="s">
-        <v>403</v>
-      </c>
-      <c r="N31" s="80"/>
-      <c r="O31" s="55" t="s">
-        <v>369</v>
-      </c>
-      <c r="P31" s="31"/>
+      <c r="M31" s="31"/>
     </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" s="1"/>
-      <c r="B32" s="61">
+      <c r="B32" s="54">
         <f>ROW(B32) - ROW($B$9)</f>
         <v>23</v>
       </c>
@@ -3753,25 +3387,15 @@
       <c r="K32" s="30">
         <v>1</v>
       </c>
-      <c r="L32" s="73">
+      <c r="L32" s="66">
         <f>K32*5</f>
         <v>5</v>
       </c>
-      <c r="M32" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N32" s="79">
-        <v>1.766</v>
-      </c>
-      <c r="O32" s="56">
-        <f>N32*L32</f>
-        <v>8.83</v>
-      </c>
-      <c r="P32" s="30"/>
+      <c r="M32" s="30"/>
     </row>
-    <row r="33" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:13" ht="24" x14ac:dyDescent="0.25">
       <c r="A33" s="1"/>
-      <c r="B33" s="62">
+      <c r="B33" s="55">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
@@ -3802,22 +3426,15 @@
       <c r="K33" s="31">
         <v>1</v>
       </c>
-      <c r="L33" s="74">
-        <f t="shared" ref="L33" si="18">K33*5</f>
+      <c r="L33" s="67">
+        <f t="shared" ref="L33" si="12">K33*5</f>
         <v>5</v>
       </c>
-      <c r="M33" s="90" t="s">
-        <v>403</v>
-      </c>
-      <c r="N33" s="80"/>
-      <c r="O33" s="55" t="s">
-        <v>369</v>
-      </c>
-      <c r="P33" s="31"/>
+      <c r="M33" s="31"/>
     </row>
-    <row r="34" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:13" ht="24" x14ac:dyDescent="0.25">
       <c r="A34" s="1"/>
-      <c r="B34" s="61">
+      <c r="B34" s="54">
         <f>ROW(B34) - ROW($B$9)</f>
         <v>25</v>
       </c>
@@ -3848,22 +3465,15 @@
       <c r="K34" s="30">
         <v>4</v>
       </c>
-      <c r="L34" s="73">
+      <c r="L34" s="66">
         <f>K34*5</f>
         <v>20</v>
       </c>
-      <c r="M34" s="90" t="s">
-        <v>403</v>
-      </c>
-      <c r="N34" s="79"/>
-      <c r="O34" s="56" t="s">
-        <v>369</v>
-      </c>
-      <c r="P34" s="30"/>
+      <c r="M34" s="30"/>
     </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A35" s="1"/>
-      <c r="B35" s="62">
+      <c r="B35" s="55">
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
@@ -3894,25 +3504,15 @@
       <c r="K35" s="31">
         <v>1</v>
       </c>
-      <c r="L35" s="74">
-        <f t="shared" ref="L35" si="19">K35*5</f>
+      <c r="L35" s="67">
+        <f t="shared" ref="L35" si="13">K35*5</f>
         <v>5</v>
       </c>
-      <c r="M35" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N35" s="80">
-        <v>0.28000000000000003</v>
-      </c>
-      <c r="O35" s="55">
-        <f t="shared" ref="O35" si="20">N35*L35</f>
-        <v>1.4000000000000001</v>
-      </c>
-      <c r="P35" s="31"/>
+      <c r="M35" s="31"/>
     </row>
-    <row r="36" spans="1:16" ht="48" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:13" ht="48" x14ac:dyDescent="0.25">
       <c r="A36" s="1"/>
-      <c r="B36" s="61">
+      <c r="B36" s="54">
         <f>ROW(B36) - ROW($B$9)</f>
         <v>27</v>
       </c>
@@ -3943,24 +3543,15 @@
       <c r="K36" s="30">
         <v>8</v>
       </c>
-      <c r="L36" s="73">
+      <c r="L36" s="66">
         <f>K36*5</f>
         <v>40</v>
       </c>
-      <c r="M36" s="90" t="s">
-        <v>403</v>
-      </c>
-      <c r="N36" s="79" t="s">
-        <v>369</v>
-      </c>
-      <c r="O36" s="56" t="s">
-        <v>369</v>
-      </c>
-      <c r="P36" s="30"/>
+      <c r="M36" s="30"/>
     </row>
-    <row r="37" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:13" ht="24" x14ac:dyDescent="0.25">
       <c r="A37" s="1"/>
-      <c r="B37" s="62">
+      <c r="B37" s="55">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
@@ -3991,24 +3582,15 @@
       <c r="K37" s="31">
         <v>1</v>
       </c>
-      <c r="L37" s="74">
-        <f t="shared" ref="L37" si="21">K37*5</f>
+      <c r="L37" s="67">
+        <f t="shared" ref="L37" si="14">K37*5</f>
         <v>5</v>
       </c>
-      <c r="M37" s="90" t="s">
-        <v>403</v>
-      </c>
-      <c r="N37" s="80" t="s">
-        <v>369</v>
-      </c>
-      <c r="O37" s="55" t="s">
-        <v>369</v>
-      </c>
-      <c r="P37" s="31"/>
+      <c r="M37" s="31"/>
     </row>
-    <row r="38" spans="1:16" ht="48" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:13" ht="48" x14ac:dyDescent="0.25">
       <c r="A38" s="1"/>
-      <c r="B38" s="61">
+      <c r="B38" s="54">
         <f>ROW(B38) - ROW($B$9)</f>
         <v>29</v>
       </c>
@@ -4039,47 +3621,38 @@
       <c r="K38" s="30">
         <v>4</v>
       </c>
-      <c r="L38" s="73">
+      <c r="L38" s="66">
         <f>K38*5</f>
         <v>20</v>
       </c>
-      <c r="M38" s="90" t="s">
-        <v>403</v>
-      </c>
-      <c r="N38" s="79" t="s">
-        <v>369</v>
-      </c>
-      <c r="O38" s="56" t="s">
-        <v>369</v>
-      </c>
-      <c r="P38" s="30"/>
+      <c r="M38" s="30"/>
     </row>
-    <row r="39" spans="1:16" ht="48" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:13" ht="48" x14ac:dyDescent="0.25">
       <c r="A39" s="1"/>
-      <c r="B39" s="62">
+      <c r="B39" s="55">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
       <c r="C39" s="45" t="s">
-        <v>406</v>
-      </c>
-      <c r="D39" s="92" t="s">
+        <v>399</v>
+      </c>
+      <c r="D39" s="74" t="s">
         <v>51</v>
       </c>
       <c r="E39" s="31" t="s">
-        <v>407</v>
+        <v>400</v>
       </c>
       <c r="F39" s="31" t="s">
         <v>370</v>
       </c>
       <c r="G39" s="31" t="s">
-        <v>408</v>
+        <v>401</v>
       </c>
       <c r="H39" s="31" t="s">
         <v>369</v>
       </c>
       <c r="I39" s="31" t="s">
-        <v>409</v>
+        <v>402</v>
       </c>
       <c r="J39" s="31" t="s">
         <v>369</v>
@@ -4087,24 +3660,15 @@
       <c r="K39" s="31">
         <v>1</v>
       </c>
-      <c r="L39" s="74">
-        <f t="shared" ref="L39" si="22">K39*5</f>
+      <c r="L39" s="67">
+        <f t="shared" ref="L39" si="15">K39*5</f>
         <v>5</v>
       </c>
-      <c r="M39" s="90" t="s">
-        <v>403</v>
-      </c>
-      <c r="N39" s="79" t="s">
-        <v>369</v>
-      </c>
-      <c r="O39" s="56" t="s">
-        <v>369</v>
-      </c>
-      <c r="P39" s="31"/>
+      <c r="M39" s="31"/>
     </row>
-    <row r="40" spans="1:16" ht="36" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:13" ht="36" x14ac:dyDescent="0.25">
       <c r="A40" s="1"/>
-      <c r="B40" s="61">
+      <c r="B40" s="54">
         <f>ROW(B40) - ROW($B$9)</f>
         <v>31</v>
       </c>
@@ -4135,41 +3699,32 @@
       <c r="K40" s="30">
         <v>1</v>
       </c>
-      <c r="L40" s="73">
+      <c r="L40" s="66">
         <f>K40*5</f>
         <v>5</v>
       </c>
-      <c r="M40" s="90" t="s">
-        <v>403</v>
-      </c>
-      <c r="N40" s="79" t="s">
-        <v>369</v>
-      </c>
-      <c r="O40" s="56" t="s">
-        <v>369</v>
-      </c>
-      <c r="P40" s="30"/>
+      <c r="M40" s="30"/>
     </row>
-    <row r="41" spans="1:16" ht="36" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:13" ht="36" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
-      <c r="B41" s="62">
+      <c r="B41" s="55">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
       <c r="C41" s="45" t="s">
-        <v>419</v>
+        <v>412</v>
       </c>
       <c r="D41" s="31" t="s">
         <v>53</v>
       </c>
       <c r="E41" s="31" t="s">
-        <v>420</v>
+        <v>413</v>
       </c>
       <c r="F41" s="31" t="s">
         <v>370</v>
       </c>
       <c r="G41" s="31" t="s">
-        <v>421</v>
+        <v>414</v>
       </c>
       <c r="H41" s="31"/>
       <c r="I41" s="31" t="s">
@@ -4181,24 +3736,15 @@
       <c r="K41" s="31">
         <v>1</v>
       </c>
-      <c r="L41" s="74">
-        <f t="shared" ref="L41" si="23">K41*5</f>
+      <c r="L41" s="67">
+        <f t="shared" ref="L41" si="16">K41*5</f>
         <v>5</v>
       </c>
-      <c r="M41" s="90" t="s">
-        <v>403</v>
-      </c>
-      <c r="N41" s="80" t="s">
-        <v>369</v>
-      </c>
-      <c r="O41" s="55" t="s">
-        <v>369</v>
-      </c>
-      <c r="P41" s="31"/>
+      <c r="M41" s="31"/>
     </row>
-    <row r="42" spans="1:16" ht="36" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:13" ht="36" x14ac:dyDescent="0.25">
       <c r="A42" s="1"/>
-      <c r="B42" s="61">
+      <c r="B42" s="54">
         <f>ROW(B42) - ROW($B$9)</f>
         <v>33</v>
       </c>
@@ -4229,24 +3775,15 @@
       <c r="K42" s="30">
         <v>2</v>
       </c>
-      <c r="L42" s="73">
+      <c r="L42" s="66">
         <f>K42*5</f>
         <v>10</v>
       </c>
-      <c r="M42" s="90" t="s">
-        <v>403</v>
-      </c>
-      <c r="N42" s="79" t="s">
-        <v>369</v>
-      </c>
-      <c r="O42" s="56" t="s">
-        <v>369</v>
-      </c>
-      <c r="P42" s="30"/>
+      <c r="M42" s="30"/>
     </row>
-    <row r="43" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A43" s="1"/>
-      <c r="B43" s="62">
+      <c r="B43" s="55">
         <f t="shared" si="0"/>
         <v>34</v>
       </c>
@@ -4257,19 +3794,19 @@
         <v>55</v>
       </c>
       <c r="E43" s="31" t="s">
-        <v>388</v>
+        <v>383</v>
       </c>
       <c r="F43" s="31" t="s">
         <v>370</v>
       </c>
       <c r="G43" s="31" t="s">
-        <v>389</v>
+        <v>384</v>
       </c>
       <c r="H43" s="31" t="s">
         <v>369</v>
       </c>
       <c r="I43" s="31" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
       <c r="J43" s="31" t="s">
         <v>369</v>
@@ -4277,25 +3814,15 @@
       <c r="K43" s="31">
         <v>3</v>
       </c>
-      <c r="L43" s="74">
-        <f t="shared" ref="L43" si="24">K43*5</f>
+      <c r="L43" s="67">
+        <f t="shared" ref="L43" si="17">K43*5</f>
         <v>15</v>
       </c>
-      <c r="M43" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N43" s="80">
-        <v>0.90900000000000003</v>
-      </c>
-      <c r="O43" s="55">
-        <f t="shared" ref="O43" si="25">N43*L43</f>
-        <v>13.635</v>
-      </c>
-      <c r="P43" s="31"/>
+      <c r="M43" s="31"/>
     </row>
-    <row r="44" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:13" ht="24" x14ac:dyDescent="0.25">
       <c r="A44" s="1"/>
-      <c r="B44" s="61">
+      <c r="B44" s="54">
         <f>ROW(B44) - ROW($B$9)</f>
         <v>35</v>
       </c>
@@ -4326,24 +3853,15 @@
       <c r="K44" s="30">
         <v>1</v>
       </c>
-      <c r="L44" s="73">
+      <c r="L44" s="66">
         <f>K44*5</f>
         <v>5</v>
       </c>
-      <c r="M44" s="90" t="s">
-        <v>403</v>
-      </c>
-      <c r="N44" s="79" t="s">
-        <v>369</v>
-      </c>
-      <c r="O44" s="56" t="s">
-        <v>369</v>
-      </c>
-      <c r="P44" s="30"/>
+      <c r="M44" s="30"/>
     </row>
-    <row r="45" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A45" s="1"/>
-      <c r="B45" s="62">
+      <c r="B45" s="55">
         <f t="shared" si="0"/>
         <v>36</v>
       </c>
@@ -4374,24 +3892,15 @@
       <c r="K45" s="31">
         <v>1</v>
       </c>
-      <c r="L45" s="74">
-        <f t="shared" ref="L45" si="26">K45*5</f>
+      <c r="L45" s="67">
+        <f t="shared" ref="L45" si="18">K45*5</f>
         <v>5</v>
       </c>
-      <c r="M45" s="90" t="s">
-        <v>403</v>
-      </c>
-      <c r="N45" s="80" t="s">
-        <v>369</v>
-      </c>
-      <c r="O45" s="55" t="s">
-        <v>369</v>
-      </c>
-      <c r="P45" s="31"/>
+      <c r="M45" s="31"/>
     </row>
-    <row r="46" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:13" ht="24" x14ac:dyDescent="0.25">
       <c r="A46" s="1"/>
-      <c r="B46" s="61">
+      <c r="B46" s="54">
         <f>ROW(B46) - ROW($B$9)</f>
         <v>37</v>
       </c>
@@ -4422,24 +3931,15 @@
       <c r="K46" s="30">
         <v>2</v>
       </c>
-      <c r="L46" s="73">
+      <c r="L46" s="66">
         <f>K46*5</f>
         <v>10</v>
       </c>
-      <c r="M46" s="90" t="s">
-        <v>403</v>
-      </c>
-      <c r="N46" s="79" t="s">
-        <v>369</v>
-      </c>
-      <c r="O46" s="79" t="s">
-        <v>369</v>
-      </c>
-      <c r="P46" s="30"/>
+      <c r="M46" s="30"/>
     </row>
-    <row r="47" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:13" ht="24" x14ac:dyDescent="0.25">
       <c r="A47" s="1"/>
-      <c r="B47" s="62">
+      <c r="B47" s="55">
         <f t="shared" si="0"/>
         <v>38</v>
       </c>
@@ -4470,24 +3970,15 @@
       <c r="K47" s="31">
         <v>1</v>
       </c>
-      <c r="L47" s="74">
-        <f t="shared" ref="L47" si="27">K47*5</f>
+      <c r="L47" s="67">
+        <f t="shared" ref="L47" si="19">K47*5</f>
         <v>5</v>
       </c>
-      <c r="M47" s="90" t="s">
-        <v>403</v>
-      </c>
-      <c r="N47" s="80" t="s">
-        <v>369</v>
-      </c>
-      <c r="O47" s="80" t="s">
-        <v>369</v>
-      </c>
-      <c r="P47" s="31"/>
+      <c r="M47" s="31"/>
     </row>
-    <row r="48" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A48" s="1"/>
-      <c r="B48" s="61">
+      <c r="B48" s="54">
         <f>ROW(B48) - ROW($B$9)</f>
         <v>39</v>
       </c>
@@ -4518,24 +4009,17 @@
       <c r="K48" s="44">
         <v>10</v>
       </c>
-      <c r="L48" s="75">
+      <c r="L48" s="68">
         <f>K48*5</f>
         <v>50</v>
       </c>
-      <c r="M48" s="88" t="s">
-        <v>369</v>
-      </c>
-      <c r="N48" s="81" t="s">
-        <v>369</v>
-      </c>
-      <c r="O48" s="44" t="s">
-        <v>369</v>
-      </c>
-      <c r="P48" s="30"/>
+      <c r="M48" s="75" t="s">
+        <v>407</v>
+      </c>
     </row>
-    <row r="49" spans="1:16384" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:16381" x14ac:dyDescent="0.25">
       <c r="A49" s="1"/>
-      <c r="B49" s="62">
+      <c r="B49" s="55">
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
@@ -4566,25 +4050,15 @@
       <c r="K49" s="31">
         <v>1</v>
       </c>
-      <c r="L49" s="74">
-        <f t="shared" ref="L49" si="28">K49*5</f>
+      <c r="L49" s="67">
+        <f t="shared" ref="L49" si="20">K49*5</f>
         <v>5</v>
       </c>
-      <c r="M49" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N49" s="80">
-        <v>0.14000000000000001</v>
-      </c>
-      <c r="O49" s="55">
-        <f t="shared" ref="O49" si="29">N49*L49</f>
-        <v>0.70000000000000007</v>
-      </c>
-      <c r="P49" s="31"/>
+      <c r="M49" s="31"/>
     </row>
-    <row r="50" spans="1:16384" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:16381" x14ac:dyDescent="0.25">
       <c r="A50" s="1"/>
-      <c r="B50" s="61">
+      <c r="B50" s="54">
         <f>ROW(B50) - ROW($B$9)</f>
         <v>41</v>
       </c>
@@ -4615,25 +4089,15 @@
       <c r="K50" s="30">
         <v>2</v>
       </c>
-      <c r="L50" s="73">
+      <c r="L50" s="66">
         <f>K50*5</f>
         <v>10</v>
       </c>
-      <c r="M50" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N50" s="79">
-        <v>0.33600000000000002</v>
-      </c>
-      <c r="O50" s="56">
-        <f>N50*L50</f>
-        <v>3.3600000000000003</v>
-      </c>
-      <c r="P50" s="30"/>
+      <c r="M50" s="30"/>
     </row>
-    <row r="51" spans="1:16384" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:16381" x14ac:dyDescent="0.25">
       <c r="A51" s="1"/>
-      <c r="B51" s="62">
+      <c r="B51" s="55">
         <f t="shared" si="0"/>
         <v>42</v>
       </c>
@@ -4664,26 +4128,17 @@
       <c r="K51" s="31">
         <v>1</v>
       </c>
-      <c r="L51" s="74">
-        <f t="shared" ref="L51" si="30">K51*5</f>
+      <c r="L51" s="67">
+        <f t="shared" ref="L51" si="21">K51*5</f>
         <v>5</v>
       </c>
-      <c r="M51" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N51" s="80" t="s">
-        <v>369</v>
-      </c>
-      <c r="O51" s="55" t="s">
-        <v>369</v>
-      </c>
-      <c r="P51" s="94" t="s">
-        <v>414</v>
+      <c r="M51" s="75" t="s">
+        <v>407</v>
       </c>
     </row>
-    <row r="52" spans="1:16384" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:16381" x14ac:dyDescent="0.25">
       <c r="A52" s="1"/>
-      <c r="B52" s="61">
+      <c r="B52" s="54">
         <f>ROW(B52) - ROW($B$9)</f>
         <v>43</v>
       </c>
@@ -4714,25 +4169,15 @@
       <c r="K52" s="30">
         <v>1</v>
       </c>
-      <c r="L52" s="73">
+      <c r="L52" s="66">
         <f>K52*5</f>
         <v>5</v>
       </c>
-      <c r="M52" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N52" s="79">
-        <v>0.1</v>
-      </c>
-      <c r="O52" s="56">
-        <f>N52*L52</f>
-        <v>0.5</v>
-      </c>
-      <c r="P52" s="30"/>
+      <c r="M52" s="30"/>
     </row>
-    <row r="53" spans="1:16384" ht="24" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:16381" ht="24" x14ac:dyDescent="0.25">
       <c r="A53" s="1"/>
-      <c r="B53" s="62">
+      <c r="B53" s="55">
         <f t="shared" si="0"/>
         <v>44</v>
       </c>
@@ -4740,7 +4185,7 @@
         <v>17</v>
       </c>
       <c r="D53" s="31" t="s">
-        <v>390</v>
+        <v>385</v>
       </c>
       <c r="E53" s="31" t="s">
         <v>137</v>
@@ -4763,33 +4208,23 @@
       <c r="K53" s="31">
         <v>12</v>
       </c>
-      <c r="L53" s="74">
-        <f t="shared" ref="L53" si="31">K53*5</f>
+      <c r="L53" s="67">
+        <f t="shared" ref="L53" si="22">K53*5</f>
         <v>60</v>
       </c>
-      <c r="M53" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N53" s="80">
-        <v>1.6199999999999999E-2</v>
-      </c>
-      <c r="O53" s="55">
-        <f t="shared" ref="O53" si="32">N53*L53</f>
-        <v>0.97199999999999998</v>
-      </c>
-      <c r="P53" s="31"/>
+      <c r="M53" s="31"/>
     </row>
-    <row r="54" spans="1:16384" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:16381" x14ac:dyDescent="0.25">
       <c r="A54" s="1"/>
-      <c r="B54" s="61">
+      <c r="B54" s="54">
         <f>ROW(B54) - ROW($B$9)</f>
         <v>45</v>
       </c>
       <c r="C54" s="45" t="s">
         <v>17</v>
       </c>
-      <c r="D54" s="91" t="s">
-        <v>410</v>
+      <c r="D54" s="73" t="s">
+        <v>403</v>
       </c>
       <c r="E54" s="30" t="s">
         <v>138</v>
@@ -4812,25 +4247,15 @@
       <c r="K54" s="30">
         <v>8</v>
       </c>
-      <c r="L54" s="73">
+      <c r="L54" s="66">
         <f>K54*5</f>
         <v>40</v>
       </c>
-      <c r="M54" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N54" s="79">
-        <v>2.5999999999999999E-2</v>
-      </c>
-      <c r="O54" s="56">
-        <f>N54*L54</f>
-        <v>1.04</v>
-      </c>
-      <c r="P54" s="30"/>
+      <c r="M54" s="30"/>
     </row>
-    <row r="55" spans="1:16384" ht="36" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:16381" ht="36" x14ac:dyDescent="0.25">
       <c r="A55" s="1"/>
-      <c r="B55" s="62">
+      <c r="B55" s="55">
         <f t="shared" si="0"/>
         <v>46</v>
       </c>
@@ -4861,24 +4286,15 @@
       <c r="K55" s="31">
         <v>1</v>
       </c>
-      <c r="L55" s="74">
-        <f t="shared" ref="L55" si="33">K55*5</f>
+      <c r="L55" s="67">
+        <f t="shared" ref="L55" si="23">K55*5</f>
         <v>5</v>
       </c>
-      <c r="M55" s="90" t="s">
-        <v>403</v>
-      </c>
-      <c r="N55" s="80" t="s">
-        <v>369</v>
-      </c>
-      <c r="O55" s="55" t="s">
-        <v>369</v>
-      </c>
-      <c r="P55" s="31"/>
+      <c r="M55" s="31"/>
     </row>
-    <row r="56" spans="1:16384" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:16381" x14ac:dyDescent="0.25">
       <c r="A56" s="1"/>
-      <c r="B56" s="61">
+      <c r="B56" s="54">
         <f>ROW(B56) - ROW($B$9)</f>
         <v>47</v>
       </c>
@@ -4909,25 +4325,15 @@
       <c r="K56" s="30">
         <v>2</v>
       </c>
-      <c r="L56" s="73">
+      <c r="L56" s="66">
         <f>K56*5</f>
         <v>10</v>
       </c>
-      <c r="M56" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N56" s="79">
-        <v>0.02</v>
-      </c>
-      <c r="O56" s="56">
-        <f>N56*L56</f>
-        <v>0.2</v>
-      </c>
-      <c r="P56" s="30"/>
+      <c r="M56" s="30"/>
     </row>
-    <row r="57" spans="1:16384" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:16381" x14ac:dyDescent="0.25">
       <c r="A57" s="1"/>
-      <c r="B57" s="62">
+      <c r="B57" s="55">
         <f t="shared" si="0"/>
         <v>48</v>
       </c>
@@ -4935,7 +4341,7 @@
         <v>17</v>
       </c>
       <c r="D57" s="31" t="s">
-        <v>391</v>
+        <v>386</v>
       </c>
       <c r="E57" s="31" t="s">
         <v>141</v>
@@ -4943,7 +4349,7 @@
       <c r="F57" s="31" t="s">
         <v>203</v>
       </c>
-      <c r="G57" s="91" t="s">
+      <c r="G57" s="73" t="s">
         <v>255</v>
       </c>
       <c r="H57" s="31" t="s">
@@ -4958,25 +4364,15 @@
       <c r="K57" s="31">
         <v>2</v>
       </c>
-      <c r="L57" s="74">
-        <f t="shared" ref="L57" si="34">K57*5</f>
+      <c r="L57" s="67">
+        <f t="shared" ref="L57" si="24">K57*5</f>
         <v>10</v>
       </c>
-      <c r="M57" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N57" s="80">
-        <v>0.02</v>
-      </c>
-      <c r="O57" s="55">
-        <f t="shared" ref="O57" si="35">N57*L57</f>
-        <v>0.2</v>
-      </c>
-      <c r="P57" s="31"/>
+      <c r="M57" s="31"/>
     </row>
-    <row r="58" spans="1:16384" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:16381" x14ac:dyDescent="0.25">
       <c r="A58" s="1"/>
-      <c r="B58" s="61">
+      <c r="B58" s="54">
         <f>ROW(B58) - ROW($B$9)</f>
         <v>49</v>
       </c>
@@ -5007,25 +4403,15 @@
       <c r="K58" s="30">
         <v>2</v>
       </c>
-      <c r="L58" s="73">
+      <c r="L58" s="66">
         <f>K58*5</f>
         <v>10</v>
       </c>
-      <c r="M58" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N58" s="79">
-        <v>1.4E-2</v>
-      </c>
-      <c r="O58" s="56">
-        <f>N58*L58</f>
-        <v>0.14000000000000001</v>
-      </c>
-      <c r="P58" s="30"/>
+      <c r="M58" s="30"/>
     </row>
-    <row r="59" spans="1:16384" ht="36" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:16381" ht="36" x14ac:dyDescent="0.25">
       <c r="A59" s="1"/>
-      <c r="B59" s="62">
+      <c r="B59" s="55">
         <f t="shared" si="0"/>
         <v>50</v>
       </c>
@@ -5056,25 +4442,15 @@
       <c r="K59" s="31">
         <v>22</v>
       </c>
-      <c r="L59" s="74">
-        <f t="shared" ref="L59" si="36">K59*5</f>
+      <c r="L59" s="67">
+        <f t="shared" ref="L59" si="25">K59*5</f>
         <v>110</v>
       </c>
-      <c r="M59" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N59" s="80">
-        <v>7.0000000000000001E-3</v>
-      </c>
-      <c r="O59" s="55">
-        <f t="shared" ref="O59" si="37">N59*L59</f>
-        <v>0.77</v>
-      </c>
-      <c r="P59" s="31"/>
+      <c r="M59" s="31"/>
     </row>
-    <row r="60" spans="1:16384" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:16381" x14ac:dyDescent="0.25">
       <c r="A60" s="1"/>
-      <c r="B60" s="61">
+      <c r="B60" s="54">
         <f>ROW(B60) - ROW($B$9)</f>
         <v>51</v>
       </c>
@@ -5105,25 +4481,15 @@
       <c r="K60" s="30">
         <v>1</v>
       </c>
-      <c r="L60" s="73">
+      <c r="L60" s="66">
         <f>K60*5</f>
         <v>5</v>
       </c>
-      <c r="M60" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N60" s="79">
-        <v>0.1</v>
-      </c>
-      <c r="O60" s="56">
-        <f>N60*L60</f>
-        <v>0.5</v>
-      </c>
-      <c r="P60" s="30"/>
+      <c r="M60" s="30"/>
     </row>
-    <row r="61" spans="1:16384" ht="24" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:16381" ht="24" x14ac:dyDescent="0.25">
       <c r="A61" s="1"/>
-      <c r="B61" s="61">
+      <c r="B61" s="54">
         <f>ROW(B61) - ROW($B$9)</f>
         <v>52</v>
       </c>
@@ -5131,7 +4497,7 @@
         <v>17</v>
       </c>
       <c r="D61" s="31" t="s">
-        <v>392</v>
+        <v>387</v>
       </c>
       <c r="E61" s="30" t="s">
         <v>149</v>
@@ -5154,42 +4520,32 @@
       <c r="K61" s="30">
         <v>11</v>
       </c>
-      <c r="L61" s="73">
+      <c r="L61" s="66">
         <f>K61*5</f>
         <v>55</v>
       </c>
-      <c r="M61" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N61" s="79">
-        <v>6.4000000000000003E-3</v>
-      </c>
-      <c r="O61" s="56">
-        <f>N61*L61</f>
-        <v>0.35200000000000004</v>
-      </c>
-      <c r="P61" s="31"/>
+      <c r="M61" s="31"/>
     </row>
-    <row r="62" spans="1:16384" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:16381" x14ac:dyDescent="0.25">
       <c r="A62" s="1"/>
-      <c r="B62" s="61">
+      <c r="B62" s="54">
         <f>ROW(B62) - ROW($B$9)</f>
         <v>53</v>
       </c>
       <c r="C62" s="45" t="s">
-        <v>393</v>
-      </c>
-      <c r="D62" s="91" t="s">
-        <v>411</v>
+        <v>388</v>
+      </c>
+      <c r="D62" s="73" t="s">
+        <v>404</v>
       </c>
       <c r="E62" s="30" t="s">
-        <v>412</v>
+        <v>405</v>
       </c>
       <c r="F62" s="30" t="s">
         <v>370</v>
       </c>
       <c r="G62" s="30" t="s">
-        <v>413</v>
+        <v>406</v>
       </c>
       <c r="H62" s="30" t="s">
         <v>369</v>
@@ -5207,17 +4563,8 @@
         <f>K62*5</f>
         <v>15</v>
       </c>
-      <c r="M62" s="93" t="s">
-        <v>402</v>
-      </c>
-      <c r="N62" s="79">
-        <v>0.1</v>
-      </c>
-      <c r="O62" s="56">
-        <f>N62*L62</f>
-        <v>1.5</v>
-      </c>
-      <c r="P62" s="31"/>
+      <c r="M62" s="31"/>
+      <c r="N62" s="1"/>
       <c r="Q62" s="1"/>
       <c r="R62" s="1"/>
       <c r="S62" s="1"/>
@@ -21583,13 +20930,10 @@
       <c r="XEY62" s="1"/>
       <c r="XEZ62" s="1"/>
       <c r="XFA62" s="1"/>
-      <c r="XFB62" s="1"/>
-      <c r="XFC62" s="1"/>
-      <c r="XFD62" s="1"/>
     </row>
-    <row r="63" spans="1:16384" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:16381" x14ac:dyDescent="0.25">
       <c r="A63" s="1"/>
-      <c r="B63" s="61">
+      <c r="B63" s="54">
         <f>ROW(B63) - ROW($B$9)</f>
         <v>54</v>
       </c>
@@ -21620,25 +20964,15 @@
       <c r="K63" s="30">
         <v>4</v>
       </c>
-      <c r="L63" s="73">
+      <c r="L63" s="66">
         <f>K63*5</f>
         <v>20</v>
       </c>
-      <c r="M63" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N63" s="79">
-        <v>1.4E-2</v>
-      </c>
-      <c r="O63" s="56">
-        <f>N63*L63</f>
-        <v>0.28000000000000003</v>
-      </c>
-      <c r="P63" s="31"/>
+      <c r="M63" s="31"/>
     </row>
-    <row r="64" spans="1:16384" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:16381" x14ac:dyDescent="0.25">
       <c r="A64" s="1"/>
-      <c r="B64" s="62">
+      <c r="B64" s="55">
         <f t="shared" si="0"/>
         <v>55</v>
       </c>
@@ -21669,25 +21003,15 @@
       <c r="K64" s="31">
         <v>1</v>
       </c>
-      <c r="L64" s="74">
-        <f t="shared" ref="L64" si="38">K64*5</f>
+      <c r="L64" s="67">
+        <f t="shared" ref="L64" si="26">K64*5</f>
         <v>5</v>
       </c>
-      <c r="M64" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N64" s="80">
-        <v>0.1</v>
-      </c>
-      <c r="O64" s="55">
-        <f t="shared" ref="O64" si="39">N64*L64</f>
-        <v>0.5</v>
-      </c>
-      <c r="P64" s="31"/>
+      <c r="M64" s="31"/>
     </row>
-    <row r="65" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A65" s="1"/>
-      <c r="B65" s="61">
+      <c r="B65" s="54">
         <f>ROW(B65) - ROW($B$9)</f>
         <v>56</v>
       </c>
@@ -21718,25 +21042,15 @@
       <c r="K65" s="30">
         <v>1</v>
       </c>
-      <c r="L65" s="73">
+      <c r="L65" s="66">
         <f>K65*5</f>
         <v>5</v>
       </c>
-      <c r="M65" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N65" s="79">
-        <v>0.1</v>
-      </c>
-      <c r="O65" s="56">
-        <f>N65*L65</f>
-        <v>0.5</v>
-      </c>
-      <c r="P65" s="30"/>
+      <c r="M65" s="30"/>
     </row>
-    <row r="66" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A66" s="1"/>
-      <c r="B66" s="62">
+      <c r="B66" s="55">
         <f t="shared" si="0"/>
         <v>57</v>
       </c>
@@ -21767,25 +21081,15 @@
       <c r="K66" s="31">
         <v>1</v>
       </c>
-      <c r="L66" s="74">
-        <f t="shared" ref="L66:L67" si="40">K66*5</f>
+      <c r="L66" s="67">
+        <f t="shared" ref="L66:L67" si="27">K66*5</f>
         <v>5</v>
       </c>
-      <c r="M66" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N66" s="80">
-        <v>0.34</v>
-      </c>
-      <c r="O66" s="55">
-        <f t="shared" ref="O66:O67" si="41">N66*L66</f>
-        <v>1.7000000000000002</v>
-      </c>
-      <c r="P66" s="31"/>
+      <c r="M66" s="31"/>
     </row>
-    <row r="67" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A67" s="1"/>
-      <c r="B67" s="62">
+      <c r="B67" s="55">
         <f t="shared" si="0"/>
         <v>58</v>
       </c>
@@ -21801,11 +21105,11 @@
       <c r="F67" s="31" t="s">
         <v>201</v>
       </c>
-      <c r="G67" s="91" t="s">
+      <c r="G67" s="73" t="s">
         <v>264</v>
       </c>
       <c r="H67" s="31" t="s">
-        <v>404</v>
+        <v>397</v>
       </c>
       <c r="I67" s="31" t="s">
         <v>317</v>
@@ -21816,25 +21120,15 @@
       <c r="K67" s="31">
         <v>4</v>
       </c>
-      <c r="L67" s="74">
-        <f t="shared" si="40"/>
+      <c r="L67" s="67">
+        <f t="shared" si="27"/>
         <v>20</v>
       </c>
-      <c r="M67" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N67" s="80">
-        <v>0.11600000000000001</v>
-      </c>
-      <c r="O67" s="55">
-        <f t="shared" si="41"/>
-        <v>2.3200000000000003</v>
-      </c>
-      <c r="P67" s="30"/>
+      <c r="M67" s="30"/>
     </row>
-    <row r="68" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A68" s="1"/>
-      <c r="B68" s="61">
+      <c r="B68" s="54">
         <f>ROW(B68) - ROW($B$9)</f>
         <v>59</v>
       </c>
@@ -21865,25 +21159,15 @@
       <c r="K68" s="30">
         <v>1</v>
       </c>
-      <c r="L68" s="73">
+      <c r="L68" s="66">
         <f>K68*5</f>
         <v>5</v>
       </c>
-      <c r="M68" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N68" s="79">
-        <v>0.1</v>
-      </c>
-      <c r="O68" s="56">
-        <f>N68*L68</f>
-        <v>0.5</v>
-      </c>
-      <c r="P68" s="31"/>
+      <c r="M68" s="31"/>
     </row>
-    <row r="69" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A69" s="1"/>
-      <c r="B69" s="62">
+      <c r="B69" s="55">
         <f t="shared" si="0"/>
         <v>60</v>
       </c>
@@ -21914,25 +21198,15 @@
       <c r="K69" s="31">
         <v>1</v>
       </c>
-      <c r="L69" s="74">
-        <f t="shared" ref="L69" si="42">K69*5</f>
+      <c r="L69" s="67">
+        <f t="shared" ref="L69" si="28">K69*5</f>
         <v>5</v>
       </c>
-      <c r="M69" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N69" s="80">
-        <v>0.41</v>
-      </c>
-      <c r="O69" s="55">
-        <f t="shared" ref="O69" si="43">N69*L69</f>
-        <v>2.0499999999999998</v>
-      </c>
-      <c r="P69" s="30"/>
+      <c r="M69" s="30"/>
     </row>
-    <row r="70" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A70" s="1"/>
-      <c r="B70" s="61">
+      <c r="B70" s="54">
         <f>ROW(B70) - ROW($B$9)</f>
         <v>61</v>
       </c>
@@ -21963,25 +21237,15 @@
       <c r="K70" s="30">
         <v>2</v>
       </c>
-      <c r="L70" s="73">
+      <c r="L70" s="66">
         <f>K70*5</f>
         <v>10</v>
       </c>
-      <c r="M70" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N70" s="79">
-        <v>1.7999999999999999E-2</v>
-      </c>
-      <c r="O70" s="56">
-        <f>N70*L70</f>
-        <v>0.18</v>
-      </c>
-      <c r="P70" s="31"/>
+      <c r="M70" s="31"/>
     </row>
-    <row r="71" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A71" s="1"/>
-      <c r="B71" s="62">
+      <c r="B71" s="55">
         <f t="shared" si="0"/>
         <v>62</v>
       </c>
@@ -22012,42 +21276,32 @@
       <c r="K71" s="31">
         <v>1</v>
       </c>
-      <c r="L71" s="74">
-        <f t="shared" ref="L71:L72" si="44">K71*5</f>
+      <c r="L71" s="67">
+        <f t="shared" ref="L71:L72" si="29">K71*5</f>
         <v>5</v>
       </c>
-      <c r="M71" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N71" s="80">
-        <v>0.1</v>
-      </c>
-      <c r="O71" s="55">
-        <f t="shared" ref="O71:O72" si="45">N71*L71</f>
-        <v>0.5</v>
-      </c>
-      <c r="P71" s="30"/>
+      <c r="M71" s="30"/>
     </row>
-    <row r="72" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A72" s="1"/>
-      <c r="B72" s="62">
+      <c r="B72" s="55">
         <f t="shared" si="0"/>
         <v>63</v>
       </c>
       <c r="C72" s="45" t="s">
-        <v>393</v>
+        <v>388</v>
       </c>
       <c r="D72" s="31" t="s">
-        <v>394</v>
+        <v>389</v>
       </c>
       <c r="E72" s="31" t="s">
-        <v>395</v>
+        <v>390</v>
       </c>
       <c r="F72" s="31" t="s">
         <v>370</v>
       </c>
       <c r="G72" s="31" t="s">
-        <v>396</v>
+        <v>391</v>
       </c>
       <c r="H72" s="31" t="s">
         <v>369</v>
@@ -22061,25 +21315,15 @@
       <c r="K72" s="31">
         <v>5</v>
       </c>
-      <c r="L72" s="74">
-        <f t="shared" si="44"/>
+      <c r="L72" s="67">
+        <f t="shared" si="29"/>
         <v>25</v>
       </c>
-      <c r="M72" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N72" s="80">
-        <v>8.9599999999999999E-2</v>
-      </c>
-      <c r="O72" s="55">
-        <f t="shared" si="45"/>
-        <v>2.2399999999999998</v>
-      </c>
-      <c r="P72" s="31"/>
+      <c r="M72" s="31"/>
     </row>
-    <row r="73" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A73" s="1"/>
-      <c r="B73" s="61">
+      <c r="B73" s="54">
         <f>ROW(B73) - ROW($B$9)</f>
         <v>64</v>
       </c>
@@ -22110,24 +21354,15 @@
       <c r="K73" s="46">
         <v>2</v>
       </c>
-      <c r="L73" s="76">
+      <c r="L73" s="69">
         <f>K73*5</f>
         <v>10</v>
       </c>
-      <c r="M73" s="88" t="s">
-        <v>369</v>
-      </c>
-      <c r="N73" s="82" t="s">
-        <v>369</v>
-      </c>
-      <c r="O73" s="46" t="s">
-        <v>369</v>
-      </c>
-      <c r="P73" s="30"/>
+      <c r="M73" s="30"/>
     </row>
-    <row r="74" spans="1:16" ht="24" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:13" ht="24" x14ac:dyDescent="0.25">
       <c r="A74" s="1"/>
-      <c r="B74" s="62">
+      <c r="B74" s="55">
         <f t="shared" si="0"/>
         <v>65</v>
       </c>
@@ -22158,25 +21393,15 @@
       <c r="K74" s="31">
         <v>1</v>
       </c>
-      <c r="L74" s="74">
-        <f t="shared" ref="L74" si="46">K74*5</f>
+      <c r="L74" s="67">
+        <f t="shared" ref="L74" si="30">K74*5</f>
         <v>5</v>
       </c>
-      <c r="M74" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N74" s="80">
-        <v>0.14000000000000001</v>
-      </c>
-      <c r="O74" s="55">
-        <f t="shared" ref="O74" si="47">N74*L74</f>
-        <v>0.70000000000000007</v>
-      </c>
-      <c r="P74" s="31"/>
+      <c r="M74" s="31"/>
     </row>
-    <row r="75" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A75" s="1"/>
-      <c r="B75" s="61">
+      <c r="B75" s="54">
         <f>ROW(B75) - ROW($B$9)</f>
         <v>66</v>
       </c>
@@ -22207,25 +21432,15 @@
       <c r="K75" s="30">
         <v>1</v>
       </c>
-      <c r="L75" s="73">
+      <c r="L75" s="66">
         <f>K75*5</f>
         <v>5</v>
       </c>
-      <c r="M75" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N75" s="79">
-        <v>5.28</v>
-      </c>
-      <c r="O75" s="56">
-        <f>N75*L75</f>
-        <v>26.400000000000002</v>
-      </c>
-      <c r="P75" s="30"/>
+      <c r="M75" s="30"/>
     </row>
-    <row r="76" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A76" s="1"/>
-      <c r="B76" s="62">
+      <c r="B76" s="55">
         <f t="shared" si="0"/>
         <v>67</v>
       </c>
@@ -22256,25 +21471,15 @@
       <c r="K76" s="31">
         <v>1</v>
       </c>
-      <c r="L76" s="74">
-        <f t="shared" ref="L76" si="48">K76*5</f>
+      <c r="L76" s="67">
+        <f t="shared" ref="L76" si="31">K76*5</f>
         <v>5</v>
       </c>
-      <c r="M76" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N76" s="80">
-        <v>0.88</v>
-      </c>
-      <c r="O76" s="55">
-        <f t="shared" ref="O76" si="49">N76*L76</f>
-        <v>4.4000000000000004</v>
-      </c>
-      <c r="P76" s="31"/>
+      <c r="M76" s="31"/>
     </row>
-    <row r="77" spans="1:16" ht="36" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:13" ht="36" x14ac:dyDescent="0.25">
       <c r="A77" s="1"/>
-      <c r="B77" s="61">
+      <c r="B77" s="54">
         <f>ROW(B77) - ROW($B$9)</f>
         <v>68</v>
       </c>
@@ -22305,24 +21510,15 @@
       <c r="K77" s="30">
         <v>1</v>
       </c>
-      <c r="L77" s="73">
+      <c r="L77" s="66">
         <f>K77*5</f>
         <v>5</v>
       </c>
-      <c r="M77" s="90" t="s">
-        <v>403</v>
-      </c>
-      <c r="N77" s="80" t="s">
-        <v>369</v>
-      </c>
-      <c r="O77" s="55" t="s">
-        <v>369</v>
-      </c>
-      <c r="P77" s="30"/>
+      <c r="M77" s="30"/>
     </row>
-    <row r="78" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A78" s="1"/>
-      <c r="B78" s="62">
+      <c r="B78" s="55">
         <f t="shared" si="0"/>
         <v>69</v>
       </c>
@@ -22353,25 +21549,15 @@
       <c r="K78" s="31">
         <v>1</v>
       </c>
-      <c r="L78" s="74">
-        <f t="shared" ref="L78" si="50">K78*5</f>
+      <c r="L78" s="67">
+        <f t="shared" ref="L78" si="32">K78*5</f>
         <v>5</v>
       </c>
-      <c r="M78" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N78" s="80">
-        <v>2.89</v>
-      </c>
-      <c r="O78" s="55">
-        <f t="shared" ref="O78" si="51">N78*L78</f>
-        <v>14.450000000000001</v>
-      </c>
-      <c r="P78" s="31"/>
+      <c r="M78" s="31"/>
     </row>
-    <row r="79" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A79" s="1"/>
-      <c r="B79" s="61">
+      <c r="B79" s="54">
         <f>ROW(B79) - ROW($B$9)</f>
         <v>70</v>
       </c>
@@ -22400,25 +21586,15 @@
       <c r="K79" s="30">
         <v>1</v>
       </c>
-      <c r="L79" s="73">
+      <c r="L79" s="66">
         <f>K79*5</f>
         <v>5</v>
       </c>
-      <c r="M79" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N79" s="79">
-        <v>1.1499999999999999</v>
-      </c>
-      <c r="O79" s="56">
-        <f>N79*L79</f>
-        <v>5.75</v>
-      </c>
-      <c r="P79" s="30"/>
+      <c r="M79" s="30"/>
     </row>
-    <row r="80" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A80" s="1"/>
-      <c r="B80" s="63">
+      <c r="B80" s="56">
         <f t="shared" si="0"/>
         <v>71</v>
       </c>
@@ -22449,25 +21625,15 @@
       <c r="K80" s="49">
         <v>1</v>
       </c>
-      <c r="L80" s="77">
-        <f t="shared" ref="L80" si="52">K80*5</f>
+      <c r="L80" s="70">
+        <f t="shared" ref="L80" si="33">K80*5</f>
         <v>5</v>
       </c>
-      <c r="M80" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N80" s="83">
-        <v>2.5099999999999998</v>
-      </c>
-      <c r="O80" s="57">
-        <f t="shared" ref="O80" si="53">N80*L80</f>
-        <v>12.549999999999999</v>
-      </c>
-      <c r="P80" s="31"/>
+      <c r="M80" s="31"/>
     </row>
-    <row r="81" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A81" s="1"/>
-      <c r="B81" s="64">
+      <c r="B81" s="57">
         <f>ROW(B81) - ROW($B$9)</f>
         <v>72</v>
       </c>
@@ -22498,25 +21664,15 @@
       <c r="K81" s="51">
         <v>1</v>
       </c>
-      <c r="L81" s="78">
+      <c r="L81" s="71">
         <f>K81*5</f>
         <v>5</v>
       </c>
-      <c r="M81" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N81" s="84">
-        <v>0.9</v>
-      </c>
-      <c r="O81" s="58">
-        <f>N81*L81</f>
-        <v>4.5</v>
-      </c>
-      <c r="P81" s="30"/>
+      <c r="M81" s="30"/>
     </row>
-    <row r="82" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A82" s="1"/>
-      <c r="B82" s="62">
+      <c r="B82" s="55">
         <f t="shared" si="0"/>
         <v>73</v>
       </c>
@@ -22545,25 +21701,15 @@
       <c r="K82" s="31">
         <v>1</v>
       </c>
-      <c r="L82" s="74">
-        <f t="shared" ref="L82" si="54">K82*5</f>
+      <c r="L82" s="67">
+        <f t="shared" ref="L82" si="34">K82*5</f>
         <v>5</v>
       </c>
-      <c r="M82" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N82" s="80">
-        <v>1.53</v>
-      </c>
-      <c r="O82" s="55">
-        <f t="shared" ref="O82" si="55">N82*L82</f>
-        <v>7.65</v>
-      </c>
-      <c r="P82" s="31"/>
+      <c r="M82" s="31"/>
     </row>
-    <row r="83" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A83" s="1"/>
-      <c r="B83" s="64">
+      <c r="B83" s="57">
         <f>ROW(B83) - ROW($B$9)</f>
         <v>74</v>
       </c>
@@ -22594,25 +21740,15 @@
       <c r="K83" s="51">
         <v>1</v>
       </c>
-      <c r="L83" s="78">
+      <c r="L83" s="71">
         <f>K83*5</f>
         <v>5</v>
       </c>
-      <c r="M83" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N83" s="84">
-        <v>3.54</v>
-      </c>
-      <c r="O83" s="58">
-        <f>N83*L83</f>
-        <v>17.7</v>
-      </c>
-      <c r="P83" s="30"/>
+      <c r="M83" s="30"/>
     </row>
-    <row r="84" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A84" s="1"/>
-      <c r="B84" s="62">
+      <c r="B84" s="55">
         <f t="shared" si="0"/>
         <v>75</v>
       </c>
@@ -22643,25 +21779,15 @@
       <c r="K84" s="31">
         <v>3</v>
       </c>
-      <c r="L84" s="74">
-        <f t="shared" ref="L84" si="56">K84*5</f>
+      <c r="L84" s="67">
+        <f t="shared" ref="L84" si="35">K84*5</f>
         <v>15</v>
       </c>
-      <c r="M84" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N84" s="80">
-        <v>1.69</v>
-      </c>
-      <c r="O84" s="55">
-        <f t="shared" ref="O84" si="57">N84*L84</f>
-        <v>25.349999999999998</v>
-      </c>
-      <c r="P84" s="31"/>
+      <c r="M84" s="31"/>
     </row>
-    <row r="85" spans="1:16" ht="60" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A85" s="1"/>
-      <c r="B85" s="61">
+      <c r="B85" s="54">
         <f>ROW(B85) - ROW($B$9)</f>
         <v>76</v>
       </c>
@@ -22692,24 +21818,15 @@
       <c r="K85" s="30">
         <v>1</v>
       </c>
-      <c r="L85" s="73">
+      <c r="L85" s="66">
         <f>K85*5</f>
         <v>5</v>
       </c>
-      <c r="M85" s="90" t="s">
-        <v>403</v>
-      </c>
-      <c r="N85" s="80" t="s">
-        <v>369</v>
-      </c>
-      <c r="O85" s="55" t="s">
-        <v>369</v>
-      </c>
-      <c r="P85" s="30"/>
+      <c r="M85" s="30"/>
     </row>
-    <row r="86" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A86" s="1"/>
-      <c r="B86" s="62">
+      <c r="B86" s="55">
         <f t="shared" si="0"/>
         <v>77</v>
       </c>
@@ -22740,25 +21857,15 @@
       <c r="K86" s="31">
         <v>1</v>
       </c>
-      <c r="L86" s="74">
-        <f t="shared" ref="L86" si="58">K86*5</f>
+      <c r="L86" s="67">
+        <f t="shared" ref="L86" si="36">K86*5</f>
         <v>5</v>
       </c>
-      <c r="M86" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N86" s="80">
-        <v>2.14</v>
-      </c>
-      <c r="O86" s="55">
-        <f t="shared" ref="O86" si="59">N86*L86</f>
-        <v>10.700000000000001</v>
-      </c>
-      <c r="P86" s="31"/>
+      <c r="M86" s="31"/>
     </row>
-    <row r="87" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A87" s="1"/>
-      <c r="B87" s="61">
+      <c r="B87" s="54">
         <f>ROW(B87) - ROW($B$9)</f>
         <v>78</v>
       </c>
@@ -22789,24 +21896,15 @@
       <c r="K87" s="30">
         <v>1</v>
       </c>
-      <c r="L87" s="73">
+      <c r="L87" s="66">
         <f>K87*5</f>
         <v>5</v>
       </c>
-      <c r="M87" s="90" t="s">
-        <v>403</v>
-      </c>
-      <c r="N87" s="80" t="s">
-        <v>369</v>
-      </c>
-      <c r="O87" s="55" t="s">
-        <v>369</v>
-      </c>
-      <c r="P87" s="30"/>
+      <c r="M87" s="30"/>
     </row>
-    <row r="88" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A88" s="1"/>
-      <c r="B88" s="62">
+      <c r="B88" s="55">
         <f t="shared" si="0"/>
         <v>79</v>
       </c>
@@ -22837,25 +21935,15 @@
       <c r="K88" s="31">
         <v>1</v>
       </c>
-      <c r="L88" s="74">
-        <f t="shared" ref="L88" si="60">K88*5</f>
+      <c r="L88" s="67">
+        <f t="shared" ref="L88" si="37">K88*5</f>
         <v>5</v>
       </c>
-      <c r="M88" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N88" s="80">
-        <v>4</v>
-      </c>
-      <c r="O88" s="55">
-        <f t="shared" ref="O88" si="61">N88*L88</f>
-        <v>20</v>
-      </c>
-      <c r="P88" s="31"/>
+      <c r="M88" s="31"/>
     </row>
-    <row r="89" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A89" s="1"/>
-      <c r="B89" s="61">
+      <c r="B89" s="54">
         <f>ROW(B89) - ROW($B$9)</f>
         <v>80</v>
       </c>
@@ -22886,25 +21974,15 @@
       <c r="K89" s="30">
         <v>1</v>
       </c>
-      <c r="L89" s="73">
+      <c r="L89" s="66">
         <f>K89*5</f>
         <v>5</v>
       </c>
-      <c r="M89" s="89" t="s">
-        <v>402</v>
-      </c>
-      <c r="N89" s="79">
-        <v>4.17</v>
-      </c>
-      <c r="O89" s="56">
-        <f>N89*L89</f>
-        <v>20.85</v>
-      </c>
-      <c r="P89" s="30"/>
+      <c r="M89" s="30"/>
     </row>
-    <row r="90" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:13" ht="24" x14ac:dyDescent="0.25">
       <c r="A90" s="1"/>
-      <c r="B90" s="62">
+      <c r="B90" s="55">
         <f t="shared" si="0"/>
         <v>81</v>
       </c>
@@ -22935,24 +22013,15 @@
       <c r="K90" s="31">
         <v>1</v>
       </c>
-      <c r="L90" s="74">
-        <f t="shared" ref="L90" si="62">K90*5</f>
+      <c r="L90" s="67">
+        <f t="shared" ref="L90" si="38">K90*5</f>
         <v>5</v>
       </c>
-      <c r="M90" s="90" t="s">
-        <v>403</v>
-      </c>
-      <c r="N90" s="80" t="s">
-        <v>369</v>
-      </c>
-      <c r="O90" s="55" t="s">
-        <v>369</v>
-      </c>
-      <c r="P90" s="31"/>
+      <c r="M90" s="31"/>
     </row>
-    <row r="91" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:13" ht="24" x14ac:dyDescent="0.25">
       <c r="A91" s="1"/>
-      <c r="B91" s="61">
+      <c r="B91" s="54">
         <f>ROW(B91) - ROW($B$9)</f>
         <v>82</v>
       </c>
@@ -22963,19 +22032,19 @@
         <v>96</v>
       </c>
       <c r="E91" s="30" t="s">
-        <v>397</v>
+        <v>392</v>
       </c>
       <c r="F91" s="30" t="s">
-        <v>398</v>
+        <v>393</v>
       </c>
       <c r="G91" s="30" t="s">
-        <v>399</v>
+        <v>394</v>
       </c>
       <c r="H91" s="30" t="s">
         <v>369</v>
       </c>
       <c r="I91" s="30" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
       <c r="J91" s="30" t="s">
         <v>365</v>
@@ -22983,135 +22052,104 @@
       <c r="K91" s="30">
         <v>1</v>
       </c>
-      <c r="L91" s="73">
+      <c r="L91" s="66">
         <f>K91*5</f>
         <v>5</v>
       </c>
-      <c r="M91" s="90" t="s">
-        <v>403</v>
-      </c>
-      <c r="N91" s="80" t="s">
-        <v>369</v>
-      </c>
-      <c r="O91" s="55" t="s">
-        <v>369</v>
-      </c>
-      <c r="P91" s="31"/>
+      <c r="M91" s="31"/>
     </row>
-    <row r="92" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A92" s="1"/>
-      <c r="B92" s="61">
+      <c r="B92" s="54">
         <f>ROW(B92) - ROW($B$9)</f>
         <v>83</v>
       </c>
       <c r="C92" s="43" t="s">
-        <v>415</v>
+        <v>408</v>
       </c>
       <c r="D92" s="51" t="s">
         <v>369</v>
       </c>
       <c r="E92" s="51" t="s">
-        <v>416</v>
+        <v>409</v>
       </c>
       <c r="F92" s="51" t="s">
         <v>369</v>
       </c>
       <c r="G92" s="51" t="s">
-        <v>417</v>
-      </c>
-      <c r="H92" s="95" t="s">
+        <v>410</v>
+      </c>
+      <c r="H92" s="76" t="s">
         <v>369</v>
       </c>
       <c r="I92" s="51" t="s">
-        <v>418</v>
+        <v>411</v>
       </c>
       <c r="J92" s="30" t="s">
         <v>369</v>
       </c>
-      <c r="K92" s="95">
+      <c r="K92" s="76">
         <v>1</v>
       </c>
-      <c r="L92" s="96">
+      <c r="L92" s="77">
         <f>K92*5</f>
         <v>5</v>
       </c>
-      <c r="M92" s="90" t="s">
-        <v>403</v>
-      </c>
-      <c r="N92" s="80" t="s">
-        <v>369</v>
-      </c>
-      <c r="O92" s="55" t="s">
-        <v>369</v>
-      </c>
-      <c r="P92" s="97"/>
+      <c r="M92" s="78"/>
     </row>
-    <row r="93" spans="1:16" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:13" ht="36" x14ac:dyDescent="0.25">
       <c r="A93" s="1"/>
-      <c r="B93" s="64">
+      <c r="B93" s="57">
         <f>ROW(B93) - ROW($B$9)</f>
         <v>84</v>
       </c>
-      <c r="C93" s="50" t="s">
-        <v>415</v>
-      </c>
-      <c r="D93" s="51"/>
-      <c r="E93" s="30" t="s">
-        <v>424</v>
-      </c>
-      <c r="F93" s="51" t="s">
+      <c r="C93" s="45" t="s">
+        <v>408</v>
+      </c>
+      <c r="D93" s="31"/>
+      <c r="E93" s="31" t="s">
+        <v>417</v>
+      </c>
+      <c r="F93" s="31" t="s">
         <v>369</v>
       </c>
-      <c r="G93" s="51" t="s">
-        <v>425</v>
-      </c>
-      <c r="H93" s="95" t="s">
+      <c r="G93" s="31" t="s">
+        <v>418</v>
+      </c>
+      <c r="H93" s="31" t="s">
         <v>369</v>
       </c>
-      <c r="I93" s="51" t="s">
+      <c r="I93" s="31" t="s">
         <v>369</v>
       </c>
-      <c r="J93" s="30" t="s">
+      <c r="J93" s="31" t="s">
         <v>369</v>
       </c>
-      <c r="K93" s="95">
-        <v>1</v>
-      </c>
-      <c r="L93" s="96">
+      <c r="K93" s="31">
+        <v>3</v>
+      </c>
+      <c r="L93" s="67">
         <f>K93*5</f>
-        <v>5</v>
-      </c>
-      <c r="M93" s="90" t="s">
-        <v>403</v>
-      </c>
-      <c r="N93" s="80"/>
-      <c r="O93" s="55"/>
-      <c r="P93" s="97"/>
+        <v>15</v>
+      </c>
+      <c r="M93" s="31"/>
     </row>
-    <row r="94" spans="1:16" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A94" s="1"/>
-      <c r="B94" s="65"/>
-      <c r="C94" s="66"/>
-      <c r="D94" s="67"/>
-      <c r="E94" s="68"/>
-      <c r="F94" s="69"/>
-      <c r="G94" s="70"/>
-      <c r="H94" s="70"/>
-      <c r="I94" s="69"/>
-      <c r="J94" s="70"/>
-      <c r="K94" s="70"/>
-      <c r="L94" s="101" t="s">
-        <v>386</v>
-      </c>
-      <c r="M94" s="102"/>
-      <c r="N94" s="103"/>
-      <c r="O94" s="59">
-        <f>SUM(O10:O91)</f>
-        <v>263.25150000000002</v>
-      </c>
-      <c r="P94" s="71"/>
+      <c r="B94" s="58"/>
+      <c r="C94" s="59"/>
+      <c r="D94" s="60"/>
+      <c r="E94" s="61"/>
+      <c r="F94" s="62"/>
+      <c r="G94" s="63"/>
+      <c r="H94" s="63"/>
+      <c r="I94" s="62"/>
+      <c r="J94" s="63"/>
+      <c r="K94" s="63"/>
+      <c r="L94" s="9"/>
+      <c r="M94" s="64"/>
     </row>
-    <row r="95" spans="1:16" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B95" s="24"/>
       <c r="C95" s="38"/>
       <c r="D95" s="8"/>
@@ -23122,80 +22160,16 @@
       <c r="I95" s="9"/>
       <c r="J95" s="9"/>
       <c r="K95" s="9"/>
-      <c r="L95" s="101" t="s">
-        <v>387</v>
-      </c>
-      <c r="M95" s="103"/>
-      <c r="N95" s="103"/>
-      <c r="O95" s="60">
-        <f>O94/5</f>
-        <v>52.650300000000001</v>
-      </c>
-      <c r="P95" s="72"/>
+      <c r="L95" s="65"/>
+      <c r="M95" s="65"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="J1:P1"/>
-    <mergeCell ref="P3:P8"/>
-    <mergeCell ref="L94:N94"/>
-    <mergeCell ref="L95:N95"/>
+  <mergeCells count="2">
+    <mergeCell ref="J1:M1"/>
+    <mergeCell ref="M3:M8"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink ref="M11" r:id="rId1"/>
-    <hyperlink ref="M12" r:id="rId2"/>
-    <hyperlink ref="M13" r:id="rId3"/>
-    <hyperlink ref="M18" r:id="rId4"/>
-    <hyperlink ref="M19" r:id="rId5"/>
-    <hyperlink ref="M20" r:id="rId6"/>
-    <hyperlink ref="M21" r:id="rId7"/>
-    <hyperlink ref="M22" r:id="rId8"/>
-    <hyperlink ref="M23" r:id="rId9"/>
-    <hyperlink ref="M24" r:id="rId10"/>
-    <hyperlink ref="M28" r:id="rId11"/>
-    <hyperlink ref="M30" r:id="rId12"/>
-    <hyperlink ref="M32" r:id="rId13"/>
-    <hyperlink ref="M35" r:id="rId14"/>
-    <hyperlink ref="M43" r:id="rId15"/>
-    <hyperlink ref="M49" r:id="rId16"/>
-    <hyperlink ref="M50" r:id="rId17"/>
-    <hyperlink ref="M51" r:id="rId18"/>
-    <hyperlink ref="M52" r:id="rId19"/>
-    <hyperlink ref="M53" r:id="rId20"/>
-    <hyperlink ref="M54" r:id="rId21"/>
-    <hyperlink ref="M56" r:id="rId22"/>
-    <hyperlink ref="M57" r:id="rId23"/>
-    <hyperlink ref="M58" r:id="rId24"/>
-    <hyperlink ref="M59" r:id="rId25"/>
-    <hyperlink ref="M60" r:id="rId26"/>
-    <hyperlink ref="M61" r:id="rId27"/>
-    <hyperlink ref="M63" r:id="rId28"/>
-    <hyperlink ref="M64" r:id="rId29"/>
-    <hyperlink ref="M65" r:id="rId30"/>
-    <hyperlink ref="M66" r:id="rId31"/>
-    <hyperlink ref="M67" r:id="rId32"/>
-    <hyperlink ref="M68" r:id="rId33"/>
-    <hyperlink ref="M69" r:id="rId34"/>
-    <hyperlink ref="M70" r:id="rId35"/>
-    <hyperlink ref="M71" r:id="rId36"/>
-    <hyperlink ref="M72" r:id="rId37"/>
-    <hyperlink ref="M74" r:id="rId38"/>
-    <hyperlink ref="M75" r:id="rId39"/>
-    <hyperlink ref="M76" r:id="rId40"/>
-    <hyperlink ref="M78" r:id="rId41"/>
-    <hyperlink ref="M79" r:id="rId42"/>
-    <hyperlink ref="M80" r:id="rId43"/>
-    <hyperlink ref="M81" r:id="rId44"/>
-    <hyperlink ref="M82" r:id="rId45"/>
-    <hyperlink ref="M83" r:id="rId46"/>
-    <hyperlink ref="M84" r:id="rId47"/>
-    <hyperlink ref="M86" r:id="rId48"/>
-    <hyperlink ref="M88" r:id="rId49"/>
-    <hyperlink ref="M89" r:id="rId50"/>
-    <hyperlink ref="M15" r:id="rId51"/>
-    <hyperlink ref="M62" r:id="rId52"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId53"/>
-  <drawing r:id="rId54"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>